<commit_message>
Fix reconciliation: PURVCHNO in bank statement, Old Account per-row PURPAIDAMT
- Bank Statement Voucher_No: PURVCHNO comma-separated (not bill numbers)
  e.g. CHQ 002562 -> "310,341,343,351,353,427,434,457,460,521,537,613,649,723,782,821,825"
- System_Purchase Old Account: PURPAIDAMT of the specific matched PAIDTRAN row
  e.g. Vou.No.427 -> OldAcct=341, Vou.No.825 -> OldAcct=93 (partial payment)
- Previous Pending: sum of PURPAIDAMT for BILLDATE < 29-May-2025 (same PADVCHNO)
  e.g. RUSHABH SURGICALS -> PrevPend=9492 (5 pre-takeover bills)

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -715,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O891"/>
+  <dimension ref="A1:N891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
@@ -803,11 +803,6 @@
           <t>Party_Name</t>
         </is>
       </c>
-      <c r="O1" s="32" t="inlineStr">
-        <is>
-          <t>Bill_Nos</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="21" t="n">
@@ -892,17 +887,14 @@
         </is>
       </c>
       <c r="L3" s="6" t="n"/>
-      <c r="M3" s="33" t="n">
-        <v>144</v>
+      <c r="M3" s="33" t="inlineStr">
+        <is>
+          <t>208,250</t>
+        </is>
       </c>
       <c r="N3" s="33" t="inlineStr">
         <is>
           <t>SHREYAA AGENCIES</t>
-        </is>
-      </c>
-      <c r="O3" s="33" t="inlineStr">
-        <is>
-          <t>684+472+500 | 472+500</t>
         </is>
       </c>
     </row>
@@ -947,17 +939,14 @@
         </is>
       </c>
       <c r="L4" s="6" t="n"/>
-      <c r="M4" s="33" t="n">
-        <v>146</v>
+      <c r="M4" s="33" t="inlineStr">
+        <is>
+          <t>276,330</t>
+        </is>
       </c>
       <c r="N4" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O4" s="33" t="inlineStr">
-        <is>
-          <t>CGSIG25I009878+CGSIG-25-I010808</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1033,10 @@
         </is>
       </c>
       <c r="L6" s="6" t="n"/>
-      <c r="M6" s="33" t="n">
-        <v>137</v>
-      </c>
+      <c r="M6" s="33" t="inlineStr"/>
       <c r="N6" s="33" t="inlineStr">
         <is>
           <t>REKHA MARKETING</t>
-        </is>
-      </c>
-      <c r="O6" s="33" t="inlineStr">
-        <is>
-          <t>RM351</t>
         </is>
       </c>
     </row>
@@ -1099,17 +1081,10 @@
         </is>
       </c>
       <c r="L7" s="28" t="n"/>
-      <c r="M7" s="33" t="n">
-        <v>126</v>
-      </c>
+      <c r="M7" s="33" t="inlineStr"/>
       <c r="N7" s="33" t="inlineStr">
         <is>
           <t>AGARWAL &amp; COMPANY</t>
-        </is>
-      </c>
-      <c r="O7" s="33" t="inlineStr">
-        <is>
-          <t>12164</t>
         </is>
       </c>
     </row>
@@ -1154,17 +1129,10 @@
         </is>
       </c>
       <c r="L8" s="28" t="n"/>
-      <c r="M8" s="33" t="n">
-        <v>126</v>
-      </c>
+      <c r="M8" s="33" t="inlineStr"/>
       <c r="N8" s="33" t="inlineStr">
         <is>
           <t>AGARWAL &amp; COMPANY</t>
-        </is>
-      </c>
-      <c r="O8" s="33" t="inlineStr">
-        <is>
-          <t>12164</t>
         </is>
       </c>
     </row>
@@ -1251,17 +1219,10 @@
         </is>
       </c>
       <c r="L10" s="6" t="n"/>
-      <c r="M10" s="33" t="n">
-        <v>126</v>
-      </c>
+      <c r="M10" s="33" t="inlineStr"/>
       <c r="N10" s="33" t="inlineStr">
         <is>
           <t>AGARWAL &amp; COMPANY</t>
-        </is>
-      </c>
-      <c r="O10" s="33" t="inlineStr">
-        <is>
-          <t>12164</t>
         </is>
       </c>
     </row>
@@ -1398,17 +1359,14 @@
         </is>
       </c>
       <c r="L13" s="6" t="n"/>
-      <c r="M13" s="33" t="n">
-        <v>63</v>
+      <c r="M13" s="33" t="inlineStr">
+        <is>
+          <t>2601</t>
+        </is>
       </c>
       <c r="N13" s="33" t="inlineStr">
         <is>
           <t>NANDINI BEAUTY</t>
-        </is>
-      </c>
-      <c r="O13" s="33" t="inlineStr">
-        <is>
-          <t>111</t>
         </is>
       </c>
     </row>
@@ -1453,17 +1411,14 @@
         </is>
       </c>
       <c r="L14" s="28" t="n"/>
-      <c r="M14" s="33" t="n">
-        <v>91</v>
+      <c r="M14" s="33" t="inlineStr">
+        <is>
+          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
+        </is>
       </c>
       <c r="N14" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O14" s="33" t="inlineStr">
-        <is>
-          <t>2425CRB314926+2425CRB316562+2425CRB317850+2425CRB319230+2425CRB320220+2425CRB320123+2425CRB321680+2425CRB322857+2425CRB324217</t>
         </is>
       </c>
     </row>
@@ -1508,17 +1463,14 @@
         </is>
       </c>
       <c r="L15" s="28" t="n"/>
-      <c r="M15" s="33" t="n">
-        <v>91</v>
+      <c r="M15" s="33" t="inlineStr">
+        <is>
+          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
+        </is>
       </c>
       <c r="N15" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O15" s="33" t="inlineStr">
-        <is>
-          <t>2425CRB314926+2425CRB316562+2425CRB317850+2425CRB319230+2425CRB320220+2425CRB320123+2425CRB321680+2425CRB322857+2425CRB324217</t>
         </is>
       </c>
     </row>
@@ -1647,17 +1599,14 @@
         </is>
       </c>
       <c r="L18" s="6" t="n"/>
-      <c r="M18" s="33" t="n">
-        <v>91</v>
+      <c r="M18" s="33" t="inlineStr">
+        <is>
+          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
+        </is>
       </c>
       <c r="N18" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O18" s="33" t="inlineStr">
-        <is>
-          <t>2425CRB314926+2425CRB316562+2425CRB317850+2425CRB319230+2425CRB320220+2425CRB320123+2425CRB321680+2425CRB322857+2425CRB324217</t>
         </is>
       </c>
     </row>
@@ -1886,15 +1835,12 @@
         </is>
       </c>
       <c r="L23" s="6" t="n"/>
-      <c r="M23" s="33" t="n">
-        <v>148</v>
-      </c>
+      <c r="M23" s="33" t="inlineStr"/>
       <c r="N23" s="33" t="inlineStr">
         <is>
           <t>VENKATESHA ENTERPRISES</t>
         </is>
       </c>
-      <c r="O23" s="33" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="21" t="n">
@@ -1933,17 +1879,10 @@
         </is>
       </c>
       <c r="L24" s="6" t="n"/>
-      <c r="M24" s="33" t="n">
-        <v>140</v>
-      </c>
+      <c r="M24" s="33" t="inlineStr"/>
       <c r="N24" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O24" s="33" t="inlineStr">
-        <is>
-          <t>CGSIG-25-I011739</t>
         </is>
       </c>
     </row>
@@ -2072,15 +2011,12 @@
         </is>
       </c>
       <c r="L27" s="28" t="n"/>
-      <c r="M27" s="33" t="n">
-        <v>70</v>
-      </c>
+      <c r="M27" s="33" t="inlineStr"/>
       <c r="N27" s="33" t="inlineStr">
         <is>
           <t>SHINDE ENTERPRISES</t>
         </is>
       </c>
-      <c r="O27" s="33" t="inlineStr"/>
     </row>
     <row r="28" customFormat="1" s="31">
       <c r="A28" s="29" t="n">
@@ -2123,17 +2059,14 @@
         </is>
       </c>
       <c r="L28" s="28" t="n"/>
-      <c r="M28" s="33" t="n">
-        <v>63</v>
+      <c r="M28" s="33" t="inlineStr">
+        <is>
+          <t>2601</t>
+        </is>
       </c>
       <c r="N28" s="33" t="inlineStr">
         <is>
           <t>NANDINI BEAUTY</t>
-        </is>
-      </c>
-      <c r="O28" s="33" t="inlineStr">
-        <is>
-          <t>111</t>
         </is>
       </c>
     </row>
@@ -2178,17 +2111,14 @@
         </is>
       </c>
       <c r="L29" s="6" t="n"/>
-      <c r="M29" s="33" t="n">
-        <v>163</v>
+      <c r="M29" s="33" t="inlineStr">
+        <is>
+          <t>317</t>
+        </is>
       </c>
       <c r="N29" s="33" t="inlineStr">
         <is>
           <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O29" s="33" t="inlineStr">
-        <is>
-          <t>1042</t>
         </is>
       </c>
     </row>
@@ -2849,17 +2779,14 @@
         </is>
       </c>
       <c r="L44" s="6" t="n"/>
-      <c r="M44" s="33" t="n">
-        <v>162</v>
+      <c r="M44" s="33" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
       </c>
       <c r="N44" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O44" s="33" t="inlineStr">
-        <is>
-          <t>AB06486</t>
         </is>
       </c>
     </row>
@@ -2904,17 +2831,14 @@
         </is>
       </c>
       <c r="L45" s="6" t="n"/>
-      <c r="M45" s="33" t="n">
-        <v>93</v>
+      <c r="M45" s="33" t="inlineStr">
+        <is>
+          <t>2518,2529,2560,2566,2561,2588,2591,2611,2620,2621,2629,2657,2666,2761,2760,2766,2798,2833,2837,2891,2909,2921,2942</t>
+        </is>
       </c>
       <c r="N45" s="33" t="inlineStr">
         <is>
           <t>MAHENDRA DISRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O45" s="33" t="inlineStr">
-        <is>
-          <t>S/48845+S/49053+S/49453+S/49542+S/49664+S/49860+S/50025+S/50342+S/50645+S/50646+S/50717+S/51248+S/51508+S/52868+S/53008+S/53172+S/53966+S/54549+S/545475+S/55720+S/56050+S/56336+S/56860</t>
         </is>
       </c>
     </row>
@@ -3177,17 +3101,10 @@
         </is>
       </c>
       <c r="L51" s="6" t="n"/>
-      <c r="M51" s="33" t="n">
-        <v>141</v>
-      </c>
+      <c r="M51" s="33" t="inlineStr"/>
       <c r="N51" s="33" t="inlineStr">
         <is>
           <t>GAURAV ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O51" s="33" t="inlineStr">
-        <is>
-          <t>CCB1384</t>
         </is>
       </c>
     </row>
@@ -3500,15 +3417,12 @@
         </is>
       </c>
       <c r="L58" s="6" t="n"/>
-      <c r="M58" s="33" t="n">
-        <v>150</v>
-      </c>
+      <c r="M58" s="33" t="inlineStr"/>
       <c r="N58" s="33" t="inlineStr">
         <is>
           <t>RAUT TRADINGS</t>
         </is>
       </c>
-      <c r="O58" s="33" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="21" t="n">
@@ -3551,17 +3465,10 @@
         </is>
       </c>
       <c r="L59" s="6" t="n"/>
-      <c r="M59" s="33" t="n">
-        <v>149</v>
-      </c>
+      <c r="M59" s="33" t="inlineStr"/>
       <c r="N59" s="33" t="inlineStr">
         <is>
           <t>SRI BALAJI FOODS</t>
-        </is>
-      </c>
-      <c r="O59" s="33" t="inlineStr">
-        <is>
-          <t>23/5/25</t>
         </is>
       </c>
     </row>
@@ -3606,15 +3513,12 @@
         </is>
       </c>
       <c r="L60" s="6" t="n"/>
-      <c r="M60" s="33" t="n">
-        <v>147</v>
-      </c>
+      <c r="M60" s="33" t="inlineStr"/>
       <c r="N60" s="33" t="inlineStr">
         <is>
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
-      <c r="O60" s="33" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="21" t="n">
@@ -3657,17 +3561,14 @@
         </is>
       </c>
       <c r="L61" s="6" t="n"/>
-      <c r="M61" s="33" t="n">
-        <v>156</v>
+      <c r="M61" s="33" t="inlineStr">
+        <is>
+          <t>406,409</t>
+        </is>
       </c>
       <c r="N61" s="33" t="inlineStr">
         <is>
           <t>YASH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O61" s="33" t="inlineStr">
-        <is>
-          <t>99+536 | 99+536</t>
         </is>
       </c>
     </row>
@@ -3712,17 +3613,14 @@
         </is>
       </c>
       <c r="L62" s="6" t="n"/>
-      <c r="M62" s="33" t="n">
-        <v>153</v>
+      <c r="M62" s="33" t="inlineStr">
+        <is>
+          <t>399</t>
+        </is>
       </c>
       <c r="N62" s="33" t="inlineStr">
         <is>
           <t>JEEVIKA HOSPITALITY SERVICES</t>
-        </is>
-      </c>
-      <c r="O62" s="33" t="inlineStr">
-        <is>
-          <t>1937</t>
         </is>
       </c>
     </row>
@@ -3901,15 +3799,12 @@
         </is>
       </c>
       <c r="L66" s="6" t="n"/>
-      <c r="M66" s="33" t="n">
-        <v>154</v>
-      </c>
+      <c r="M66" s="33" t="inlineStr"/>
       <c r="N66" s="33" t="inlineStr">
         <is>
           <t>APARNA LOGITECH PRIVATE LIMITE</t>
         </is>
       </c>
-      <c r="O66" s="33" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="21" t="n">
@@ -3952,17 +3847,14 @@
         </is>
       </c>
       <c r="L67" s="6" t="n"/>
-      <c r="M67" s="33" t="n">
-        <v>158</v>
+      <c r="M67" s="33" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
       </c>
       <c r="N67" s="33" t="inlineStr">
         <is>
           <t>JAI SHREE GANESH AGENCIES</t>
-        </is>
-      </c>
-      <c r="O67" s="33" t="inlineStr">
-        <is>
-          <t>I/25-26/002382</t>
         </is>
       </c>
     </row>
@@ -4007,15 +3899,12 @@
         </is>
       </c>
       <c r="L68" s="6" t="n"/>
-      <c r="M68" s="33" t="n">
-        <v>138</v>
-      </c>
+      <c r="M68" s="33" t="inlineStr"/>
       <c r="N68" s="33" t="inlineStr">
         <is>
           <t>ASHA MOHAN ENTERPRISES</t>
         </is>
       </c>
-      <c r="O68" s="33" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="21" t="n">
@@ -4318,15 +4207,12 @@
         </is>
       </c>
       <c r="L75" s="6" t="n"/>
-      <c r="M75" s="33" t="n">
-        <v>160</v>
-      </c>
+      <c r="M75" s="33" t="inlineStr"/>
       <c r="N75" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
-      <c r="O75" s="33" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="21" t="n">
@@ -4369,17 +4255,14 @@
         </is>
       </c>
       <c r="L76" s="6" t="n"/>
-      <c r="M76" s="33" t="n">
-        <v>92</v>
+      <c r="M76" s="33" t="inlineStr">
+        <is>
+          <t>2828,2835,2848,2852,2866,2867,2877,2884</t>
+        </is>
       </c>
       <c r="N76" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O76" s="33" t="inlineStr">
-        <is>
-          <t>2425CRB325627+2425CRB326899+2425CRB327937+2425CRB328965+2425CRB330059+2425CRB331328+2425CRB332623+2425CRB333885</t>
         </is>
       </c>
     </row>
@@ -4508,17 +4391,14 @@
         </is>
       </c>
       <c r="L79" s="6" t="n"/>
-      <c r="M79" s="33" t="n">
-        <v>152</v>
+      <c r="M79" s="33" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
       </c>
       <c r="N79" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O79" s="33" t="inlineStr">
-        <is>
-          <t>20170 | 20170</t>
         </is>
       </c>
     </row>
@@ -5103,17 +4983,14 @@
         </is>
       </c>
       <c r="L92" s="6" t="n"/>
-      <c r="M92" s="33" t="n">
-        <v>173</v>
+      <c r="M92" s="33" t="inlineStr">
+        <is>
+          <t>412</t>
+        </is>
       </c>
       <c r="N92" s="33" t="inlineStr">
         <is>
           <t>ANURAG CORPORATION PVT.LTD</t>
-        </is>
-      </c>
-      <c r="O92" s="33" t="inlineStr">
-        <is>
-          <t>1913</t>
         </is>
       </c>
     </row>
@@ -5158,15 +5035,12 @@
         </is>
       </c>
       <c r="L93" s="6" t="n"/>
-      <c r="M93" s="33" t="n">
-        <v>165</v>
-      </c>
+      <c r="M93" s="33" t="inlineStr"/>
       <c r="N93" s="33" t="inlineStr">
         <is>
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
-      <c r="O93" s="33" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="21" t="n">
@@ -5251,15 +5125,12 @@
         </is>
       </c>
       <c r="L95" s="6" t="n"/>
-      <c r="M95" s="33" t="n">
-        <v>116</v>
-      </c>
+      <c r="M95" s="33" t="inlineStr"/>
       <c r="N95" s="33" t="inlineStr">
         <is>
           <t>DP SOLUTIONS</t>
         </is>
       </c>
-      <c r="O95" s="33" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="21" t="n">
@@ -5478,17 +5349,14 @@
         </is>
       </c>
       <c r="L100" s="6" t="n"/>
-      <c r="M100" s="33" t="n">
-        <v>164</v>
+      <c r="M100" s="33" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
       </c>
       <c r="N100" s="33" t="inlineStr">
         <is>
           <t>KAYDEE SONS LLP</t>
-        </is>
-      </c>
-      <c r="O100" s="33" t="inlineStr">
-        <is>
-          <t>1152601597</t>
         </is>
       </c>
     </row>
@@ -6019,17 +5887,14 @@
         </is>
       </c>
       <c r="L112" s="6" t="n"/>
-      <c r="M112" s="33" t="n">
-        <v>178</v>
+      <c r="M112" s="33" t="inlineStr">
+        <is>
+          <t>2916,2926,2928,2934,2939,2958,6,11,17,22,30,40,48,61,75,77,96,109,112,123,139,149,164,170,178,186,200,203,218,236,248,252,270,272,291,297,304,306,326,338,348,356,361,371,387,394,401,408,417</t>
+        </is>
       </c>
       <c r="N112" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O112" s="33" t="inlineStr">
-        <is>
-          <t>2425CRB338228+2425CRB339264+2425CRB340692+2425CRB341892+2425CRB343132+2425CRB344273+2526CRB916+2526CRB2240+2526CRB3521+2526CRB3616+2526CRB4707+2526CRB8694+2526CRB9681+2526CRB10996+2526CRB11983+2526CRB</t>
         </is>
       </c>
     </row>
@@ -6074,15 +5939,12 @@
         </is>
       </c>
       <c r="L113" s="6" t="n"/>
-      <c r="M113" s="33" t="n">
-        <v>159</v>
-      </c>
+      <c r="M113" s="33" t="inlineStr"/>
       <c r="N113" s="33" t="inlineStr">
         <is>
           <t>JAI SHREE GANESH AGENCIES</t>
         </is>
       </c>
-      <c r="O113" s="33" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="21" t="n">
@@ -6125,15 +5987,12 @@
         </is>
       </c>
       <c r="L114" s="6" t="n"/>
-      <c r="M114" s="33" t="n">
-        <v>180</v>
-      </c>
+      <c r="M114" s="33" t="inlineStr"/>
       <c r="N114" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
-      <c r="O114" s="33" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="21" t="n">
@@ -6176,15 +6035,12 @@
         </is>
       </c>
       <c r="L115" s="6" t="n"/>
-      <c r="M115" s="33" t="n">
-        <v>170</v>
-      </c>
+      <c r="M115" s="33" t="inlineStr"/>
       <c r="N115" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
         </is>
       </c>
-      <c r="O115" s="33" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="21" t="n">
@@ -6617,17 +6473,10 @@
         </is>
       </c>
       <c r="L125" s="6" t="n"/>
-      <c r="M125" s="33" t="n">
-        <v>172</v>
-      </c>
+      <c r="M125" s="33" t="inlineStr"/>
       <c r="N125" s="33" t="inlineStr">
         <is>
           <t>N R ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O125" s="33" t="inlineStr">
-        <is>
-          <t>25295909 BY MANOJ</t>
         </is>
       </c>
     </row>
@@ -7204,17 +7053,14 @@
         </is>
       </c>
       <c r="L138" s="6" t="n"/>
-      <c r="M138" s="33" t="n">
-        <v>189</v>
+      <c r="M138" s="33" t="inlineStr">
+        <is>
+          <t>500,501</t>
+        </is>
       </c>
       <c r="N138" s="33" t="inlineStr">
         <is>
           <t>CHINTAMANI DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O138" s="33" t="inlineStr">
-        <is>
-          <t>Z-1519 | Z-1519+Z-1518</t>
         </is>
       </c>
     </row>
@@ -7259,17 +7105,10 @@
         </is>
       </c>
       <c r="L139" s="6" t="n"/>
-      <c r="M139" s="33" t="n">
-        <v>176</v>
-      </c>
+      <c r="M139" s="33" t="inlineStr"/>
       <c r="N139" s="33" t="inlineStr">
         <is>
           <t>AARADHYA AGENCIES</t>
-        </is>
-      </c>
-      <c r="O139" s="33" t="inlineStr">
-        <is>
-          <t>5982</t>
         </is>
       </c>
     </row>
@@ -7448,17 +7287,10 @@
         </is>
       </c>
       <c r="L143" s="6" t="n"/>
-      <c r="M143" s="33" t="n">
-        <v>177</v>
-      </c>
+      <c r="M143" s="33" t="inlineStr"/>
       <c r="N143" s="33" t="inlineStr">
         <is>
           <t>ANURAG CORPORATION PVT.LTD</t>
-        </is>
-      </c>
-      <c r="O143" s="33" t="inlineStr">
-        <is>
-          <t>2243</t>
         </is>
       </c>
     </row>
@@ -7503,15 +7335,12 @@
         </is>
       </c>
       <c r="L144" s="6" t="n"/>
-      <c r="M144" s="33" t="n">
-        <v>171</v>
-      </c>
+      <c r="M144" s="33" t="inlineStr"/>
       <c r="N144" s="33" t="inlineStr">
         <is>
           <t>MOHAN CHEMIST</t>
         </is>
       </c>
-      <c r="O144" s="33" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="21" t="n">
@@ -7604,17 +7433,14 @@
         </is>
       </c>
       <c r="L146" s="6" t="n"/>
-      <c r="M146" s="33" t="n">
-        <v>190</v>
+      <c r="M146" s="33" t="inlineStr">
+        <is>
+          <t>510</t>
+        </is>
       </c>
       <c r="N146" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O146" s="33" t="inlineStr">
-        <is>
-          <t>26507 | 26507</t>
         </is>
       </c>
     </row>
@@ -7885,17 +7711,10 @@
         </is>
       </c>
       <c r="L152" s="6" t="n"/>
-      <c r="M152" s="33" t="n">
-        <v>175</v>
-      </c>
+      <c r="M152" s="33" t="inlineStr"/>
       <c r="N152" s="33" t="inlineStr">
         <is>
           <t>SUYASH MEDICALS</t>
-        </is>
-      </c>
-      <c r="O152" s="33" t="inlineStr">
-        <is>
-          <t>CA/1019</t>
         </is>
       </c>
     </row>
@@ -7940,17 +7759,10 @@
         </is>
       </c>
       <c r="L153" s="6" t="n"/>
-      <c r="M153" s="33" t="n">
-        <v>174</v>
-      </c>
+      <c r="M153" s="33" t="inlineStr"/>
       <c r="N153" s="33" t="inlineStr">
         <is>
           <t>THE PLUS ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O153" s="33" t="inlineStr">
-        <is>
-          <t>5794</t>
         </is>
       </c>
     </row>
@@ -7995,17 +7807,10 @@
         </is>
       </c>
       <c r="L154" s="6" t="n"/>
-      <c r="M154" s="33" t="n">
-        <v>181</v>
-      </c>
+      <c r="M154" s="33" t="inlineStr"/>
       <c r="N154" s="33" t="inlineStr">
         <is>
           <t>SHREE SAI MEDICAL DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O154" s="33" t="inlineStr">
-        <is>
-          <t>CC-1645</t>
         </is>
       </c>
     </row>
@@ -8050,17 +7855,14 @@
         </is>
       </c>
       <c r="L155" s="6" t="n"/>
-      <c r="M155" s="33" t="n">
-        <v>157</v>
+      <c r="M155" s="33" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
       </c>
       <c r="N155" s="33" t="inlineStr">
         <is>
           <t>SHREE DATTA KRUPA AGENCY</t>
-        </is>
-      </c>
-      <c r="O155" s="33" t="inlineStr">
-        <is>
-          <t>4280+4331+5870 | 4280/25-26</t>
         </is>
       </c>
     </row>
@@ -8105,17 +7907,14 @@
         </is>
       </c>
       <c r="L156" s="6" t="n"/>
-      <c r="M156" s="33" t="n">
-        <v>197</v>
+      <c r="M156" s="33" t="inlineStr">
+        <is>
+          <t>466,555</t>
+        </is>
       </c>
       <c r="N156" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O156" s="33" t="inlineStr">
-        <is>
-          <t>/25512+/27544</t>
         </is>
       </c>
     </row>
@@ -8332,17 +8131,10 @@
         </is>
       </c>
       <c r="L161" s="6" t="n"/>
-      <c r="M161" s="33" t="n">
-        <v>169</v>
-      </c>
+      <c r="M161" s="33" t="inlineStr"/>
       <c r="N161" s="33" t="inlineStr">
         <is>
           <t>ROYAL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O161" s="33" t="inlineStr">
-        <is>
-          <t>224 BY MANOJ</t>
         </is>
       </c>
     </row>
@@ -8529,17 +8321,10 @@
         </is>
       </c>
       <c r="L165" s="6" t="n"/>
-      <c r="M165" s="33" t="n">
-        <v>211</v>
-      </c>
+      <c r="M165" s="33" t="inlineStr"/>
       <c r="N165" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O165" s="33" t="inlineStr">
-        <is>
-          <t>AB09499</t>
         </is>
       </c>
     </row>
@@ -8802,17 +8587,10 @@
         </is>
       </c>
       <c r="L171" s="6" t="n"/>
-      <c r="M171" s="33" t="n">
-        <v>191</v>
-      </c>
+      <c r="M171" s="33" t="inlineStr"/>
       <c r="N171" s="33" t="inlineStr">
         <is>
           <t>ADK ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O171" s="33" t="inlineStr">
-        <is>
-          <t>T14530AAA2526</t>
         </is>
       </c>
     </row>
@@ -8857,17 +8635,14 @@
         </is>
       </c>
       <c r="L172" s="6" t="n"/>
-      <c r="M172" s="33" t="n">
-        <v>186</v>
+      <c r="M172" s="33" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
       </c>
       <c r="N172" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O172" s="33" t="inlineStr">
-        <is>
-          <t>16688+15655 | CGSIG-25-I015655</t>
         </is>
       </c>
     </row>
@@ -8912,17 +8687,14 @@
         </is>
       </c>
       <c r="L173" s="6" t="n"/>
-      <c r="M173" s="33" t="n">
-        <v>145</v>
+      <c r="M173" s="33" t="inlineStr">
+        <is>
+          <t>259,252,266,578,573,773</t>
+        </is>
       </c>
       <c r="N173" s="33" t="inlineStr">
         <is>
           <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O173" s="33" t="inlineStr">
-        <is>
-          <t>CR-549+CR-554+CR-651+CR-1453+CR-1501+CR-1979</t>
         </is>
       </c>
     </row>
@@ -8967,17 +8739,10 @@
         </is>
       </c>
       <c r="L174" s="6" t="n"/>
-      <c r="M174" s="33" t="n">
-        <v>195</v>
-      </c>
+      <c r="M174" s="33" t="inlineStr"/>
       <c r="N174" s="33" t="inlineStr">
         <is>
           <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O174" s="33" t="inlineStr">
-        <is>
-          <t>1670</t>
         </is>
       </c>
     </row>
@@ -9022,17 +8787,10 @@
         </is>
       </c>
       <c r="L175" s="6" t="n"/>
-      <c r="M175" s="33" t="n">
-        <v>188</v>
-      </c>
+      <c r="M175" s="33" t="inlineStr"/>
       <c r="N175" s="33" t="inlineStr">
         <is>
           <t>KHAMANG BEST CHIWDA</t>
-        </is>
-      </c>
-      <c r="O175" s="33" t="inlineStr">
-        <is>
-          <t>A635</t>
         </is>
       </c>
     </row>
@@ -9303,17 +9061,10 @@
         </is>
       </c>
       <c r="L181" s="6" t="n"/>
-      <c r="M181" s="33" t="n">
-        <v>192</v>
-      </c>
+      <c r="M181" s="33" t="inlineStr"/>
       <c r="N181" s="33" t="inlineStr">
         <is>
           <t>DHYAANI NEXUS PVT.LTD.</t>
-        </is>
-      </c>
-      <c r="O181" s="33" t="inlineStr">
-        <is>
-          <t>CC-1796</t>
         </is>
       </c>
     </row>
@@ -10150,17 +9901,10 @@
         </is>
       </c>
       <c r="L200" s="6" t="n"/>
-      <c r="M200" s="33" t="n">
-        <v>193</v>
-      </c>
+      <c r="M200" s="33" t="inlineStr"/>
       <c r="N200" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O200" s="33" t="inlineStr">
-        <is>
-          <t>485/25-26</t>
         </is>
       </c>
     </row>
@@ -11077,15 +10821,12 @@
         </is>
       </c>
       <c r="L221" s="6" t="n"/>
-      <c r="M221" s="33" t="n">
-        <v>217</v>
-      </c>
+      <c r="M221" s="33" t="inlineStr"/>
       <c r="N221" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
-      <c r="O221" s="33" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="21" t="n">
@@ -11128,17 +10869,10 @@
         </is>
       </c>
       <c r="L222" s="6" t="n"/>
-      <c r="M222" s="33" t="n">
-        <v>212</v>
-      </c>
+      <c r="M222" s="33" t="inlineStr"/>
       <c r="N222" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
-        </is>
-      </c>
-      <c r="O222" s="33" t="inlineStr">
-        <is>
-          <t>PD/25/2658</t>
         </is>
       </c>
     </row>
@@ -11183,15 +10917,12 @@
         </is>
       </c>
       <c r="L223" s="6" t="n"/>
-      <c r="M223" s="33" t="n">
-        <v>218</v>
-      </c>
+      <c r="M223" s="33" t="inlineStr"/>
       <c r="N223" s="33" t="inlineStr">
         <is>
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
-      <c r="O223" s="33" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="21" t="n">
@@ -11234,17 +10965,10 @@
         </is>
       </c>
       <c r="L224" s="6" t="n"/>
-      <c r="M224" s="33" t="n">
-        <v>194</v>
-      </c>
+      <c r="M224" s="33" t="inlineStr"/>
       <c r="N224" s="33" t="inlineStr">
         <is>
           <t>YASH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O224" s="33" t="inlineStr">
-        <is>
-          <t>177</t>
         </is>
       </c>
     </row>
@@ -11507,17 +11231,10 @@
         </is>
       </c>
       <c r="L230" s="6" t="n"/>
-      <c r="M230" s="33" t="n">
-        <v>215</v>
-      </c>
+      <c r="M230" s="33" t="inlineStr"/>
       <c r="N230" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O230" s="33" t="inlineStr">
-        <is>
-          <t>A000892</t>
         </is>
       </c>
     </row>
@@ -11742,17 +11459,10 @@
         </is>
       </c>
       <c r="L235" s="6" t="n"/>
-      <c r="M235" s="33" t="n">
-        <v>185</v>
-      </c>
+      <c r="M235" s="33" t="inlineStr"/>
       <c r="N235" s="33" t="inlineStr">
         <is>
           <t>RADIANT ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O235" s="33" t="inlineStr">
-        <is>
-          <t>1773/25-26</t>
         </is>
       </c>
     </row>
@@ -12595,17 +12305,10 @@
         </is>
       </c>
       <c r="L254" s="6" t="n"/>
-      <c r="M254" s="33" t="n">
-        <v>182</v>
-      </c>
+      <c r="M254" s="33" t="inlineStr"/>
       <c r="N254" s="33" t="inlineStr">
         <is>
           <t>SAMARTH AYURVEDIC</t>
-        </is>
-      </c>
-      <c r="O254" s="33" t="inlineStr">
-        <is>
-          <t>2526CCB811</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12351,14 @@
         </is>
       </c>
       <c r="L255" s="6" t="n"/>
-      <c r="M255" s="33" t="n">
-        <v>235</v>
+      <c r="M255" s="33" t="inlineStr">
+        <is>
+          <t>514,588</t>
+        </is>
       </c>
       <c r="N255" s="33" t="inlineStr">
         <is>
           <t>SHINDE ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O255" s="33" t="inlineStr">
-        <is>
-          <t>CC/1739+CC/1949</t>
         </is>
       </c>
     </row>
@@ -12701,15 +12401,12 @@
         </is>
       </c>
       <c r="L256" s="6" t="n"/>
-      <c r="M256" s="33" t="n">
-        <v>219</v>
-      </c>
+      <c r="M256" s="33" t="inlineStr"/>
       <c r="N256" s="33" t="inlineStr">
         <is>
           <t>SAI KRUPA AGENCY</t>
         </is>
       </c>
-      <c r="O256" s="33" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="21" t="n">
@@ -12750,17 +12447,14 @@
         </is>
       </c>
       <c r="L257" s="6" t="n"/>
-      <c r="M257" s="33" t="n">
-        <v>233</v>
+      <c r="M257" s="33" t="inlineStr">
+        <is>
+          <t>5,8,46,49,91,105,138,152,162,180,188,215,220,237,243,263,288,299,325,342,346,358,365,378,388,392,404,433</t>
+        </is>
       </c>
       <c r="N257" s="33" t="inlineStr">
         <is>
           <t>MAHENDRA DISRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O257" s="33" t="inlineStr">
-        <is>
-          <t>S/76+S/250+S/1180+S/1296+S/1965+S/2576+S/3044+S/3450+S/3553+S/3861+S/4144+S/4657+S/4841+S/5193+S/5336+S/5702+S/5991+S/6161+S/6542+S/6819+S/6975+S/7219+S/7356+S/7537+S/7657+S/7885+S/8080+S/8804</t>
         </is>
       </c>
     </row>
@@ -12803,17 +12497,10 @@
         </is>
       </c>
       <c r="L258" s="6" t="n"/>
-      <c r="M258" s="33" t="n">
-        <v>216</v>
-      </c>
+      <c r="M258" s="33" t="inlineStr"/>
       <c r="N258" s="33" t="inlineStr">
         <is>
           <t>V R ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O258" s="33" t="inlineStr">
-        <is>
-          <t>SR25-26/01066</t>
         </is>
       </c>
     </row>
@@ -13068,17 +12755,14 @@
         </is>
       </c>
       <c r="L264" s="6" t="n"/>
-      <c r="M264" s="33" t="n">
-        <v>234</v>
+      <c r="M264" s="33" t="inlineStr">
+        <is>
+          <t>513</t>
+        </is>
       </c>
       <c r="N264" s="33" t="inlineStr">
         <is>
           <t>MANGAL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O264" s="33" t="inlineStr">
-        <is>
-          <t>DR/25-26/02243</t>
         </is>
       </c>
     </row>
@@ -13209,15 +12893,12 @@
         </is>
       </c>
       <c r="L267" s="6" t="n"/>
-      <c r="M267" s="33" t="n">
-        <v>161</v>
-      </c>
+      <c r="M267" s="33" t="inlineStr"/>
       <c r="N267" s="33" t="inlineStr">
         <is>
           <t>KRISHNA MEDICAL &amp; SURGICAL</t>
         </is>
       </c>
-      <c r="O267" s="33" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" s="21" t="n">
@@ -13258,17 +12939,10 @@
         </is>
       </c>
       <c r="L268" s="6" t="n"/>
-      <c r="M268" s="33" t="n">
-        <v>221</v>
-      </c>
+      <c r="M268" s="33" t="inlineStr"/>
       <c r="N268" s="33" t="inlineStr">
         <is>
           <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O268" s="33" t="inlineStr">
-        <is>
-          <t>A045502359</t>
         </is>
       </c>
     </row>
@@ -13311,17 +12985,10 @@
         </is>
       </c>
       <c r="L269" s="6" t="n"/>
-      <c r="M269" s="33" t="n">
-        <v>261</v>
-      </c>
+      <c r="M269" s="33" t="inlineStr"/>
       <c r="N269" s="33" t="inlineStr">
         <is>
           <t>SHREE GANESH ENTERPISES</t>
-        </is>
-      </c>
-      <c r="O269" s="33" t="inlineStr">
-        <is>
-          <t>- SGE534</t>
         </is>
       </c>
     </row>
@@ -13500,17 +13167,10 @@
         </is>
       </c>
       <c r="L273" s="6" t="n"/>
-      <c r="M273" s="33" t="n">
-        <v>213</v>
-      </c>
+      <c r="M273" s="33" t="inlineStr"/>
       <c r="N273" s="33" t="inlineStr">
         <is>
           <t>ARIHANT ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O273" s="33" t="inlineStr">
-        <is>
-          <t>A2VL-2526/0394</t>
         </is>
       </c>
     </row>
@@ -13553,17 +13213,10 @@
         </is>
       </c>
       <c r="L274" s="6" t="n"/>
-      <c r="M274" s="33" t="n">
-        <v>243</v>
-      </c>
+      <c r="M274" s="33" t="inlineStr"/>
       <c r="N274" s="33" t="inlineStr">
         <is>
           <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O274" s="33" t="inlineStr">
-        <is>
-          <t>2052</t>
         </is>
       </c>
     </row>
@@ -13694,17 +13347,10 @@
         </is>
       </c>
       <c r="L277" s="6" t="n"/>
-      <c r="M277" s="33" t="n">
-        <v>246</v>
-      </c>
+      <c r="M277" s="33" t="inlineStr"/>
       <c r="N277" s="33" t="inlineStr">
         <is>
           <t>AARADHYA AGENCIES</t>
-        </is>
-      </c>
-      <c r="O277" s="33" t="inlineStr">
-        <is>
-          <t>IN10056782507963</t>
         </is>
       </c>
     </row>
@@ -13747,17 +13393,10 @@
         </is>
       </c>
       <c r="L278" s="6" t="n"/>
-      <c r="M278" s="33" t="n">
-        <v>244</v>
-      </c>
+      <c r="M278" s="33" t="inlineStr"/>
       <c r="N278" s="33" t="inlineStr">
         <is>
           <t>SHRI KULSWAMINI DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O278" s="33" t="inlineStr">
-        <is>
-          <t>4565</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13439,10 @@
         </is>
       </c>
       <c r="L279" s="6" t="n"/>
-      <c r="M279" s="33" t="n">
-        <v>214</v>
-      </c>
+      <c r="M279" s="33" t="inlineStr"/>
       <c r="N279" s="33" t="inlineStr">
         <is>
           <t>SAI MARKETING</t>
-        </is>
-      </c>
-      <c r="O279" s="33" t="inlineStr">
-        <is>
-          <t>CC-1380</t>
         </is>
       </c>
     </row>
@@ -13853,17 +13485,10 @@
         </is>
       </c>
       <c r="L280" s="6" t="n"/>
-      <c r="M280" s="33" t="n">
-        <v>240</v>
-      </c>
+      <c r="M280" s="33" t="inlineStr"/>
       <c r="N280" s="33" t="inlineStr">
         <is>
           <t>RAUT TRADINGS</t>
-        </is>
-      </c>
-      <c r="O280" s="33" t="inlineStr">
-        <is>
-          <t>INV-017656</t>
         </is>
       </c>
     </row>
@@ -14082,17 +13707,10 @@
         </is>
       </c>
       <c r="L285" s="6" t="n"/>
-      <c r="M285" s="33" t="n">
-        <v>265</v>
-      </c>
+      <c r="M285" s="33" t="inlineStr"/>
       <c r="N285" s="33" t="inlineStr">
         <is>
           <t>YASH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O285" s="33" t="inlineStr">
-        <is>
-          <t>-73 DATE 2/5/25</t>
         </is>
       </c>
     </row>
@@ -14135,15 +13753,12 @@
         </is>
       </c>
       <c r="L286" s="6" t="n"/>
-      <c r="M286" s="33" t="n">
-        <v>245</v>
-      </c>
+      <c r="M286" s="33" t="inlineStr"/>
       <c r="N286" s="33" t="inlineStr">
         <is>
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
-      <c r="O286" s="33" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="21" t="n">
@@ -14232,17 +13847,10 @@
         </is>
       </c>
       <c r="L288" s="6" t="n"/>
-      <c r="M288" s="33" t="n">
-        <v>220</v>
-      </c>
+      <c r="M288" s="33" t="inlineStr"/>
       <c r="N288" s="33" t="inlineStr">
         <is>
           <t>SONIGARA DISTRIBUTOR</t>
-        </is>
-      </c>
-      <c r="O288" s="33" t="inlineStr">
-        <is>
-          <t>SD-2267/25-26</t>
         </is>
       </c>
     </row>
@@ -14285,17 +13893,10 @@
         </is>
       </c>
       <c r="L289" s="6" t="n"/>
-      <c r="M289" s="33" t="n">
-        <v>262</v>
-      </c>
+      <c r="M289" s="33" t="inlineStr"/>
       <c r="N289" s="33" t="inlineStr">
         <is>
           <t>N R ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O289" s="33" t="inlineStr">
-        <is>
-          <t>-IBAL25302084</t>
         </is>
       </c>
     </row>
@@ -14338,17 +13939,10 @@
         </is>
       </c>
       <c r="L290" s="6" t="n"/>
-      <c r="M290" s="33" t="n">
-        <v>242</v>
-      </c>
+      <c r="M290" s="33" t="inlineStr"/>
       <c r="N290" s="33" t="inlineStr">
         <is>
           <t>TAPADIYA COSMOGEN</t>
-        </is>
-      </c>
-      <c r="O290" s="33" t="inlineStr">
-        <is>
-          <t>PCC4182/25-26</t>
         </is>
       </c>
     </row>
@@ -14391,15 +13985,12 @@
         </is>
       </c>
       <c r="L291" s="6" t="n"/>
-      <c r="M291" s="33" t="n">
-        <v>183</v>
-      </c>
+      <c r="M291" s="33" t="inlineStr"/>
       <c r="N291" s="33" t="inlineStr">
         <is>
           <t>GOVINDA FOODS</t>
         </is>
       </c>
-      <c r="O291" s="33" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" s="21" t="n">
@@ -14440,17 +14031,14 @@
         </is>
       </c>
       <c r="L292" s="6" t="n"/>
-      <c r="M292" s="33" t="n">
-        <v>241</v>
+      <c r="M292" s="33" t="inlineStr">
+        <is>
+          <t>386,420,440,483</t>
+        </is>
       </c>
       <c r="N292" s="33" t="inlineStr">
         <is>
           <t>SUMEET AGENCIES</t>
-        </is>
-      </c>
-      <c r="O292" s="33" t="inlineStr">
-        <is>
-          <t>GTB33883+GTB36082+GTB35991+GTB38086</t>
         </is>
       </c>
     </row>
@@ -14789,17 +14377,10 @@
         </is>
       </c>
       <c r="L300" s="6" t="n"/>
-      <c r="M300" s="33" t="n">
-        <v>260</v>
-      </c>
+      <c r="M300" s="33" t="inlineStr"/>
       <c r="N300" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O300" s="33" t="inlineStr">
-        <is>
-          <t>-45/25-26</t>
         </is>
       </c>
     </row>
@@ -14842,17 +14423,10 @@
         </is>
       </c>
       <c r="L301" s="6" t="n"/>
-      <c r="M301" s="33" t="n">
-        <v>257</v>
-      </c>
+      <c r="M301" s="33" t="inlineStr"/>
       <c r="N301" s="33" t="inlineStr">
         <is>
           <t>SHINDE ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O301" s="33" t="inlineStr">
-        <is>
-          <t>-MLB161752507125</t>
         </is>
       </c>
     </row>
@@ -15559,17 +15133,10 @@
         </is>
       </c>
       <c r="L318" s="6" t="n"/>
-      <c r="M318" s="33" t="n">
-        <v>254</v>
-      </c>
+      <c r="M318" s="33" t="inlineStr"/>
       <c r="N318" s="33" t="inlineStr">
         <is>
           <t>JEEVIKA HOSPITALITY SERVICES</t>
-        </is>
-      </c>
-      <c r="O318" s="33" t="inlineStr">
-        <is>
-          <t>3545</t>
         </is>
       </c>
     </row>
@@ -16256,17 +15823,10 @@
         </is>
       </c>
       <c r="L334" s="6" t="n"/>
-      <c r="M334" s="33" t="n">
-        <v>264</v>
-      </c>
+      <c r="M334" s="33" t="inlineStr"/>
       <c r="N334" s="33" t="inlineStr">
         <is>
           <t>SUMEET AGENCIES</t>
-        </is>
-      </c>
-      <c r="O334" s="33" t="inlineStr">
-        <is>
-          <t>-GTB49382</t>
         </is>
       </c>
     </row>
@@ -16397,17 +15957,14 @@
         </is>
       </c>
       <c r="L337" s="6" t="n"/>
-      <c r="M337" s="33" t="n">
-        <v>83</v>
+      <c r="M337" s="33" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
       </c>
       <c r="N337" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O337" s="33" t="inlineStr">
-        <is>
-          <t>169/25-26</t>
         </is>
       </c>
     </row>
@@ -16450,17 +16007,10 @@
         </is>
       </c>
       <c r="L338" s="6" t="n"/>
-      <c r="M338" s="33" t="n">
-        <v>268</v>
-      </c>
+      <c r="M338" s="33" t="inlineStr"/>
       <c r="N338" s="33" t="inlineStr">
         <is>
           <t>CHINTAMANI DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O338" s="33" t="inlineStr">
-        <is>
-          <t>-H-3461 ,Z-2132</t>
         </is>
       </c>
     </row>
@@ -16503,17 +16053,10 @@
         </is>
       </c>
       <c r="L339" s="6" t="n"/>
-      <c r="M339" s="33" t="n">
-        <v>248</v>
-      </c>
+      <c r="M339" s="33" t="inlineStr"/>
       <c r="N339" s="33" t="inlineStr">
         <is>
           <t>UNICO AGENCIES</t>
-        </is>
-      </c>
-      <c r="O339" s="33" t="inlineStr">
-        <is>
-          <t>A001385</t>
         </is>
       </c>
     </row>
@@ -16556,17 +16099,10 @@
         </is>
       </c>
       <c r="L340" s="6" t="n"/>
-      <c r="M340" s="33" t="n">
-        <v>21</v>
-      </c>
+      <c r="M340" s="33" t="inlineStr"/>
       <c r="N340" s="33" t="inlineStr">
         <is>
           <t>PRASHANT-NX</t>
-        </is>
-      </c>
-      <c r="O340" s="33" t="inlineStr">
-        <is>
-          <t>CA-172</t>
         </is>
       </c>
     </row>
@@ -16609,17 +16145,14 @@
         </is>
       </c>
       <c r="L341" s="6" t="n"/>
-      <c r="M341" s="33" t="n">
-        <v>83</v>
+      <c r="M341" s="33" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
       </c>
       <c r="N341" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O341" s="33" t="inlineStr">
-        <is>
-          <t>169/25-26</t>
         </is>
       </c>
     </row>
@@ -17046,17 +16579,10 @@
         </is>
       </c>
       <c r="L351" s="6" t="n"/>
-      <c r="M351" s="33" t="n">
-        <v>259</v>
-      </c>
+      <c r="M351" s="33" t="inlineStr"/>
       <c r="N351" s="33" t="inlineStr">
         <is>
           <t>ASHA MOHAN ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O351" s="33" t="inlineStr">
-        <is>
-          <t>-002474</t>
         </is>
       </c>
     </row>
@@ -17267,17 +16793,10 @@
         </is>
       </c>
       <c r="L356" s="6" t="n"/>
-      <c r="M356" s="33" t="n">
-        <v>289</v>
-      </c>
+      <c r="M356" s="33" t="inlineStr"/>
       <c r="N356" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O356" s="33" t="inlineStr">
-        <is>
-          <t>AB13968</t>
         </is>
       </c>
     </row>
@@ -17320,17 +16839,10 @@
         </is>
       </c>
       <c r="L357" s="6" t="n"/>
-      <c r="M357" s="33" t="n">
-        <v>280</v>
-      </c>
+      <c r="M357" s="33" t="inlineStr"/>
       <c r="N357" s="33" t="inlineStr">
         <is>
           <t>RAUT TRADINGS</t>
-        </is>
-      </c>
-      <c r="O357" s="33" t="inlineStr">
-        <is>
-          <t>-INV-017740</t>
         </is>
       </c>
     </row>
@@ -17373,17 +16885,14 @@
         </is>
       </c>
       <c r="L358" s="6" t="n"/>
-      <c r="M358" s="33" t="n">
-        <v>269</v>
+      <c r="M358" s="33" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
       </c>
       <c r="N358" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O358" s="33" t="inlineStr">
-        <is>
-          <t>-38382 | 38382</t>
         </is>
       </c>
     </row>
@@ -17806,17 +17315,14 @@
         </is>
       </c>
       <c r="L368" s="6" t="n"/>
-      <c r="M368" s="33" t="n">
-        <v>279</v>
+      <c r="M368" s="33" t="inlineStr">
+        <is>
+          <t>2864,2878,2886,2889,2901,2914,2915,2923,2925,2937,2944,2949,2950,16,34,159,213,249,269,289,302,311,375,416,432</t>
+        </is>
       </c>
       <c r="N368" s="33" t="inlineStr">
         <is>
           <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O368" s="33" t="inlineStr">
-        <is>
-          <t>MD/32148+MD/32294+MD/32369+MD/32481+MD/32569+MD/32740+MD/32840+MD/32918+MD/32945+MD/33069+MD/33292+MD/33420+MD/33414+MD/343+MD/862+MD/2391+MD/3141+MD/3605+MD/3879+MD/4096+MD/4248+MD/4330+MD/5111+MD/57</t>
         </is>
       </c>
     </row>
@@ -17939,17 +17445,10 @@
         </is>
       </c>
       <c r="L371" s="6" t="n"/>
-      <c r="M371" s="33" t="n">
-        <v>281</v>
-      </c>
+      <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
           <t>G K ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O371" s="33" t="inlineStr">
-        <is>
-          <t>-15975</t>
         </is>
       </c>
     </row>
@@ -18336,15 +17835,12 @@
         </is>
       </c>
       <c r="L380" s="6" t="n"/>
-      <c r="M380" s="33" t="n">
-        <v>283</v>
-      </c>
+      <c r="M380" s="33" t="inlineStr"/>
       <c r="N380" s="33" t="inlineStr">
         <is>
           <t>SANIKA ENTERPRISES</t>
         </is>
       </c>
-      <c r="O380" s="33" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" s="21" t="n">
@@ -18425,17 +17921,10 @@
         </is>
       </c>
       <c r="L382" s="6" t="n"/>
-      <c r="M382" s="33" t="n">
-        <v>284</v>
-      </c>
+      <c r="M382" s="33" t="inlineStr"/>
       <c r="N382" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O382" s="33" t="inlineStr">
-        <is>
-          <t>-720/25-26  683/25-26</t>
         </is>
       </c>
     </row>
@@ -18518,17 +18007,10 @@
         </is>
       </c>
       <c r="L384" s="6" t="n"/>
-      <c r="M384" s="33" t="n">
-        <v>287</v>
-      </c>
+      <c r="M384" s="33" t="inlineStr"/>
       <c r="N384" s="33" t="inlineStr">
         <is>
           <t>SHREE GANESH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O384" s="33" t="inlineStr">
-        <is>
-          <t>SGE616</t>
         </is>
       </c>
     </row>
@@ -18787,17 +18269,10 @@
         </is>
       </c>
       <c r="L390" s="6" t="n"/>
-      <c r="M390" s="33" t="n">
-        <v>296</v>
-      </c>
+      <c r="M390" s="33" t="inlineStr"/>
       <c r="N390" s="33" t="inlineStr">
         <is>
           <t>V R ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O390" s="33" t="inlineStr">
-        <is>
-          <t>-SR25-26/0415</t>
         </is>
       </c>
     </row>
@@ -18840,17 +18315,10 @@
         </is>
       </c>
       <c r="L391" s="6" t="n"/>
-      <c r="M391" s="33" t="n">
-        <v>282</v>
-      </c>
+      <c r="M391" s="33" t="inlineStr"/>
       <c r="N391" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O391" s="33" t="inlineStr">
-        <is>
-          <t>-39624</t>
         </is>
       </c>
     </row>
@@ -18893,17 +18361,14 @@
         </is>
       </c>
       <c r="L392" s="6" t="n"/>
-      <c r="M392" s="33" t="n">
-        <v>263</v>
+      <c r="M392" s="33" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
       </c>
       <c r="N392" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O392" s="33" t="inlineStr">
-        <is>
-          <t>-37304 | 37304</t>
         </is>
       </c>
     </row>
@@ -18994,17 +18459,10 @@
         </is>
       </c>
       <c r="L394" s="6" t="n"/>
-      <c r="M394" s="33" t="n">
-        <v>292</v>
-      </c>
+      <c r="M394" s="33" t="inlineStr"/>
       <c r="N394" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
-        </is>
-      </c>
-      <c r="O394" s="33" t="inlineStr">
-        <is>
-          <t>PD/25/3601</t>
         </is>
       </c>
     </row>
@@ -19087,17 +18545,10 @@
         </is>
       </c>
       <c r="L396" s="6" t="n"/>
-      <c r="M396" s="33" t="n">
-        <v>288</v>
-      </c>
+      <c r="M396" s="33" t="inlineStr"/>
       <c r="N396" s="33" t="inlineStr">
         <is>
           <t>REKHA MARKETING</t>
-        </is>
-      </c>
-      <c r="O396" s="33" t="inlineStr">
-        <is>
-          <t>-RM832</t>
         </is>
       </c>
     </row>
@@ -19140,17 +18591,10 @@
         </is>
       </c>
       <c r="L397" s="6" t="n"/>
-      <c r="M397" s="33" t="n">
-        <v>299</v>
-      </c>
+      <c r="M397" s="33" t="inlineStr"/>
       <c r="N397" s="33" t="inlineStr">
         <is>
           <t>NANDINI BEAUTY</t>
-        </is>
-      </c>
-      <c r="O397" s="33" t="inlineStr">
-        <is>
-          <t>49 BILL DATE 03/05/202</t>
         </is>
       </c>
     </row>
@@ -19241,17 +18685,10 @@
         </is>
       </c>
       <c r="L399" s="6" t="n"/>
-      <c r="M399" s="33" t="n">
-        <v>285</v>
-      </c>
+      <c r="M399" s="33" t="inlineStr"/>
       <c r="N399" s="33" t="inlineStr">
         <is>
           <t>JAI SHREE GANESH AGENCIES</t>
-        </is>
-      </c>
-      <c r="O399" s="33" t="inlineStr">
-        <is>
-          <t>-I/25-26/006642</t>
         </is>
       </c>
     </row>
@@ -19294,17 +18731,10 @@
         </is>
       </c>
       <c r="L400" s="6" t="n"/>
-      <c r="M400" s="33" t="n">
-        <v>270</v>
-      </c>
+      <c r="M400" s="33" t="inlineStr"/>
       <c r="N400" s="33" t="inlineStr">
         <is>
           <t>HEALTH PLUS MEDICO</t>
-        </is>
-      </c>
-      <c r="O400" s="33" t="inlineStr">
-        <is>
-          <t>- CR/2930</t>
         </is>
       </c>
     </row>
@@ -19347,17 +18777,10 @@
         </is>
       </c>
       <c r="L401" s="6" t="n"/>
-      <c r="M401" s="33" t="n">
-        <v>291</v>
-      </c>
+      <c r="M401" s="33" t="inlineStr"/>
       <c r="N401" s="33" t="inlineStr">
         <is>
           <t>SARTHAK SALES AGENCY</t>
-        </is>
-      </c>
-      <c r="O401" s="33" t="inlineStr">
-        <is>
-          <t>SSA/163/2025-26</t>
         </is>
       </c>
     </row>
@@ -19528,15 +18951,12 @@
         </is>
       </c>
       <c r="L405" s="6" t="n"/>
-      <c r="M405" s="33" t="n">
-        <v>336</v>
-      </c>
+      <c r="M405" s="33" t="inlineStr"/>
       <c r="N405" s="33" t="inlineStr">
         <is>
           <t>SHREYAA AGENCIES</t>
         </is>
       </c>
-      <c r="O405" s="33" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" s="21" t="n">
@@ -20341,17 +19761,10 @@
         </is>
       </c>
       <c r="L424" s="6" t="n"/>
-      <c r="M424" s="33" t="n">
-        <v>293</v>
-      </c>
+      <c r="M424" s="33" t="inlineStr"/>
       <c r="N424" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O424" s="33" t="inlineStr">
-        <is>
-          <t>-A001234</t>
         </is>
       </c>
     </row>
@@ -20394,17 +19807,10 @@
         </is>
       </c>
       <c r="L425" s="6" t="n"/>
-      <c r="M425" s="33" t="n">
-        <v>297</v>
-      </c>
+      <c r="M425" s="33" t="inlineStr"/>
       <c r="N425" s="33" t="inlineStr">
         <is>
           <t>SUMEET AGENCIES</t>
-        </is>
-      </c>
-      <c r="O425" s="33" t="inlineStr">
-        <is>
-          <t>-GTB46294,GTB43549</t>
         </is>
       </c>
     </row>
@@ -20487,17 +19893,14 @@
         </is>
       </c>
       <c r="L427" s="6" t="n"/>
-      <c r="M427" s="33" t="n">
-        <v>83</v>
+      <c r="M427" s="33" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
       </c>
       <c r="N427" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O427" s="33" t="inlineStr">
-        <is>
-          <t>169/25-26</t>
         </is>
       </c>
     </row>
@@ -20716,17 +20119,10 @@
         </is>
       </c>
       <c r="L432" s="6" t="n"/>
-      <c r="M432" s="33" t="n">
-        <v>300</v>
-      </c>
+      <c r="M432" s="33" t="inlineStr"/>
       <c r="N432" s="33" t="inlineStr">
         <is>
           <t>THE MEDI SHOPEE</t>
-        </is>
-      </c>
-      <c r="O432" s="33" t="inlineStr">
-        <is>
-          <t>CC/TMS551</t>
         </is>
       </c>
     </row>
@@ -20857,17 +20253,10 @@
         </is>
       </c>
       <c r="L435" s="6" t="n"/>
-      <c r="M435" s="33" t="n">
-        <v>270</v>
-      </c>
+      <c r="M435" s="33" t="inlineStr"/>
       <c r="N435" s="33" t="inlineStr">
         <is>
           <t>HEALTH PLUS MEDICO</t>
-        </is>
-      </c>
-      <c r="O435" s="33" t="inlineStr">
-        <is>
-          <t>- CR/2930</t>
         </is>
       </c>
     </row>
@@ -20958,15 +20347,12 @@
         </is>
       </c>
       <c r="L437" s="6" t="n"/>
-      <c r="M437" s="33" t="n">
-        <v>304</v>
-      </c>
+      <c r="M437" s="33" t="inlineStr"/>
       <c r="N437" s="33" t="inlineStr">
         <is>
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
-      <c r="O437" s="33" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" s="21" t="n">
@@ -21007,15 +20393,12 @@
         </is>
       </c>
       <c r="L438" s="6" t="n"/>
-      <c r="M438" s="33" t="n">
-        <v>306</v>
-      </c>
+      <c r="M438" s="33" t="inlineStr"/>
       <c r="N438" s="33" t="inlineStr">
         <is>
           <t>MOHAN CHEMIST</t>
         </is>
       </c>
-      <c r="O438" s="33" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" s="21" t="n">
@@ -21188,17 +20571,10 @@
         </is>
       </c>
       <c r="L442" s="6" t="n"/>
-      <c r="M442" s="33" t="n">
-        <v>312</v>
-      </c>
+      <c r="M442" s="33" t="inlineStr"/>
       <c r="N442" s="33" t="inlineStr">
         <is>
           <t>N R ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O442" s="33" t="inlineStr">
-        <is>
-          <t>IBAL25306531</t>
         </is>
       </c>
     </row>
@@ -21241,17 +20617,14 @@
         </is>
       </c>
       <c r="L443" s="6" t="n"/>
-      <c r="M443" s="33" t="n">
-        <v>294</v>
+      <c r="M443" s="33" t="inlineStr">
+        <is>
+          <t>419,453,541,717</t>
+        </is>
       </c>
       <c r="N443" s="33" t="inlineStr">
         <is>
           <t>SHREE DATTA KRUPA AGENCY</t>
-        </is>
-      </c>
-      <c r="O443" s="33" t="inlineStr">
-        <is>
-          <t>5953/25-26+5979/25-26+7084/25-26+8522/25-26</t>
         </is>
       </c>
     </row>
@@ -21966,17 +21339,10 @@
         </is>
       </c>
       <c r="L460" s="6" t="n"/>
-      <c r="M460" s="33" t="n">
-        <v>301</v>
-      </c>
+      <c r="M460" s="33" t="inlineStr"/>
       <c r="N460" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O460" s="33" t="inlineStr">
-        <is>
-          <t>20716</t>
         </is>
       </c>
     </row>
@@ -22311,17 +21677,10 @@
         </is>
       </c>
       <c r="L468" s="6" t="n"/>
-      <c r="M468" s="33" t="n">
-        <v>305</v>
-      </c>
+      <c r="M468" s="33" t="inlineStr"/>
       <c r="N468" s="33" t="inlineStr">
         <is>
           <t>JEEVIKA HOSPITALITY SERVICES</t>
-        </is>
-      </c>
-      <c r="O468" s="33" t="inlineStr">
-        <is>
-          <t>4640</t>
         </is>
       </c>
     </row>
@@ -22404,17 +21763,10 @@
         </is>
       </c>
       <c r="L470" s="6" t="n"/>
-      <c r="M470" s="33" t="n">
-        <v>302</v>
-      </c>
+      <c r="M470" s="33" t="inlineStr"/>
       <c r="N470" s="33" t="inlineStr">
         <is>
           <t>SWARA ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O470" s="33" t="inlineStr">
-        <is>
-          <t>-A000638 ,A000524 AMOUNT</t>
         </is>
       </c>
     </row>
@@ -23709,15 +23061,12 @@
         </is>
       </c>
       <c r="L501" s="6" t="n"/>
-      <c r="M501" s="33" t="n">
-        <v>310</v>
-      </c>
+      <c r="M501" s="33" t="inlineStr"/>
       <c r="N501" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
         </is>
       </c>
-      <c r="O501" s="33" t="inlineStr"/>
     </row>
     <row r="502">
       <c r="A502" s="21" t="n">
@@ -23758,17 +23107,10 @@
         </is>
       </c>
       <c r="L502" s="6" t="n"/>
-      <c r="M502" s="33" t="n">
-        <v>307</v>
-      </c>
+      <c r="M502" s="33" t="inlineStr"/>
       <c r="N502" s="33" t="inlineStr">
         <is>
           <t>HEALTH PLUS MEDICO</t>
-        </is>
-      </c>
-      <c r="O502" s="33" t="inlineStr">
-        <is>
-          <t>CR/4179</t>
         </is>
       </c>
     </row>
@@ -23891,17 +23233,10 @@
         </is>
       </c>
       <c r="L505" s="6" t="n"/>
-      <c r="M505" s="33" t="n">
-        <v>309</v>
-      </c>
+      <c r="M505" s="33" t="inlineStr"/>
       <c r="N505" s="33" t="inlineStr">
         <is>
           <t>DHYAANI NEXUS PVT.LTD.</t>
-        </is>
-      </c>
-      <c r="O505" s="33" t="inlineStr">
-        <is>
-          <t>-CC-2948</t>
         </is>
       </c>
     </row>
@@ -24112,17 +23447,10 @@
         </is>
       </c>
       <c r="L510" s="6" t="n"/>
-      <c r="M510" s="33" t="n">
-        <v>313</v>
-      </c>
+      <c r="M510" s="33" t="inlineStr"/>
       <c r="N510" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O510" s="33" t="inlineStr">
-        <is>
-          <t>A001441</t>
         </is>
       </c>
     </row>
@@ -24165,17 +23493,14 @@
         </is>
       </c>
       <c r="L511" s="6" t="n"/>
-      <c r="M511" s="33" t="n">
-        <v>322</v>
+      <c r="M511" s="33" t="inlineStr">
+        <is>
+          <t>947</t>
+        </is>
       </c>
       <c r="N511" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
-        </is>
-      </c>
-      <c r="O511" s="33" t="inlineStr">
-        <is>
-          <t>DL25-1,531</t>
         </is>
       </c>
     </row>
@@ -24218,17 +23543,10 @@
         </is>
       </c>
       <c r="L512" s="6" t="n"/>
-      <c r="M512" s="33" t="n">
-        <v>311</v>
-      </c>
+      <c r="M512" s="33" t="inlineStr"/>
       <c r="N512" s="33" t="inlineStr">
         <is>
           <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O512" s="33" t="inlineStr">
-        <is>
-          <t>844/25-26</t>
         </is>
       </c>
     </row>
@@ -24271,17 +23589,10 @@
         </is>
       </c>
       <c r="L513" s="6" t="n"/>
-      <c r="M513" s="33" t="n">
-        <v>324</v>
-      </c>
+      <c r="M513" s="33" t="inlineStr"/>
       <c r="N513" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O513" s="33" t="inlineStr">
-        <is>
-          <t>-AB17251</t>
         </is>
       </c>
     </row>
@@ -24324,17 +23635,10 @@
         </is>
       </c>
       <c r="L514" s="6" t="n"/>
-      <c r="M514" s="33" t="n">
-        <v>313</v>
-      </c>
+      <c r="M514" s="33" t="inlineStr"/>
       <c r="N514" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O514" s="33" t="inlineStr">
-        <is>
-          <t>A001441</t>
         </is>
       </c>
     </row>
@@ -24545,17 +23849,10 @@
         </is>
       </c>
       <c r="L519" s="6" t="n"/>
-      <c r="M519" s="33" t="n">
-        <v>308</v>
-      </c>
+      <c r="M519" s="33" t="inlineStr"/>
       <c r="N519" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O519" s="33" t="inlineStr">
-        <is>
-          <t>CGSIG-25-1030145</t>
         </is>
       </c>
     </row>
@@ -24598,17 +23895,10 @@
         </is>
       </c>
       <c r="L520" s="6" t="n"/>
-      <c r="M520" s="33" t="n">
-        <v>332</v>
-      </c>
+      <c r="M520" s="33" t="inlineStr"/>
       <c r="N520" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O520" s="33" t="inlineStr">
-        <is>
-          <t>43955</t>
         </is>
       </c>
     </row>
@@ -24651,17 +23941,10 @@
         </is>
       </c>
       <c r="L521" s="6" t="n"/>
-      <c r="M521" s="33" t="n">
-        <v>317</v>
-      </c>
+      <c r="M521" s="33" t="inlineStr"/>
       <c r="N521" s="33" t="inlineStr">
         <is>
           <t>ANNUGRAH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O521" s="33" t="inlineStr">
-        <is>
-          <t>L001048</t>
         </is>
       </c>
     </row>
@@ -24824,17 +24107,10 @@
         </is>
       </c>
       <c r="L525" s="6" t="n"/>
-      <c r="M525" s="33" t="n">
-        <v>325</v>
-      </c>
+      <c r="M525" s="33" t="inlineStr"/>
       <c r="N525" s="33" t="inlineStr">
         <is>
           <t>ARIHANT ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O525" s="33" t="inlineStr">
-        <is>
-          <t>2526CCB1206</t>
         </is>
       </c>
     </row>
@@ -25101,17 +24377,10 @@
         </is>
       </c>
       <c r="L531" s="6" t="n"/>
-      <c r="M531" s="33" t="n">
-        <v>333</v>
-      </c>
+      <c r="M531" s="33" t="inlineStr"/>
       <c r="N531" s="33" t="inlineStr">
         <is>
           <t>SHRI KULSWAMINI DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O531" s="33" t="inlineStr">
-        <is>
-          <t>2719 22/05 3061 30/05 5</t>
         </is>
       </c>
     </row>
@@ -25154,17 +24423,10 @@
         </is>
       </c>
       <c r="L532" s="6" t="n"/>
-      <c r="M532" s="33" t="n">
-        <v>330</v>
-      </c>
+      <c r="M532" s="33" t="inlineStr"/>
       <c r="N532" s="33" t="inlineStr">
         <is>
           <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O532" s="33" t="inlineStr">
-        <is>
-          <t>AB18261</t>
         </is>
       </c>
     </row>
@@ -25207,17 +24469,10 @@
         </is>
       </c>
       <c r="L533" s="6" t="n"/>
-      <c r="M533" s="33" t="n">
-        <v>318</v>
-      </c>
+      <c r="M533" s="33" t="inlineStr"/>
       <c r="N533" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O533" s="33" t="inlineStr">
-        <is>
-          <t>50891</t>
         </is>
       </c>
     </row>
@@ -25720,17 +24975,10 @@
         </is>
       </c>
       <c r="L545" s="6" t="n"/>
-      <c r="M545" s="33" t="n">
-        <v>319</v>
-      </c>
+      <c r="M545" s="33" t="inlineStr"/>
       <c r="N545" s="33" t="inlineStr">
         <is>
           <t>ATUL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O545" s="33" t="inlineStr">
-        <is>
-          <t>-417</t>
         </is>
       </c>
     </row>
@@ -25773,17 +25021,10 @@
         </is>
       </c>
       <c r="L546" s="6" t="n"/>
-      <c r="M546" s="33" t="n">
-        <v>319</v>
-      </c>
+      <c r="M546" s="33" t="inlineStr"/>
       <c r="N546" s="33" t="inlineStr">
         <is>
           <t>ATUL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O546" s="33" t="inlineStr">
-        <is>
-          <t>-417</t>
         </is>
       </c>
     </row>
@@ -26162,17 +25403,10 @@
         </is>
       </c>
       <c r="L555" s="6" t="n"/>
-      <c r="M555" s="33" t="n">
-        <v>321</v>
-      </c>
+      <c r="M555" s="33" t="inlineStr"/>
       <c r="N555" s="33" t="inlineStr">
         <is>
           <t>VED AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O555" s="33" t="inlineStr">
-        <is>
-          <t>CCN-005005</t>
         </is>
       </c>
     </row>
@@ -26495,17 +25729,10 @@
         </is>
       </c>
       <c r="L563" s="6" t="n"/>
-      <c r="M563" s="33" t="n">
-        <v>303</v>
-      </c>
+      <c r="M563" s="33" t="inlineStr"/>
       <c r="N563" s="33" t="inlineStr">
         <is>
           <t>SARA MARKETING</t>
-        </is>
-      </c>
-      <c r="O563" s="33" t="inlineStr">
-        <is>
-          <t>CREDIT/1145</t>
         </is>
       </c>
     </row>
@@ -26596,17 +25823,10 @@
         </is>
       </c>
       <c r="L565" s="6" t="n"/>
-      <c r="M565" s="33" t="n">
-        <v>331</v>
-      </c>
+      <c r="M565" s="33" t="inlineStr"/>
       <c r="N565" s="33" t="inlineStr">
         <is>
           <t>G K ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O565" s="33" t="inlineStr">
-        <is>
-          <t>002571</t>
         </is>
       </c>
     </row>
@@ -26737,17 +25957,14 @@
         </is>
       </c>
       <c r="L568" s="6" t="n"/>
-      <c r="M568" s="33" t="n">
-        <v>323</v>
+      <c r="M568" s="33" t="inlineStr">
+        <is>
+          <t>310,341,343,351,353,427,434,457,460,521,537,613,649,723,782,821,825</t>
+        </is>
       </c>
       <c r="N568" s="33" t="inlineStr">
         <is>
           <t>RUSHABH SURGICALS</t>
-        </is>
-      </c>
-      <c r="O568" s="33" t="inlineStr">
-        <is>
-          <t>RS/13847+RS/14227+RS/14796+RS/15053+RS/15545+RS/18334+RS/18820+RS/19778+RS/20425+RS/22086+RS/22791+RS/25542+RS/27373+RS/29397+RS/32340+RS/34211+RS/34550</t>
         </is>
       </c>
     </row>
@@ -26918,17 +26135,10 @@
         </is>
       </c>
       <c r="L572" s="6" t="n"/>
-      <c r="M572" s="33" t="n">
-        <v>334</v>
-      </c>
+      <c r="M572" s="33" t="inlineStr"/>
       <c r="N572" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O572" s="33" t="inlineStr">
-        <is>
-          <t>20716 ,1034757</t>
         </is>
       </c>
     </row>
@@ -27179,17 +26389,10 @@
         </is>
       </c>
       <c r="L578" s="6" t="n"/>
-      <c r="M578" s="33" t="n">
-        <v>335</v>
-      </c>
+      <c r="M578" s="33" t="inlineStr"/>
       <c r="N578" s="33" t="inlineStr">
         <is>
           <t>REKHA MARKETING</t>
-        </is>
-      </c>
-      <c r="O578" s="33" t="inlineStr">
-        <is>
-          <t>002576</t>
         </is>
       </c>
     </row>
@@ -27896,17 +27099,10 @@
         </is>
       </c>
       <c r="L595" s="6" t="n"/>
-      <c r="M595" s="33" t="n">
-        <v>339</v>
-      </c>
+      <c r="M595" s="33" t="inlineStr"/>
       <c r="N595" s="33" t="inlineStr">
         <is>
           <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O595" s="33" t="inlineStr">
-        <is>
-          <t>51738</t>
         </is>
       </c>
     </row>
@@ -28117,17 +27313,14 @@
         </is>
       </c>
       <c r="L600" s="6" t="n"/>
-      <c r="M600" s="33" t="n">
-        <v>329</v>
+      <c r="M600" s="33" t="inlineStr">
+        <is>
+          <t>463,468,470,486,526,552,614,584,595,608,628,677,685,701,713,721,738,756,755,757,768,784,795,811,822,852,873,886,908,926,935</t>
+        </is>
       </c>
       <c r="N600" s="33" t="inlineStr">
         <is>
           <t>MAHENDRA DISRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O600" s="33" t="inlineStr">
-        <is>
-          <t>S/9218+S/9347+S/9559+S/9782+S/10387+S/10895+S/10976+S/11474+S/11662+S/12045+S/12564+S/13312+S/13497+S/13876+S/14067+S/14263+S/14619+S/14870+S/15044+S/15253+S/15467+S/15621+S/15791+S/16088+S/16259+S/17</t>
         </is>
       </c>
     </row>
@@ -28170,17 +27363,14 @@
         </is>
       </c>
       <c r="L601" s="6" t="n"/>
-      <c r="M601" s="33" t="n">
-        <v>326</v>
+      <c r="M601" s="33" t="inlineStr">
+        <is>
+          <t>2099,854,1444,1445,2406</t>
+        </is>
       </c>
       <c r="N601" s="33" t="inlineStr">
         <is>
           <t>TRIDENT MEDLIFE PVT LTD</t>
-        </is>
-      </c>
-      <c r="O601" s="33" t="inlineStr">
-        <is>
-          <t>CC-3226+CC-716+CC-1154+CC-1153+CC-1937</t>
         </is>
       </c>
     </row>
@@ -28223,17 +27413,10 @@
         </is>
       </c>
       <c r="L602" s="6" t="n"/>
-      <c r="M602" s="33" t="n">
-        <v>340</v>
-      </c>
+      <c r="M602" s="33" t="inlineStr"/>
       <c r="N602" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O602" s="33" t="inlineStr">
-        <is>
-          <t>37896</t>
         </is>
       </c>
     </row>
@@ -28276,17 +27459,10 @@
         </is>
       </c>
       <c r="L603" s="6" t="n"/>
-      <c r="M603" s="33" t="n">
-        <v>345</v>
-      </c>
+      <c r="M603" s="33" t="inlineStr"/>
       <c r="N603" s="33" t="inlineStr">
         <is>
           <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O603" s="33" t="inlineStr">
-        <is>
-          <t>A045504073</t>
         </is>
       </c>
     </row>
@@ -28329,17 +27505,10 @@
         </is>
       </c>
       <c r="L604" s="6" t="n"/>
-      <c r="M604" s="33" t="n">
-        <v>345</v>
-      </c>
+      <c r="M604" s="33" t="inlineStr"/>
       <c r="N604" s="33" t="inlineStr">
         <is>
           <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O604" s="33" t="inlineStr">
-        <is>
-          <t>A045504073</t>
         </is>
       </c>
     </row>
@@ -28382,17 +27551,10 @@
         </is>
       </c>
       <c r="L605" s="6" t="n"/>
-      <c r="M605" s="33" t="n">
-        <v>313</v>
-      </c>
+      <c r="M605" s="33" t="inlineStr"/>
       <c r="N605" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O605" s="33" t="inlineStr">
-        <is>
-          <t>A001441</t>
         </is>
       </c>
     </row>
@@ -28515,17 +27677,10 @@
         </is>
       </c>
       <c r="L608" s="6" t="n"/>
-      <c r="M608" s="33" t="n">
-        <v>345</v>
-      </c>
+      <c r="M608" s="33" t="inlineStr"/>
       <c r="N608" s="33" t="inlineStr">
         <is>
           <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O608" s="33" t="inlineStr">
-        <is>
-          <t>A045504073</t>
         </is>
       </c>
     </row>
@@ -28776,17 +27931,10 @@
         </is>
       </c>
       <c r="L614" s="6" t="n"/>
-      <c r="M614" s="33" t="n">
-        <v>341</v>
-      </c>
+      <c r="M614" s="33" t="inlineStr"/>
       <c r="N614" s="33" t="inlineStr">
         <is>
           <t>ANNUGRAH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O614" s="33" t="inlineStr">
-        <is>
-          <t>L001244</t>
         </is>
       </c>
     </row>
@@ -28829,17 +27977,10 @@
         </is>
       </c>
       <c r="L615" s="6" t="n"/>
-      <c r="M615" s="33" t="n">
-        <v>338</v>
-      </c>
+      <c r="M615" s="33" t="inlineStr"/>
       <c r="N615" s="33" t="inlineStr">
         <is>
           <t>CHINTAMANI DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O615" s="33" t="inlineStr">
-        <is>
-          <t>Z-3011</t>
         </is>
       </c>
     </row>
@@ -29266,15 +28407,12 @@
         </is>
       </c>
       <c r="L625" s="6" t="n"/>
-      <c r="M625" s="33" t="n">
-        <v>348</v>
-      </c>
+      <c r="M625" s="33" t="inlineStr"/>
       <c r="N625" s="33" t="inlineStr">
         <is>
           <t>MAULI AGENCIES</t>
         </is>
       </c>
-      <c r="O625" s="33" t="inlineStr"/>
     </row>
     <row r="626">
       <c r="A626" s="21" t="n">
@@ -30663,17 +29801,10 @@
         </is>
       </c>
       <c r="L658" s="6" t="n"/>
-      <c r="M658" s="33" t="n">
-        <v>346</v>
-      </c>
+      <c r="M658" s="33" t="inlineStr"/>
       <c r="N658" s="33" t="inlineStr">
         <is>
           <t>SONIGARA DISTRIBUTOR</t>
-        </is>
-      </c>
-      <c r="O658" s="33" t="inlineStr">
-        <is>
-          <t>SD-4175/25-26</t>
         </is>
       </c>
     </row>
@@ -31452,17 +30583,10 @@
         </is>
       </c>
       <c r="L677" s="6" t="n"/>
-      <c r="M677" s="33" t="n">
-        <v>313</v>
-      </c>
+      <c r="M677" s="33" t="inlineStr"/>
       <c r="N677" s="33" t="inlineStr">
         <is>
           <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O677" s="33" t="inlineStr">
-        <is>
-          <t>A001441</t>
         </is>
       </c>
     </row>
@@ -31505,17 +30629,10 @@
         </is>
       </c>
       <c r="L678" s="6" t="n"/>
-      <c r="M678" s="33" t="n">
-        <v>319</v>
-      </c>
+      <c r="M678" s="33" t="inlineStr"/>
       <c r="N678" s="33" t="inlineStr">
         <is>
           <t>ATUL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O678" s="33" t="inlineStr">
-        <is>
-          <t>-417</t>
         </is>
       </c>
     </row>
@@ -31894,15 +31011,12 @@
         </is>
       </c>
       <c r="L687" s="6" t="n"/>
-      <c r="M687" s="33" t="n">
-        <v>360</v>
-      </c>
+      <c r="M687" s="33" t="inlineStr"/>
       <c r="N687" s="33" t="inlineStr">
         <is>
           <t>G K ENTERPRISES</t>
         </is>
       </c>
-      <c r="O687" s="33" t="inlineStr"/>
     </row>
     <row r="688">
       <c r="A688" s="21" t="n">
@@ -32243,17 +31357,10 @@
         </is>
       </c>
       <c r="L695" s="6" t="n"/>
-      <c r="M695" s="33" t="n">
-        <v>347</v>
-      </c>
+      <c r="M695" s="33" t="inlineStr"/>
       <c r="N695" s="33" t="inlineStr">
         <is>
           <t>THE PLUS ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O695" s="33" t="inlineStr">
-        <is>
-          <t>6854</t>
         </is>
       </c>
     </row>
@@ -32296,15 +31403,12 @@
         </is>
       </c>
       <c r="L696" s="6" t="n"/>
-      <c r="M696" s="33" t="n">
-        <v>354</v>
-      </c>
+      <c r="M696" s="33" t="inlineStr"/>
       <c r="N696" s="33" t="inlineStr">
         <is>
           <t>AARADHYA AGENCIES</t>
         </is>
       </c>
-      <c r="O696" s="33" t="inlineStr"/>
     </row>
     <row r="697">
       <c r="A697" s="21" t="n">
@@ -32345,17 +31449,10 @@
         </is>
       </c>
       <c r="L697" s="6" t="n"/>
-      <c r="M697" s="33" t="n">
-        <v>353</v>
-      </c>
+      <c r="M697" s="33" t="inlineStr"/>
       <c r="N697" s="33" t="inlineStr">
         <is>
           <t>SHINDE ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O697" s="33" t="inlineStr">
-        <is>
-          <t>MLB161752513308</t>
         </is>
       </c>
     </row>
@@ -32398,17 +31495,14 @@
         </is>
       </c>
       <c r="L698" s="6" t="n"/>
-      <c r="M698" s="33" t="n">
-        <v>343</v>
+      <c r="M698" s="33" t="inlineStr">
+        <is>
+          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
+        </is>
       </c>
       <c r="N698" s="33" t="inlineStr">
         <is>
           <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O698" s="33" t="inlineStr">
-        <is>
-          <t>MD/7068+MD/7263+MD/7438+MD/7437+MD/7557+MD/7480+MD/7824+MD/8188+MD/8361+MD/8816+MD/9469+MD/10527+MD/11303+MD/11595+MD/12420+MD/12713+MD/12926</t>
         </is>
       </c>
     </row>
@@ -32451,17 +31545,14 @@
         </is>
       </c>
       <c r="L699" s="6" t="n"/>
-      <c r="M699" s="33" t="n">
-        <v>343</v>
+      <c r="M699" s="33" t="inlineStr">
+        <is>
+          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
+        </is>
       </c>
       <c r="N699" s="33" t="inlineStr">
         <is>
           <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O699" s="33" t="inlineStr">
-        <is>
-          <t>MD/7068+MD/7263+MD/7438+MD/7437+MD/7557+MD/7480+MD/7824+MD/8188+MD/8361+MD/8816+MD/9469+MD/10527+MD/11303+MD/11595+MD/12420+MD/12713+MD/12926</t>
         </is>
       </c>
     </row>
@@ -32808,17 +31899,10 @@
         </is>
       </c>
       <c r="L707" s="6" t="n"/>
-      <c r="M707" s="33" t="n">
-        <v>358</v>
-      </c>
+      <c r="M707" s="33" t="inlineStr"/>
       <c r="N707" s="33" t="inlineStr">
         <is>
           <t>AV TRADERS</t>
-        </is>
-      </c>
-      <c r="O707" s="33" t="inlineStr">
-        <is>
-          <t>AV/25-26/8671</t>
         </is>
       </c>
     </row>
@@ -32861,17 +31945,10 @@
         </is>
       </c>
       <c r="L708" s="6" t="n"/>
-      <c r="M708" s="33" t="n">
-        <v>356</v>
-      </c>
+      <c r="M708" s="33" t="inlineStr"/>
       <c r="N708" s="33" t="inlineStr">
         <is>
           <t>CG MARKETING PVT LTD</t>
-        </is>
-      </c>
-      <c r="O708" s="33" t="inlineStr">
-        <is>
-          <t>CGSIG-25-I043141</t>
         </is>
       </c>
     </row>
@@ -33226,17 +32303,10 @@
         </is>
       </c>
       <c r="L716" s="6" t="n"/>
-      <c r="M716" s="33" t="n">
-        <v>363</v>
-      </c>
+      <c r="M716" s="33" t="inlineStr"/>
       <c r="N716" s="33" t="inlineStr">
         <is>
           <t>SHREE SIDDHESHWAR ENTERISES</t>
-        </is>
-      </c>
-      <c r="O716" s="33" t="inlineStr">
-        <is>
-          <t>.SE3639/25-26</t>
         </is>
       </c>
     </row>
@@ -33279,15 +32349,12 @@
         </is>
       </c>
       <c r="L717" s="6" t="n"/>
-      <c r="M717" s="33" t="n">
-        <v>361</v>
-      </c>
+      <c r="M717" s="33" t="inlineStr"/>
       <c r="N717" s="33" t="inlineStr">
         <is>
           <t>SAI KRUPA AGENCY</t>
         </is>
       </c>
-      <c r="O717" s="33" t="inlineStr"/>
     </row>
     <row r="718">
       <c r="A718" s="21" t="n">
@@ -33328,17 +32395,14 @@
         </is>
       </c>
       <c r="L718" s="6" t="n"/>
-      <c r="M718" s="33" t="n">
-        <v>350</v>
+      <c r="M718" s="33" t="inlineStr">
+        <is>
+          <t>426,438,445,447,465,473,476,482,495,544,540,535,536,547,550,568,571,582,591,604,621,622,626,635,639,641,646,659,660,674,688</t>
+        </is>
       </c>
       <c r="N718" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O718" s="33" t="inlineStr">
-        <is>
-          <t>2526CRB60057+2526CRB61602+2526CRB62662+2526CRB62619+2526CRB 65536+256CRB65284+2526CRB65210+2526CRB66570+2526CRB67769+2526CRB71838*+2526CRB 72845+2526CRB 74129+2526CRB 74246+2526CRB 75305+2526CRB 75255</t>
         </is>
       </c>
     </row>
@@ -33509,15 +32573,12 @@
         </is>
       </c>
       <c r="L722" s="6" t="n"/>
-      <c r="M722" s="33" t="n">
-        <v>359</v>
-      </c>
+      <c r="M722" s="33" t="inlineStr"/>
       <c r="N722" s="33" t="inlineStr">
         <is>
           <t>VISION SALES</t>
         </is>
       </c>
-      <c r="O722" s="33" t="inlineStr"/>
     </row>
     <row r="723">
       <c r="A723" s="21" t="n">
@@ -35498,17 +34559,14 @@
         </is>
       </c>
       <c r="L769" s="6" t="n"/>
-      <c r="M769" s="33" t="n">
-        <v>351</v>
+      <c r="M769" s="33" t="inlineStr">
+        <is>
+          <t>703,712,720,730,737,743,754,761,762,773,788,798,810,820,830,839,854,855,877,885,864,911,923,924,936,943</t>
+        </is>
       </c>
       <c r="N769" s="33" t="inlineStr">
         <is>
           <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O769" s="33" t="inlineStr">
-        <is>
-          <t>2526CRB94806+2526CRB96137+2526CRB97366+2526CRB98461+2526CRB99664+2526CRB101219+2526CRB102536+2526CRB103746+2526CRB103733+2526CRB104995*+2526CRB106107*+2526CRB107117+2526CRB108889+2526CRB110067*+2526CR</t>
         </is>
       </c>
     </row>
@@ -35639,17 +34697,14 @@
         </is>
       </c>
       <c r="L772" s="6" t="n"/>
-      <c r="M772" s="33" t="n">
-        <v>343</v>
+      <c r="M772" s="33" t="inlineStr">
+        <is>
+          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
+        </is>
       </c>
       <c r="N772" s="33" t="inlineStr">
         <is>
           <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O772" s="33" t="inlineStr">
-        <is>
-          <t>MD/7068+MD/7263+MD/7438+MD/7437+MD/7557+MD/7480+MD/7824+MD/8188+MD/8361+MD/8816+MD/9469+MD/10527+MD/11303+MD/11595+MD/12420+MD/12713+MD/12926</t>
         </is>
       </c>
     </row>
@@ -36108,17 +35163,10 @@
         </is>
       </c>
       <c r="L783" s="6" t="n"/>
-      <c r="M783" s="33" t="n">
-        <v>364</v>
-      </c>
+      <c r="M783" s="33" t="inlineStr"/>
       <c r="N783" s="33" t="inlineStr">
         <is>
           <t>HEALTH PLUS MEDICO</t>
-        </is>
-      </c>
-      <c r="O783" s="33" t="inlineStr">
-        <is>
-          <t>CR/5173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete reconciliation: Pending column, GPAY/NEFT matching, NOT_IN_SYSTEM flag
System_Purchase:
- Pending = full Amount for 516 unpaid bills (no PAIDTRAN entry)
- Pending = PURBALAMT for 2 partially paid bills
- Cash column filled for CASH type payments

Bank Statement:
- GPAY/NEFT: 64 additional rows matched by exact withdrawal amount
- NOT_IN_SYSTEM flag on 109 CHQ rows (pre-takeover, not in new software)
- Match_Status column: CHQ_MATCHED / GPAY_AMT_MATCHED / NOT_IN_SYSTEM

Old Account = PURPAIDAMT of specific matched PAIDTRAN row (per Vou.No.)
Previous Pending = sum PURPAIDAMT for bills before 29-May-2025 takeover

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -68,7 +68,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -103,6 +103,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2CFEF"/>
+        <bgColor rgb="00E2CFEF"/>
       </patternFill>
     </fill>
   </fills>
@@ -274,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -337,6 +349,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -715,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N891"/>
+  <dimension ref="A1:O891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
@@ -803,6 +817,11 @@
           <t>Party_Name</t>
         </is>
       </c>
+      <c r="O1" s="32" t="inlineStr">
+        <is>
+          <t>Match_Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="21" t="n">
@@ -897,6 +916,11 @@
           <t>SHREYAA AGENCIES</t>
         </is>
       </c>
+      <c r="O3" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="n">
@@ -949,6 +973,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O4" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="n">
@@ -991,6 +1020,11 @@
         </is>
       </c>
       <c r="L5" s="6" t="n"/>
+      <c r="O5" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="n">
@@ -1039,6 +1073,11 @@
           <t>REKHA MARKETING</t>
         </is>
       </c>
+      <c r="O6" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="1" s="31">
       <c r="A7" s="29" t="n">
@@ -1087,6 +1126,11 @@
           <t>AGARWAL &amp; COMPANY</t>
         </is>
       </c>
+      <c r="O7" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="1" s="31">
       <c r="A8" s="29" t="n">
@@ -1135,6 +1179,11 @@
           <t>AGARWAL &amp; COMPANY</t>
         </is>
       </c>
+      <c r="O8" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="n">
@@ -1225,6 +1274,11 @@
           <t>AGARWAL &amp; COMPANY</t>
         </is>
       </c>
+      <c r="O10" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="n">
@@ -1369,6 +1423,11 @@
           <t>NANDINI BEAUTY</t>
         </is>
       </c>
+      <c r="O13" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="1" s="31">
       <c r="A14" s="29" t="n">
@@ -1421,6 +1480,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O14" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="15" customFormat="1" s="31">
       <c r="A15" s="29" t="n">
@@ -1473,6 +1537,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O15" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="n">
@@ -1609,6 +1678,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O18" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="21" t="n">
@@ -1841,6 +1915,11 @@
           <t>VENKATESHA ENTERPRISES</t>
         </is>
       </c>
+      <c r="O23" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="21" t="n">
@@ -1885,6 +1964,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O24" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="25" customFormat="1" s="31">
       <c r="A25" s="29" t="n">
@@ -2017,6 +2101,11 @@
           <t>SHINDE ENTERPRISES</t>
         </is>
       </c>
+      <c r="O27" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="28" customFormat="1" s="31">
       <c r="A28" s="29" t="n">
@@ -2069,6 +2158,11 @@
           <t>NANDINI BEAUTY</t>
         </is>
       </c>
+      <c r="O28" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="n">
@@ -2121,6 +2215,11 @@
           <t>RAJLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O29" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="n">
@@ -2163,6 +2262,21 @@
         </is>
       </c>
       <c r="L30" s="6" t="n"/>
+      <c r="M30" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N30" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O30" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="n">
@@ -2557,6 +2671,21 @@
         </is>
       </c>
       <c r="L39" s="6" t="n"/>
+      <c r="M39" s="35" t="inlineStr">
+        <is>
+          <t>327,344</t>
+        </is>
+      </c>
+      <c r="N39" s="35" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O39" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
@@ -2599,6 +2728,21 @@
         </is>
       </c>
       <c r="L40" s="6" t="n"/>
+      <c r="M40" s="35" t="inlineStr">
+        <is>
+          <t>293,298,307,319</t>
+        </is>
+      </c>
+      <c r="N40" s="35" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O40" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
@@ -2789,6 +2933,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O44" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
@@ -2841,6 +2990,11 @@
           <t>MAHENDRA DISRIBUTORS</t>
         </is>
       </c>
+      <c r="O45" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="n">
@@ -2967,6 +3121,21 @@
         </is>
       </c>
       <c r="L48" s="6" t="n"/>
+      <c r="M48" s="35" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="N48" s="35" t="inlineStr">
+        <is>
+          <t>HDFC BANK</t>
+        </is>
+      </c>
+      <c r="O48" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="n">
@@ -3009,6 +3178,21 @@
         </is>
       </c>
       <c r="L49" s="6" t="n"/>
+      <c r="M49" s="35" t="inlineStr">
+        <is>
+          <t>334,347,357,379,390,391,402,414,428,435,446</t>
+        </is>
+      </c>
+      <c r="N49" s="35" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O49" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="n">
@@ -3107,6 +3291,11 @@
           <t>GAURAV ENTERPRISES</t>
         </is>
       </c>
+      <c r="O51" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="21" t="n">
@@ -3233,6 +3422,21 @@
         </is>
       </c>
       <c r="L54" s="6" t="n"/>
+      <c r="M54" s="35" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="N54" s="35" t="inlineStr">
+        <is>
+          <t>HDFC BANK</t>
+        </is>
+      </c>
+      <c r="O54" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="n">
@@ -3275,6 +3479,21 @@
         </is>
       </c>
       <c r="L55" s="6" t="n"/>
+      <c r="M55" s="35" t="inlineStr">
+        <is>
+          <t>475</t>
+        </is>
+      </c>
+      <c r="N55" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O55" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="n">
@@ -3423,6 +3642,11 @@
           <t>RAUT TRADINGS</t>
         </is>
       </c>
+      <c r="O58" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="21" t="n">
@@ -3471,6 +3695,11 @@
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
+      <c r="O59" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="21" t="n">
@@ -3519,6 +3748,11 @@
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
+      <c r="O60" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="21" t="n">
@@ -3571,6 +3805,11 @@
           <t>YASH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O61" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="21" t="n">
@@ -3623,6 +3862,11 @@
           <t>JEEVIKA HOSPITALITY SERVICES</t>
         </is>
       </c>
+      <c r="O62" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="n">
@@ -3707,6 +3951,21 @@
         </is>
       </c>
       <c r="L64" s="6" t="n"/>
+      <c r="M64" s="35" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="N64" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O64" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="n">
@@ -3805,6 +4064,11 @@
           <t>APARNA LOGITECH PRIVATE LIMITE</t>
         </is>
       </c>
+      <c r="O66" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="21" t="n">
@@ -3857,6 +4121,11 @@
           <t>JAI SHREE GANESH AGENCIES</t>
         </is>
       </c>
+      <c r="O67" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="21" t="n">
@@ -3905,6 +4174,11 @@
           <t>ASHA MOHAN ENTERPRISES</t>
         </is>
       </c>
+      <c r="O68" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="21" t="n">
@@ -3989,6 +4263,21 @@
         </is>
       </c>
       <c r="L70" s="6" t="n"/>
+      <c r="M70" s="35" t="inlineStr">
+        <is>
+          <t>42,180,235,189,253,259</t>
+        </is>
+      </c>
+      <c r="N70" s="35" t="inlineStr">
+        <is>
+          <t>YASHVI AGENCIES</t>
+        </is>
+      </c>
+      <c r="O70" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="21" t="n">
@@ -4213,6 +4502,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O75" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="21" t="n">
@@ -4265,6 +4559,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O76" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="21" t="n">
@@ -4307,6 +4606,11 @@
         </is>
       </c>
       <c r="L77" s="6" t="n"/>
+      <c r="O77" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="21" t="n">
@@ -4401,6 +4705,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O79" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="21" t="n">
@@ -4845,6 +5154,21 @@
         </is>
       </c>
       <c r="L89" s="6" t="n"/>
+      <c r="M89" s="35" t="inlineStr">
+        <is>
+          <t>508</t>
+        </is>
+      </c>
+      <c r="N89" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O89" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="n">
@@ -4993,6 +5317,11 @@
           <t>ANURAG CORPORATION PVT.LTD</t>
         </is>
       </c>
+      <c r="O92" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="n">
@@ -5041,6 +5370,11 @@
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
+      <c r="O93" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="21" t="n">
@@ -5083,6 +5417,11 @@
         </is>
       </c>
       <c r="L94" s="6" t="n"/>
+      <c r="O94" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="21" t="n">
@@ -5131,6 +5470,11 @@
           <t>DP SOLUTIONS</t>
         </is>
       </c>
+      <c r="O95" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="21" t="n">
@@ -5359,6 +5703,11 @@
           <t>KAYDEE SONS LLP</t>
         </is>
       </c>
+      <c r="O100" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="21" t="n">
@@ -5401,6 +5750,21 @@
         </is>
       </c>
       <c r="L101" s="6" t="n"/>
+      <c r="M101" s="35" t="inlineStr">
+        <is>
+          <t>488</t>
+        </is>
+      </c>
+      <c r="N101" s="35" t="inlineStr">
+        <is>
+          <t>DHANVANTARI SALES</t>
+        </is>
+      </c>
+      <c r="O101" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="21" t="n">
@@ -5443,6 +5807,21 @@
         </is>
       </c>
       <c r="L102" s="6" t="n"/>
+      <c r="M102" s="35" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="N102" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O102" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="21" t="n">
@@ -5711,6 +6090,21 @@
         </is>
       </c>
       <c r="L108" s="6" t="n"/>
+      <c r="M108" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N108" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O108" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="21" t="n">
@@ -5753,6 +6147,21 @@
         </is>
       </c>
       <c r="L109" s="6" t="n"/>
+      <c r="M109" s="35" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="N109" s="35" t="inlineStr">
+        <is>
+          <t>HDFC BANK</t>
+        </is>
+      </c>
+      <c r="O109" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="21" t="n">
@@ -5897,6 +6306,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O112" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="21" t="n">
@@ -5945,6 +6359,11 @@
           <t>JAI SHREE GANESH AGENCIES</t>
         </is>
       </c>
+      <c r="O113" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="21" t="n">
@@ -5993,6 +6412,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O114" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="21" t="n">
@@ -6041,6 +6465,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O115" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="21" t="n">
@@ -6167,6 +6596,21 @@
         </is>
       </c>
       <c r="L118" s="6" t="n"/>
+      <c r="M118" s="35" t="inlineStr">
+        <is>
+          <t>567,549</t>
+        </is>
+      </c>
+      <c r="N118" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O118" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="21" t="n">
@@ -6251,6 +6695,21 @@
         </is>
       </c>
       <c r="L120" s="6" t="n"/>
+      <c r="M120" s="35" t="inlineStr">
+        <is>
+          <t>484,464,469,487,506,522</t>
+        </is>
+      </c>
+      <c r="N120" s="35" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O120" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="21" t="n">
@@ -6339,6 +6798,21 @@
         </is>
       </c>
       <c r="L122" s="6" t="n"/>
+      <c r="M122" s="35" t="inlineStr">
+        <is>
+          <t>689</t>
+        </is>
+      </c>
+      <c r="N122" s="35" t="inlineStr">
+        <is>
+          <t>SUPARSHWA MEDCARE LLP</t>
+        </is>
+      </c>
+      <c r="O122" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="21" t="n">
@@ -6479,6 +6953,11 @@
           <t>N R ENTERPRISES</t>
         </is>
       </c>
+      <c r="O125" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="21" t="n">
@@ -6521,6 +7000,21 @@
         </is>
       </c>
       <c r="L126" s="6" t="n"/>
+      <c r="M126" s="35" t="inlineStr">
+        <is>
+          <t>523</t>
+        </is>
+      </c>
+      <c r="N126" s="35" t="inlineStr">
+        <is>
+          <t>ABHAY PHARMA</t>
+        </is>
+      </c>
+      <c r="O126" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="21" t="n">
@@ -6563,6 +7057,21 @@
         </is>
       </c>
       <c r="L127" s="6" t="n"/>
+      <c r="M127" s="35" t="inlineStr">
+        <is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="N127" s="35" t="inlineStr">
+        <is>
+          <t>PRIME AYURVED</t>
+        </is>
+      </c>
+      <c r="O127" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="21" t="n">
@@ -6605,6 +7114,21 @@
         </is>
       </c>
       <c r="L128" s="6" t="n"/>
+      <c r="M128" s="35" t="inlineStr">
+        <is>
+          <t>42,180,235,189,253,259</t>
+        </is>
+      </c>
+      <c r="N128" s="35" t="inlineStr">
+        <is>
+          <t>YASHVI AGENCIES</t>
+        </is>
+      </c>
+      <c r="O128" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="21" t="n">
@@ -6823,6 +7347,21 @@
         </is>
       </c>
       <c r="L133" s="6" t="n"/>
+      <c r="M133" s="35" t="inlineStr">
+        <is>
+          <t>578,577</t>
+        </is>
+      </c>
+      <c r="N133" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O133" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="21" t="n">
@@ -6961,6 +7500,21 @@
           <t>salary</t>
         </is>
       </c>
+      <c r="M136" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N136" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O136" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="21" t="n">
@@ -7063,6 +7617,11 @@
           <t>CHINTAMANI DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O138" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="21" t="n">
@@ -7111,6 +7670,11 @@
           <t>AARADHYA AGENCIES</t>
         </is>
       </c>
+      <c r="O139" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="21" t="n">
@@ -7293,6 +7857,11 @@
           <t>ANURAG CORPORATION PVT.LTD</t>
         </is>
       </c>
+      <c r="O143" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="21" t="n">
@@ -7341,6 +7910,11 @@
           <t>MOHAN CHEMIST</t>
         </is>
       </c>
+      <c r="O144" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="21" t="n">
@@ -7443,6 +8017,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O146" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="21" t="n">
@@ -7527,6 +8106,21 @@
         </is>
       </c>
       <c r="L148" s="6" t="n"/>
+      <c r="M148" s="35" t="inlineStr">
+        <is>
+          <t>597</t>
+        </is>
+      </c>
+      <c r="N148" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O148" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="21" t="n">
@@ -7717,6 +8311,11 @@
           <t>SUYASH MEDICALS</t>
         </is>
       </c>
+      <c r="O152" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="21" t="n">
@@ -7765,6 +8364,11 @@
           <t>THE PLUS ENTERPRISES</t>
         </is>
       </c>
+      <c r="O153" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="21" t="n">
@@ -7813,6 +8417,11 @@
           <t>SHREE SAI MEDICAL DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O154" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="21" t="n">
@@ -7865,6 +8474,11 @@
           <t>SHREE DATTA KRUPA AGENCY</t>
         </is>
       </c>
+      <c r="O155" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="21" t="n">
@@ -7917,6 +8531,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O156" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="21" t="n">
@@ -7959,6 +8578,21 @@
         </is>
       </c>
       <c r="L157" s="6" t="n"/>
+      <c r="M157" s="35" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="N157" s="35" t="inlineStr">
+        <is>
+          <t>HDFC BANK</t>
+        </is>
+      </c>
+      <c r="O157" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="21" t="n">
@@ -8137,6 +8771,11 @@
           <t>ROYAL ENTERPRISES</t>
         </is>
       </c>
+      <c r="O161" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="21" t="n">
@@ -8327,6 +8966,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O165" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="21" t="n">
@@ -8495,6 +9139,21 @@
         </is>
       </c>
       <c r="L169" s="6" t="n"/>
+      <c r="M169" s="35" t="inlineStr">
+        <is>
+          <t>583,596,607</t>
+        </is>
+      </c>
+      <c r="N169" s="35" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O169" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="21" t="n">
@@ -8593,6 +9252,11 @@
           <t>ADK ENTERPRISES</t>
         </is>
       </c>
+      <c r="O171" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="21" t="n">
@@ -8645,6 +9309,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O172" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="21" t="n">
@@ -8697,6 +9366,11 @@
           <t>YASHVI AGENCIES</t>
         </is>
       </c>
+      <c r="O173" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="21" t="n">
@@ -8745,6 +9419,11 @@
           <t>RAJLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O174" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="21" t="n">
@@ -8793,6 +9472,11 @@
           <t>KHAMANG BEST CHIWDA</t>
         </is>
       </c>
+      <c r="O175" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="21" t="n">
@@ -9019,6 +9703,11 @@
         </is>
       </c>
       <c r="L180" s="6" t="n"/>
+      <c r="O180" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="21" t="n">
@@ -9067,6 +9756,11 @@
           <t>DHYAANI NEXUS PVT.LTD.</t>
         </is>
       </c>
+      <c r="O181" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="21" t="n">
@@ -9243,6 +9937,21 @@
         </is>
       </c>
       <c r="L185" s="6" t="n"/>
+      <c r="M185" s="35" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="N185" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O185" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="21" t="n">
@@ -9907,6 +10616,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O200" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="21" t="n">
@@ -10033,6 +10747,21 @@
         </is>
       </c>
       <c r="L203" s="6" t="n"/>
+      <c r="M203" s="35" t="inlineStr">
+        <is>
+          <t>629,630</t>
+        </is>
+      </c>
+      <c r="N203" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O203" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="21" t="n">
@@ -10125,6 +10854,11 @@
         </is>
       </c>
       <c r="L205" s="6" t="n"/>
+      <c r="O205" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="21" t="n">
@@ -10167,6 +10901,11 @@
         </is>
       </c>
       <c r="L206" s="6" t="n"/>
+      <c r="O206" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="21" t="n">
@@ -10209,6 +10948,21 @@
         </is>
       </c>
       <c r="L207" s="6" t="n"/>
+      <c r="M207" s="35" t="inlineStr">
+        <is>
+          <t>638</t>
+        </is>
+      </c>
+      <c r="N207" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O207" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="21" t="n">
@@ -10335,6 +11089,21 @@
         </is>
       </c>
       <c r="L210" s="6" t="n"/>
+      <c r="M210" s="35" t="inlineStr">
+        <is>
+          <t>472,467,481,505,525,532,546,548,586,592,606</t>
+        </is>
+      </c>
+      <c r="N210" s="35" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O210" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="21" t="n">
@@ -10603,6 +11372,21 @@
         </is>
       </c>
       <c r="L216" s="6" t="n"/>
+      <c r="M216" s="35" t="inlineStr">
+        <is>
+          <t>651</t>
+        </is>
+      </c>
+      <c r="N216" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O216" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="21" t="n">
@@ -10729,6 +11513,21 @@
         </is>
       </c>
       <c r="L219" s="6" t="n"/>
+      <c r="M219" s="35" t="inlineStr">
+        <is>
+          <t>216,221,234,244,265,292,301,305,308,324,333,349,363,362,372,389,393,400,418,429,437</t>
+        </is>
+      </c>
+      <c r="N219" s="35" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O219" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="21" t="n">
@@ -10827,6 +11626,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O221" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="21" t="n">
@@ -10875,6 +11679,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O222" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="21" t="n">
@@ -10923,6 +11732,11 @@
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
+      <c r="O223" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="21" t="n">
@@ -10971,6 +11785,11 @@
           <t>YASH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O224" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="21" t="n">
@@ -11139,6 +11958,21 @@
         </is>
       </c>
       <c r="L228" s="6" t="n"/>
+      <c r="M228" s="35" t="inlineStr">
+        <is>
+          <t>471,474,479,485,507,524,533,553,570</t>
+        </is>
+      </c>
+      <c r="N228" s="35" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O228" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="21" t="n">
@@ -11237,6 +12071,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O230" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="21" t="n">
@@ -11375,6 +12214,21 @@
         </is>
       </c>
       <c r="L233" s="6" t="n"/>
+      <c r="M233" s="35" t="inlineStr">
+        <is>
+          <t>670,673</t>
+        </is>
+      </c>
+      <c r="N233" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O233" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="21" t="n">
@@ -11465,6 +12319,11 @@
           <t>RADIANT ENTERPRISES</t>
         </is>
       </c>
+      <c r="O235" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="21" t="n">
@@ -11599,6 +12458,21 @@
         </is>
       </c>
       <c r="L238" s="6" t="n"/>
+      <c r="M238" s="35" t="inlineStr">
+        <is>
+          <t>126,127,133,151,179,189,209,240,246,258,303,337,411,355,364,376,415,425</t>
+        </is>
+      </c>
+      <c r="N238" s="35" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O238" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="21" t="n">
@@ -11641,6 +12515,21 @@
         </is>
       </c>
       <c r="L239" s="6" t="n"/>
+      <c r="M239" s="35" t="inlineStr">
+        <is>
+          <t>504,538,551,566,609,633,644</t>
+        </is>
+      </c>
+      <c r="N239" s="35" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O239" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="21" t="n">
@@ -11867,6 +12756,11 @@
         </is>
       </c>
       <c r="L244" s="6" t="n"/>
+      <c r="O244" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="21" t="n">
@@ -12089,6 +12983,17 @@
         </is>
       </c>
       <c r="L249" s="6" t="n"/>
+      <c r="M249" s="35" t="inlineStr"/>
+      <c r="N249" s="35" t="inlineStr">
+        <is>
+          <t>MSEDCL  -----------X----------</t>
+        </is>
+      </c>
+      <c r="O249" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="21" t="n">
@@ -12131,6 +13036,21 @@
         </is>
       </c>
       <c r="L250" s="6" t="n"/>
+      <c r="M250" s="35" t="inlineStr">
+        <is>
+          <t>671,692,657,672,691,690</t>
+        </is>
+      </c>
+      <c r="N250" s="35" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O250" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="21" t="n">
@@ -12311,6 +13231,11 @@
           <t>SAMARTH AYURVEDIC</t>
         </is>
       </c>
+      <c r="O254" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="21" t="n">
@@ -12361,6 +13286,11 @@
           <t>SHINDE ENTERPRISES</t>
         </is>
       </c>
+      <c r="O255" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="21" t="n">
@@ -12407,6 +13337,11 @@
           <t>SAI KRUPA AGENCY</t>
         </is>
       </c>
+      <c r="O256" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="21" t="n">
@@ -12457,6 +13392,11 @@
           <t>MAHENDRA DISRIBUTORS</t>
         </is>
       </c>
+      <c r="O257" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="21" t="n">
@@ -12503,6 +13443,11 @@
           <t>V R ENTERPRISES</t>
         </is>
       </c>
+      <c r="O258" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="21" t="n">
@@ -12543,6 +13488,11 @@
         </is>
       </c>
       <c r="L259" s="6" t="n"/>
+      <c r="O259" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="21" t="n">
@@ -12583,6 +13533,21 @@
         </is>
       </c>
       <c r="L260" s="6" t="n"/>
+      <c r="M260" s="35" t="inlineStr">
+        <is>
+          <t>610</t>
+        </is>
+      </c>
+      <c r="N260" s="35" t="inlineStr">
+        <is>
+          <t>DHANWANTRI PHARMA</t>
+        </is>
+      </c>
+      <c r="O260" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="21" t="n">
@@ -12623,6 +13588,21 @@
         </is>
       </c>
       <c r="L261" s="6" t="n"/>
+      <c r="M261" s="35" t="inlineStr">
+        <is>
+          <t>682,705</t>
+        </is>
+      </c>
+      <c r="N261" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O261" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="21" t="n">
@@ -12765,6 +13745,11 @@
           <t>MANGAL ENTERPRISES</t>
         </is>
       </c>
+      <c r="O264" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="21" t="n">
@@ -12899,6 +13884,11 @@
           <t>KRISHNA MEDICAL &amp; SURGICAL</t>
         </is>
       </c>
+      <c r="O267" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="21" t="n">
@@ -12945,6 +13935,11 @@
           <t>M/S MANDAR AGENCY</t>
         </is>
       </c>
+      <c r="O268" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="21" t="n">
@@ -12991,6 +13986,11 @@
           <t>SHREE GANESH ENTERPISES</t>
         </is>
       </c>
+      <c r="O269" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="21" t="n">
@@ -13031,6 +14031,21 @@
         </is>
       </c>
       <c r="L270" s="6" t="n"/>
+      <c r="M270" s="35" t="inlineStr">
+        <is>
+          <t>719</t>
+        </is>
+      </c>
+      <c r="N270" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O270" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="21" t="n">
@@ -13173,6 +14188,11 @@
           <t>ARIHANT ENTERPRISES</t>
         </is>
       </c>
+      <c r="O273" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="21" t="n">
@@ -13219,6 +14239,11 @@
           <t>RAJLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O274" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="21" t="n">
@@ -13307,6 +14332,11 @@
         </is>
       </c>
       <c r="L276" s="6" t="n"/>
+      <c r="O276" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="21" t="n">
@@ -13353,6 +14383,11 @@
           <t>AARADHYA AGENCIES</t>
         </is>
       </c>
+      <c r="O277" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="21" t="n">
@@ -13399,6 +14434,11 @@
           <t>SHRI KULSWAMINI DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O278" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="21" t="n">
@@ -13445,6 +14485,11 @@
           <t>SAI MARKETING</t>
         </is>
       </c>
+      <c r="O279" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="21" t="n">
@@ -13491,6 +14536,11 @@
           <t>RAUT TRADINGS</t>
         </is>
       </c>
+      <c r="O280" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="21" t="n">
@@ -13713,6 +14763,11 @@
           <t>YASH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O285" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="21" t="n">
@@ -13759,6 +14814,11 @@
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
+      <c r="O286" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="21" t="n">
@@ -13853,6 +14913,11 @@
           <t>SONIGARA DISTRIBUTOR</t>
         </is>
       </c>
+      <c r="O288" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="21" t="n">
@@ -13899,6 +14964,11 @@
           <t>N R ENTERPRISES</t>
         </is>
       </c>
+      <c r="O289" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="21" t="n">
@@ -13945,6 +15015,11 @@
           <t>TAPADIYA COSMOGEN</t>
         </is>
       </c>
+      <c r="O290" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="21" t="n">
@@ -13991,6 +15066,11 @@
           <t>GOVINDA FOODS</t>
         </is>
       </c>
+      <c r="O291" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="21" t="n">
@@ -14041,6 +15121,11 @@
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
+      <c r="O292" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="21" t="n">
@@ -14081,6 +15166,21 @@
         </is>
       </c>
       <c r="L293" s="6" t="n"/>
+      <c r="M293" s="35" t="inlineStr">
+        <is>
+          <t>42,180,235,189,253,259</t>
+        </is>
+      </c>
+      <c r="N293" s="35" t="inlineStr">
+        <is>
+          <t>YASHVI AGENCIES</t>
+        </is>
+      </c>
+      <c r="O293" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="21" t="n">
@@ -14337,6 +15437,11 @@
         </is>
       </c>
       <c r="L299" s="6" t="n"/>
+      <c r="O299" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="21" t="n">
@@ -14383,6 +15488,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O300" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="21" t="n">
@@ -14429,6 +15539,11 @@
           <t>SHINDE ENTERPRISES</t>
         </is>
       </c>
+      <c r="O301" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="21" t="n">
@@ -14549,6 +15664,17 @@
         </is>
       </c>
       <c r="L304" s="6" t="n"/>
+      <c r="M304" s="35" t="inlineStr"/>
+      <c r="N304" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O304" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="21" t="n">
@@ -14589,6 +15715,21 @@
         </is>
       </c>
       <c r="L305" s="6" t="n"/>
+      <c r="M305" s="35" t="inlineStr">
+        <is>
+          <t>689</t>
+        </is>
+      </c>
+      <c r="N305" s="35" t="inlineStr">
+        <is>
+          <t>SUPARSHWA MEDCARE LLP</t>
+        </is>
+      </c>
+      <c r="O305" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="21" t="n">
@@ -14753,6 +15894,21 @@
         </is>
       </c>
       <c r="L309" s="6" t="n"/>
+      <c r="M309" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N309" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O309" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="21" t="n">
@@ -15139,6 +16295,11 @@
           <t>JEEVIKA HOSPITALITY SERVICES</t>
         </is>
       </c>
+      <c r="O318" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="21" t="n">
@@ -15179,6 +16340,17 @@
         </is>
       </c>
       <c r="L319" s="6" t="n"/>
+      <c r="M319" s="35" t="inlineStr"/>
+      <c r="N319" s="35" t="inlineStr">
+        <is>
+          <t>SHUBH ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O319" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="21" t="n">
@@ -15219,6 +16391,21 @@
         </is>
       </c>
       <c r="L320" s="6" t="n"/>
+      <c r="M320" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N320" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O320" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="321" customFormat="1" s="2">
       <c r="A321" s="22" t="n">
@@ -15783,6 +16970,11 @@
         </is>
       </c>
       <c r="L333" s="6" t="n"/>
+      <c r="O333" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="21" t="n">
@@ -15829,6 +17021,11 @@
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
+      <c r="O334" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="21" t="n">
@@ -15967,6 +17164,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O337" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="21" t="n">
@@ -16013,6 +17215,11 @@
           <t>CHINTAMANI DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O338" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="21" t="n">
@@ -16059,6 +17266,11 @@
           <t>UNICO AGENCIES</t>
         </is>
       </c>
+      <c r="O339" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="21" t="n">
@@ -16105,6 +17317,11 @@
           <t>PRASHANT-NX</t>
         </is>
       </c>
+      <c r="O340" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="21" t="n">
@@ -16155,6 +17372,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O341" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="21" t="n">
@@ -16243,6 +17465,11 @@
         </is>
       </c>
       <c r="L343" s="6" t="n"/>
+      <c r="O343" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="21" t="n">
@@ -16451,6 +17678,21 @@
         </is>
       </c>
       <c r="L348" s="6" t="n"/>
+      <c r="M348" s="35" t="inlineStr">
+        <is>
+          <t>497,656</t>
+        </is>
+      </c>
+      <c r="N348" s="35" t="inlineStr">
+        <is>
+          <t>SHREYAA AGENCIES</t>
+        </is>
+      </c>
+      <c r="O348" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="21" t="n">
@@ -16585,6 +17827,11 @@
           <t>ASHA MOHAN ENTERPRISES</t>
         </is>
       </c>
+      <c r="O351" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="21" t="n">
@@ -16799,6 +18046,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O356" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="21" t="n">
@@ -16845,6 +18097,11 @@
           <t>RAUT TRADINGS</t>
         </is>
       </c>
+      <c r="O357" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="21" t="n">
@@ -16895,6 +18152,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O358" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="21" t="n">
@@ -16935,6 +18197,11 @@
         </is>
       </c>
       <c r="L359" s="6" t="n"/>
+      <c r="O359" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="21" t="n">
@@ -17325,6 +18592,11 @@
           <t>MEDIRAJ DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O368" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="21" t="n">
@@ -17365,6 +18637,11 @@
         </is>
       </c>
       <c r="L369" s="6" t="n"/>
+      <c r="O369" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="21" t="n">
@@ -17405,6 +18682,11 @@
         </is>
       </c>
       <c r="L370" s="6" t="n"/>
+      <c r="O370" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="21" t="n">
@@ -17451,6 +18733,11 @@
           <t>G K ENTERPRISES</t>
         </is>
       </c>
+      <c r="O371" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="21" t="n">
@@ -17539,6 +18826,11 @@
         </is>
       </c>
       <c r="L373" s="6" t="n"/>
+      <c r="O373" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="21" t="n">
@@ -17659,6 +18951,21 @@
         </is>
       </c>
       <c r="L376" s="6" t="n"/>
+      <c r="M376" s="35" t="inlineStr">
+        <is>
+          <t>804,753,805,770</t>
+        </is>
+      </c>
+      <c r="N376" s="35" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O376" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="21" t="n">
@@ -17841,6 +19148,11 @@
           <t>SANIKA ENTERPRISES</t>
         </is>
       </c>
+      <c r="O380" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="21" t="n">
@@ -17881,6 +19193,17 @@
         </is>
       </c>
       <c r="L381" s="6" t="n"/>
+      <c r="M381" s="35" t="inlineStr"/>
+      <c r="N381" s="35" t="inlineStr">
+        <is>
+          <t>SUMEET AGENCIES</t>
+        </is>
+      </c>
+      <c r="O381" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="21" t="n">
@@ -17927,6 +19250,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O382" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="21" t="n">
@@ -18013,6 +19341,11 @@
           <t>SHREE GANESH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O384" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="21" t="n">
@@ -18275,6 +19608,11 @@
           <t>V R ENTERPRISES</t>
         </is>
       </c>
+      <c r="O390" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="391">
       <c r="A391" s="21" t="n">
@@ -18321,6 +19659,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O391" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="21" t="n">
@@ -18371,6 +19714,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O392" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="21" t="n">
@@ -18465,6 +19813,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O394" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="21" t="n">
@@ -18505,6 +19858,11 @@
         </is>
       </c>
       <c r="L395" s="6" t="n"/>
+      <c r="O395" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="21" t="n">
@@ -18551,6 +19909,11 @@
           <t>REKHA MARKETING</t>
         </is>
       </c>
+      <c r="O396" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="21" t="n">
@@ -18597,6 +19960,11 @@
           <t>NANDINI BEAUTY</t>
         </is>
       </c>
+      <c r="O397" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="21" t="n">
@@ -18691,6 +20059,11 @@
           <t>JAI SHREE GANESH AGENCIES</t>
         </is>
       </c>
+      <c r="O399" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="21" t="n">
@@ -18737,6 +20110,11 @@
           <t>HEALTH PLUS MEDICO</t>
         </is>
       </c>
+      <c r="O400" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="21" t="n">
@@ -18783,6 +20161,11 @@
           <t>SARTHAK SALES AGENCY</t>
         </is>
       </c>
+      <c r="O401" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="21" t="n">
@@ -18957,6 +20340,11 @@
           <t>SHREYAA AGENCIES</t>
         </is>
       </c>
+      <c r="O405" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="21" t="n">
@@ -18997,6 +20385,11 @@
         </is>
       </c>
       <c r="L406" s="6" t="n"/>
+      <c r="O406" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="21" t="n">
@@ -19421,6 +20814,21 @@
         </is>
       </c>
       <c r="L416" s="6" t="n"/>
+      <c r="M416" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N416" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O416" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" s="21" t="n">
@@ -19509,6 +20917,11 @@
         </is>
       </c>
       <c r="L418" s="6" t="n"/>
+      <c r="O418" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" s="21" t="n">
@@ -19593,6 +21006,11 @@
         </is>
       </c>
       <c r="L420" s="6" t="n"/>
+      <c r="O420" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="21" t="n">
@@ -19633,6 +21051,11 @@
         </is>
       </c>
       <c r="L421" s="6" t="n"/>
+      <c r="O421" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" s="21" t="n">
@@ -19767,6 +21190,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O424" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" s="21" t="n">
@@ -19813,6 +21241,11 @@
           <t>SUMEET AGENCIES</t>
         </is>
       </c>
+      <c r="O425" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" s="21" t="n">
@@ -19903,6 +21336,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O427" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="21" t="n">
@@ -20039,6 +21477,11 @@
         </is>
       </c>
       <c r="L430" s="6" t="n"/>
+      <c r="O430" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="21" t="n">
@@ -20079,6 +21522,11 @@
         </is>
       </c>
       <c r="L431" s="6" t="n"/>
+      <c r="O431" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="21" t="n">
@@ -20125,6 +21573,11 @@
           <t>THE MEDI SHOPEE</t>
         </is>
       </c>
+      <c r="O432" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="21" t="n">
@@ -20259,6 +21712,11 @@
           <t>HEALTH PLUS MEDICO</t>
         </is>
       </c>
+      <c r="O435" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="21" t="n">
@@ -20353,6 +21811,11 @@
           <t>SRI BALAJI FOODS</t>
         </is>
       </c>
+      <c r="O437" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" s="21" t="n">
@@ -20399,6 +21862,11 @@
           <t>MOHAN CHEMIST</t>
         </is>
       </c>
+      <c r="O438" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="21" t="n">
@@ -20577,6 +22045,11 @@
           <t>N R ENTERPRISES</t>
         </is>
       </c>
+      <c r="O442" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="21" t="n">
@@ -20627,6 +22100,11 @@
           <t>SHREE DATTA KRUPA AGENCY</t>
         </is>
       </c>
+      <c r="O443" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="21" t="n">
@@ -20667,6 +22145,11 @@
         </is>
       </c>
       <c r="L444" s="6" t="n"/>
+      <c r="O444" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="21" t="n">
@@ -20747,6 +22230,21 @@
         </is>
       </c>
       <c r="L446" s="6" t="n"/>
+      <c r="M446" s="35" t="inlineStr">
+        <is>
+          <t>623,632,640,648,661,676,687,707,722,728,736,744,750,758,774,783,807,818,857,875,894,902,909,925,934,941</t>
+        </is>
+      </c>
+      <c r="N446" s="35" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O446" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="21" t="n">
@@ -20915,6 +22413,11 @@
         </is>
       </c>
       <c r="L450" s="6" t="n"/>
+      <c r="O450" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="21" t="n">
@@ -21175,6 +22678,21 @@
         </is>
       </c>
       <c r="L456" s="6" t="n"/>
+      <c r="M456" s="35" t="inlineStr">
+        <is>
+          <t>477,678,776,869,960</t>
+        </is>
+      </c>
+      <c r="N456" s="35" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O456" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="21" t="n">
@@ -21259,6 +22777,11 @@
         </is>
       </c>
       <c r="L458" s="6" t="n"/>
+      <c r="O458" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="21" t="n">
@@ -21299,6 +22822,11 @@
         </is>
       </c>
       <c r="L459" s="6" t="n"/>
+      <c r="O459" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="21" t="n">
@@ -21345,6 +22873,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O460" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="21" t="n">
@@ -21683,6 +23216,11 @@
           <t>JEEVIKA HOSPITALITY SERVICES</t>
         </is>
       </c>
+      <c r="O468" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="469">
       <c r="A469" s="21" t="n">
@@ -21723,6 +23261,11 @@
         </is>
       </c>
       <c r="L469" s="6" t="n"/>
+      <c r="O469" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="21" t="n">
@@ -21769,6 +23312,11 @@
           <t>SWARA ENTERPRISES</t>
         </is>
       </c>
+      <c r="O470" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="21" t="n">
@@ -21809,6 +23357,11 @@
         </is>
       </c>
       <c r="L471" s="6" t="n"/>
+      <c r="O471" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="21" t="n">
@@ -21897,6 +23450,11 @@
         </is>
       </c>
       <c r="L473" s="6" t="n"/>
+      <c r="O473" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="474">
       <c r="A474" s="21" t="n">
@@ -22097,6 +23655,21 @@
         </is>
       </c>
       <c r="L478" s="6" t="n"/>
+      <c r="M478" s="35" t="inlineStr">
+        <is>
+          <t>585,593,594,605,620,631,642,647,658,679,686,706,729,742,752,759,760,775,785,799,808,817,819,828,840,858,878,893,905,922,937,942</t>
+        </is>
+      </c>
+      <c r="N478" s="35" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O478" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" s="21" t="n">
@@ -22261,6 +23834,21 @@
         </is>
       </c>
       <c r="L482" s="6" t="n"/>
+      <c r="M482" s="35" t="inlineStr">
+        <is>
+          <t>488</t>
+        </is>
+      </c>
+      <c r="N482" s="35" t="inlineStr">
+        <is>
+          <t>DHANVANTARI SALES</t>
+        </is>
+      </c>
+      <c r="O482" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" s="21" t="n">
@@ -22349,6 +23937,11 @@
         </is>
       </c>
       <c r="L484" s="6" t="n"/>
+      <c r="O484" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" s="21" t="n">
@@ -22389,6 +23982,11 @@
         </is>
       </c>
       <c r="L485" s="6" t="n"/>
+      <c r="O485" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" s="21" t="n">
@@ -22429,6 +24027,11 @@
         </is>
       </c>
       <c r="L486" s="6" t="n"/>
+      <c r="O486" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="487">
       <c r="A487" s="21" t="n">
@@ -22925,6 +24528,21 @@
         </is>
       </c>
       <c r="L498" s="6" t="n"/>
+      <c r="M498" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N498" s="35" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O498" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" s="21" t="n">
@@ -23067,6 +24685,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O501" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" s="21" t="n">
@@ -23113,6 +24736,11 @@
           <t>HEALTH PLUS MEDICO</t>
         </is>
       </c>
+      <c r="O502" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" s="21" t="n">
@@ -23153,6 +24781,11 @@
         </is>
       </c>
       <c r="L503" s="6" t="n"/>
+      <c r="O503" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="504">
       <c r="A504" s="21" t="n">
@@ -23239,6 +24872,11 @@
           <t>DHYAANI NEXUS PVT.LTD.</t>
         </is>
       </c>
+      <c r="O505" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="506">
       <c r="A506" s="21" t="n">
@@ -23453,6 +25091,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O510" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" s="21" t="n">
@@ -23503,6 +25146,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O511" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="512">
       <c r="A512" s="21" t="n">
@@ -23549,6 +25197,11 @@
           <t>3P'S ENTERPRISES</t>
         </is>
       </c>
+      <c r="O512" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" s="21" t="n">
@@ -23595,6 +25248,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O513" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" s="21" t="n">
@@ -23641,6 +25299,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O514" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" s="21" t="n">
@@ -23809,6 +25472,11 @@
         </is>
       </c>
       <c r="L518" s="6" t="n"/>
+      <c r="O518" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="519">
       <c r="A519" s="21" t="n">
@@ -23855,6 +25523,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O519" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" s="21" t="n">
@@ -23901,6 +25574,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O520" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" s="21" t="n">
@@ -23947,6 +25625,11 @@
           <t>ANNUGRAH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O521" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="522">
       <c r="A522" s="21" t="n">
@@ -23987,6 +25670,11 @@
         </is>
       </c>
       <c r="L522" s="6" t="n"/>
+      <c r="O522" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" s="21" t="n">
@@ -24027,6 +25715,11 @@
         </is>
       </c>
       <c r="L523" s="6" t="n"/>
+      <c r="O523" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="524">
       <c r="A524" s="21" t="n">
@@ -24067,6 +25760,11 @@
         </is>
       </c>
       <c r="L524" s="6" t="n"/>
+      <c r="O524" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="525">
       <c r="A525" s="21" t="n">
@@ -24113,6 +25811,11 @@
           <t>ARIHANT ENTERPRISES</t>
         </is>
       </c>
+      <c r="O525" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" s="21" t="n">
@@ -24383,6 +26086,11 @@
           <t>SHRI KULSWAMINI DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O531" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="532">
       <c r="A532" s="21" t="n">
@@ -24429,6 +26137,11 @@
           <t>SHUBH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O532" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="533">
       <c r="A533" s="21" t="n">
@@ -24475,6 +26188,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O533" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="534">
       <c r="A534" s="21" t="n">
@@ -24555,6 +26273,21 @@
         </is>
       </c>
       <c r="L535" s="6" t="n"/>
+      <c r="M535" s="35" t="inlineStr">
+        <is>
+          <t>2359,680,683,684,704,726,735,741,746,751,763,789,796,824,829,843,853,874,887,906,910,933</t>
+        </is>
+      </c>
+      <c r="N535" s="35" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O535" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="21" t="n">
@@ -24639,6 +26372,21 @@
           <t>salary</t>
         </is>
       </c>
+      <c r="M537" s="35" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N537" s="35" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O537" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" s="21" t="n">
@@ -24981,6 +26729,11 @@
           <t>ATUL ENTERPRISES</t>
         </is>
       </c>
+      <c r="O545" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="546">
       <c r="A546" s="21" t="n">
@@ -25027,6 +26780,11 @@
           <t>ATUL ENTERPRISES</t>
         </is>
       </c>
+      <c r="O546" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="547">
       <c r="A547" s="21" t="n">
@@ -25409,6 +27167,11 @@
           <t>VED AUSHADHALAYA</t>
         </is>
       </c>
+      <c r="O555" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="556">
       <c r="A556" s="21" t="n">
@@ -25449,6 +27212,11 @@
         </is>
       </c>
       <c r="L556" s="6" t="n"/>
+      <c r="O556" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="557">
       <c r="A557" s="21" t="n">
@@ -25489,6 +27257,11 @@
         </is>
       </c>
       <c r="L557" s="6" t="n"/>
+      <c r="O557" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="558">
       <c r="A558" s="21" t="n">
@@ -25735,6 +27508,11 @@
           <t>SARA MARKETING</t>
         </is>
       </c>
+      <c r="O563" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="564">
       <c r="A564" s="21" t="n">
@@ -25829,6 +27607,11 @@
           <t>G K ENTERPRISES</t>
         </is>
       </c>
+      <c r="O565" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" s="21" t="n">
@@ -25967,6 +27750,11 @@
           <t>RUSHABH SURGICALS</t>
         </is>
       </c>
+      <c r="O568" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="569">
       <c r="A569" s="21" t="n">
@@ -26047,6 +27835,21 @@
         </is>
       </c>
       <c r="L570" s="6" t="n"/>
+      <c r="M570" s="35" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="N570" s="35" t="inlineStr">
+        <is>
+          <t>NAVMAHARASTRA ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O570" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" s="21" t="n">
@@ -26141,6 +27944,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O572" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" s="21" t="n">
@@ -26181,6 +27989,11 @@
         </is>
       </c>
       <c r="L573" s="6" t="n"/>
+      <c r="O573" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" s="21" t="n">
@@ -26349,6 +28162,11 @@
         </is>
       </c>
       <c r="L577" s="6" t="n"/>
+      <c r="O577" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" s="21" t="n">
@@ -26395,6 +28213,11 @@
           <t>REKHA MARKETING</t>
         </is>
       </c>
+      <c r="O578" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" s="21" t="n">
@@ -27019,6 +28842,11 @@
         </is>
       </c>
       <c r="L593" s="6" t="n"/>
+      <c r="O593" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="594">
       <c r="A594" s="21" t="n">
@@ -27059,6 +28887,11 @@
         </is>
       </c>
       <c r="L594" s="6" t="n"/>
+      <c r="O594" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="595">
       <c r="A595" s="21" t="n">
@@ -27105,6 +28938,11 @@
           <t>DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
+      <c r="O595" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="596">
       <c r="A596" s="21" t="n">
@@ -27323,6 +29161,11 @@
           <t>MAHENDRA DISRIBUTORS</t>
         </is>
       </c>
+      <c r="O600" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="601">
       <c r="A601" s="21" t="n">
@@ -27373,6 +29216,11 @@
           <t>TRIDENT MEDLIFE PVT LTD</t>
         </is>
       </c>
+      <c r="O601" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="602">
       <c r="A602" s="21" t="n">
@@ -27419,6 +29267,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O602" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="603">
       <c r="A603" s="21" t="n">
@@ -27465,6 +29318,11 @@
           <t>M/S MANDAR AGENCY</t>
         </is>
       </c>
+      <c r="O603" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="604">
       <c r="A604" s="21" t="n">
@@ -27511,6 +29369,11 @@
           <t>M/S MANDAR AGENCY</t>
         </is>
       </c>
+      <c r="O604" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="605">
       <c r="A605" s="21" t="n">
@@ -27557,6 +29420,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O605" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="606">
       <c r="A606" s="21" t="n">
@@ -27597,6 +29465,11 @@
         </is>
       </c>
       <c r="L606" s="6" t="n"/>
+      <c r="O606" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="607">
       <c r="A607" s="21" t="n">
@@ -27683,6 +29556,11 @@
           <t>M/S MANDAR AGENCY</t>
         </is>
       </c>
+      <c r="O608" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="609">
       <c r="A609" s="21" t="n">
@@ -27763,6 +29641,21 @@
         </is>
       </c>
       <c r="L610" s="6" t="n"/>
+      <c r="M610" s="35" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="N610" s="35" t="inlineStr">
+        <is>
+          <t>LOCAL PURCHASE</t>
+        </is>
+      </c>
+      <c r="O610" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="611">
       <c r="A611" s="21" t="n">
@@ -27937,6 +29830,11 @@
           <t>ANNUGRAH ENTERPRISES</t>
         </is>
       </c>
+      <c r="O614" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="615">
       <c r="A615" s="21" t="n">
@@ -27983,6 +29881,11 @@
           <t>CHINTAMANI DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O615" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="616">
       <c r="A616" s="21" t="n">
@@ -28023,6 +29926,11 @@
         </is>
       </c>
       <c r="L616" s="6" t="n"/>
+      <c r="O616" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="617">
       <c r="A617" s="21" t="n">
@@ -28063,6 +29971,11 @@
         </is>
       </c>
       <c r="L617" s="6" t="n"/>
+      <c r="O617" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="618">
       <c r="A618" s="21" t="n">
@@ -28413,6 +30326,11 @@
           <t>MAULI AGENCIES</t>
         </is>
       </c>
+      <c r="O625" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="626">
       <c r="A626" s="21" t="n">
@@ -28453,6 +30371,11 @@
         </is>
       </c>
       <c r="L626" s="6" t="n"/>
+      <c r="O626" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="627">
       <c r="A627" s="21" t="n">
@@ -28581,6 +30504,11 @@
         </is>
       </c>
       <c r="L629" s="6" t="n"/>
+      <c r="O629" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="630">
       <c r="A630" s="21" t="n">
@@ -29205,6 +31133,11 @@
         </is>
       </c>
       <c r="L644" s="6" t="n"/>
+      <c r="O644" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="645">
       <c r="A645" s="21" t="n">
@@ -29381,6 +31314,21 @@
         </is>
       </c>
       <c r="L648" s="6" t="n"/>
+      <c r="M648" s="35" t="inlineStr">
+        <is>
+          <t>949,957,969,980,987,1006,1011,1023,1032,1039,1053,1068,1076,1106</t>
+        </is>
+      </c>
+      <c r="N648" s="35" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O648" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="21" t="n">
@@ -29505,6 +31453,21 @@
         </is>
       </c>
       <c r="L651" s="6" t="n"/>
+      <c r="M651" s="35" t="inlineStr">
+        <is>
+          <t>1083,1108,1128</t>
+        </is>
+      </c>
+      <c r="N651" s="35" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O651" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" s="21" t="n">
@@ -29807,6 +31770,11 @@
           <t>SONIGARA DISTRIBUTOR</t>
         </is>
       </c>
+      <c r="O658" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="659">
       <c r="A659" s="21" t="n">
@@ -29847,6 +31815,11 @@
         </is>
       </c>
       <c r="L659" s="6" t="n"/>
+      <c r="O659" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="660">
       <c r="A660" s="21" t="n">
@@ -29887,6 +31860,11 @@
         </is>
       </c>
       <c r="L660" s="6" t="n"/>
+      <c r="O660" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="661">
       <c r="A661" s="21" t="n">
@@ -30175,6 +32153,11 @@
         </is>
       </c>
       <c r="L667" s="6" t="n"/>
+      <c r="O667" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="668">
       <c r="A668" s="21" t="n">
@@ -30215,6 +32198,11 @@
         </is>
       </c>
       <c r="L668" s="6" t="n"/>
+      <c r="O668" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="669">
       <c r="A669" s="21" t="n">
@@ -30255,6 +32243,11 @@
         </is>
       </c>
       <c r="L669" s="6" t="n"/>
+      <c r="O669" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="670">
       <c r="A670" s="21" t="n">
@@ -30295,6 +32288,11 @@
         </is>
       </c>
       <c r="L670" s="6" t="n"/>
+      <c r="O670" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="671">
       <c r="A671" s="21" t="n">
@@ -30589,6 +32587,11 @@
           <t>R M ENTERPRISES</t>
         </is>
       </c>
+      <c r="O677" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="678">
       <c r="A678" s="21" t="n">
@@ -30635,6 +32638,11 @@
           <t>ATUL ENTERPRISES</t>
         </is>
       </c>
+      <c r="O678" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="679">
       <c r="A679" s="21" t="n">
@@ -31017,6 +33025,11 @@
           <t>G K ENTERPRISES</t>
         </is>
       </c>
+      <c r="O687" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="688">
       <c r="A688" s="21" t="n">
@@ -31363,6 +33376,11 @@
           <t>THE PLUS ENTERPRISES</t>
         </is>
       </c>
+      <c r="O695" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="696">
       <c r="A696" s="21" t="n">
@@ -31409,6 +33427,11 @@
           <t>AARADHYA AGENCIES</t>
         </is>
       </c>
+      <c r="O696" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="697">
       <c r="A697" s="21" t="n">
@@ -31455,6 +33478,11 @@
           <t>SHINDE ENTERPRISES</t>
         </is>
       </c>
+      <c r="O697" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="698">
       <c r="A698" s="21" t="n">
@@ -31505,6 +33533,11 @@
           <t>MEDIRAJ DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O698" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="699">
       <c r="A699" s="21" t="n">
@@ -31555,6 +33588,11 @@
           <t>MEDIRAJ DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O699" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="700">
       <c r="A700" s="21" t="n">
@@ -31691,6 +33729,11 @@
         </is>
       </c>
       <c r="L702" s="6" t="n"/>
+      <c r="O702" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="703">
       <c r="A703" s="21" t="n">
@@ -31779,6 +33822,11 @@
         </is>
       </c>
       <c r="L704" s="6" t="n"/>
+      <c r="O704" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="705">
       <c r="A705" s="21" t="n">
@@ -31819,6 +33867,11 @@
         </is>
       </c>
       <c r="L705" s="6" t="n"/>
+      <c r="O705" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="706">
       <c r="A706" s="21" t="n">
@@ -31905,6 +33958,11 @@
           <t>AV TRADERS</t>
         </is>
       </c>
+      <c r="O707" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="708">
       <c r="A708" s="21" t="n">
@@ -31951,6 +34009,11 @@
           <t>CG MARKETING PVT LTD</t>
         </is>
       </c>
+      <c r="O708" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="709">
       <c r="A709" s="21" t="n">
@@ -32309,6 +34372,11 @@
           <t>SHREE SIDDHESHWAR ENTERISES</t>
         </is>
       </c>
+      <c r="O716" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="717">
       <c r="A717" s="21" t="n">
@@ -32355,6 +34423,11 @@
           <t>SAI KRUPA AGENCY</t>
         </is>
       </c>
+      <c r="O717" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="718">
       <c r="A718" s="21" t="n">
@@ -32405,6 +34478,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O718" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="719">
       <c r="A719" s="21" t="n">
@@ -32445,6 +34523,11 @@
         </is>
       </c>
       <c r="L719" s="6" t="n"/>
+      <c r="O719" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="720">
       <c r="A720" s="21" t="n">
@@ -32485,6 +34568,11 @@
         </is>
       </c>
       <c r="L720" s="6" t="n"/>
+      <c r="O720" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="721">
       <c r="A721" s="21" t="n">
@@ -32579,6 +34667,11 @@
           <t>VISION SALES</t>
         </is>
       </c>
+      <c r="O722" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="723">
       <c r="A723" s="21" t="n">
@@ -32619,6 +34712,11 @@
         </is>
       </c>
       <c r="L723" s="6" t="n"/>
+      <c r="O723" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="724">
       <c r="A724" s="21" t="n">
@@ -32747,6 +34845,21 @@
         </is>
       </c>
       <c r="L726" s="6" t="n"/>
+      <c r="M726" s="35" t="inlineStr">
+        <is>
+          <t>201,199</t>
+        </is>
+      </c>
+      <c r="N726" s="35" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O726" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="727">
       <c r="A727" s="21" t="n">
@@ -32787,6 +34900,11 @@
         </is>
       </c>
       <c r="L727" s="6" t="n"/>
+      <c r="O727" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" s="21" t="n">
@@ -32827,6 +34945,11 @@
         </is>
       </c>
       <c r="L728" s="6" t="n"/>
+      <c r="O728" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="729">
       <c r="A729" s="21" t="n">
@@ -32955,6 +35078,11 @@
         </is>
       </c>
       <c r="L731" s="6" t="n"/>
+      <c r="O731" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="732">
       <c r="A732" s="21" t="n">
@@ -32995,6 +35123,11 @@
         </is>
       </c>
       <c r="L732" s="6" t="n"/>
+      <c r="O732" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="733">
       <c r="A733" s="21" t="n">
@@ -33035,6 +35168,11 @@
         </is>
       </c>
       <c r="L733" s="6" t="n"/>
+      <c r="O733" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="734">
       <c r="A734" s="21" t="n">
@@ -33159,6 +35297,11 @@
         </is>
       </c>
       <c r="L736" s="6" t="n"/>
+      <c r="O736" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="737">
       <c r="A737" s="21" t="n">
@@ -33247,6 +35390,11 @@
         </is>
       </c>
       <c r="L738" s="6" t="n"/>
+      <c r="O738" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="739">
       <c r="A739" s="21" t="n">
@@ -33287,6 +35435,11 @@
         </is>
       </c>
       <c r="L739" s="6" t="n"/>
+      <c r="O739" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" s="21" t="n">
@@ -33471,6 +35624,11 @@
         </is>
       </c>
       <c r="L743" s="6" t="n"/>
+      <c r="O743" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="744">
       <c r="A744" s="21" t="n">
@@ -33511,6 +35669,11 @@
         </is>
       </c>
       <c r="L744" s="6" t="n"/>
+      <c r="O744" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="745">
       <c r="A745" s="21" t="n">
@@ -33595,6 +35758,21 @@
         </is>
       </c>
       <c r="L746" s="6" t="n"/>
+      <c r="M746" s="35" t="inlineStr">
+        <is>
+          <t>42,180,235,189,253,259</t>
+        </is>
+      </c>
+      <c r="N746" s="35" t="inlineStr">
+        <is>
+          <t>YASHVI AGENCIES</t>
+        </is>
+      </c>
+      <c r="O746" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="747">
       <c r="A747" s="21" t="n">
@@ -33727,6 +35905,11 @@
         </is>
       </c>
       <c r="L749" s="6" t="n"/>
+      <c r="O749" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="750">
       <c r="A750" s="21" t="n">
@@ -33767,6 +35950,11 @@
         </is>
       </c>
       <c r="L750" s="6" t="n"/>
+      <c r="O750" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="751">
       <c r="A751" s="21" t="n">
@@ -33975,6 +36163,11 @@
         </is>
       </c>
       <c r="L755" s="6" t="n"/>
+      <c r="O755" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="756">
       <c r="A756" s="21" t="n">
@@ -34015,6 +36208,11 @@
         </is>
       </c>
       <c r="L756" s="6" t="n"/>
+      <c r="O756" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="757">
       <c r="A757" s="21" t="n">
@@ -34263,6 +36461,11 @@
         </is>
       </c>
       <c r="L762" s="6" t="n"/>
+      <c r="O762" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="763">
       <c r="A763" s="21" t="n">
@@ -34569,6 +36772,11 @@
           <t>SENIOR AGENCY</t>
         </is>
       </c>
+      <c r="O769" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" s="21" t="n">
@@ -34707,6 +36915,11 @@
           <t>MEDIRAJ DISTRIBUTORS</t>
         </is>
       </c>
+      <c r="O772" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="773">
       <c r="A773" s="21" t="n">
@@ -35169,6 +37382,11 @@
           <t>HEALTH PLUS MEDICO</t>
         </is>
       </c>
+      <c r="O783" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="784">
       <c r="A784" s="21" t="n">
@@ -35209,6 +37427,11 @@
         </is>
       </c>
       <c r="L784" s="6" t="n"/>
+      <c r="O784" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="785">
       <c r="A785" s="21" t="n">
@@ -35509,6 +37732,11 @@
         </is>
       </c>
       <c r="L791" s="6" t="n"/>
+      <c r="O791" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="792">
       <c r="A792" s="21" t="n">
@@ -35549,6 +37777,11 @@
         </is>
       </c>
       <c r="L792" s="6" t="n"/>
+      <c r="O792" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="793">
       <c r="A793" s="21" t="n">
@@ -35589,6 +37822,11 @@
         </is>
       </c>
       <c r="L793" s="6" t="n"/>
+      <c r="O793" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="794">
       <c r="A794" s="21" t="n">
@@ -35629,6 +37867,11 @@
         </is>
       </c>
       <c r="L794" s="6" t="n"/>
+      <c r="O794" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="795">
       <c r="A795" s="21" t="n">
@@ -35757,6 +38000,11 @@
         </is>
       </c>
       <c r="L797" s="6" t="n"/>
+      <c r="O797" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="798">
       <c r="A798" s="21" t="n">
@@ -35929,6 +38177,21 @@
         </is>
       </c>
       <c r="L801" s="6" t="n"/>
+      <c r="M801" s="35" t="inlineStr">
+        <is>
+          <t>42,180,235,189,253,259</t>
+        </is>
+      </c>
+      <c r="N801" s="35" t="inlineStr">
+        <is>
+          <t>YASHVI AGENCIES</t>
+        </is>
+      </c>
+      <c r="O801" s="35" t="inlineStr">
+        <is>
+          <t>GPAY_AMT_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="802">
       <c r="A802" s="21" t="n">
@@ -36017,6 +38280,11 @@
         </is>
       </c>
       <c r="L803" s="6" t="n"/>
+      <c r="O803" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="804">
       <c r="A804" s="21" t="n">
@@ -36057,6 +38325,11 @@
         </is>
       </c>
       <c r="L804" s="6" t="n"/>
+      <c r="O804" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="805">
       <c r="A805" s="21" t="n">
@@ -36185,6 +38458,11 @@
         </is>
       </c>
       <c r="L807" s="6" t="n"/>
+      <c r="O807" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="808">
       <c r="A808" s="21" t="n">
@@ -36273,6 +38551,11 @@
         </is>
       </c>
       <c r="L809" s="6" t="n"/>
+      <c r="O809" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="810">
       <c r="A810" s="21" t="n">
@@ -36393,6 +38676,11 @@
         </is>
       </c>
       <c r="L812" s="6" t="n"/>
+      <c r="O812" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="813">
       <c r="A813" s="21" t="n">
@@ -36905,6 +39193,11 @@
         </is>
       </c>
       <c r="L824" s="6" t="n"/>
+      <c r="O824" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="825">
       <c r="A825" s="21" t="n">
@@ -37113,6 +39406,11 @@
         </is>
       </c>
       <c r="L829" s="6" t="n"/>
+      <c r="O829" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="830">
       <c r="A830" s="21" t="n">
@@ -37153,6 +39451,11 @@
         </is>
       </c>
       <c r="L830" s="6" t="n"/>
+      <c r="O830" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="831">
       <c r="A831" s="21" t="n">
@@ -37285,6 +39588,11 @@
         </is>
       </c>
       <c r="L833" s="6" t="n"/>
+      <c r="O833" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="834">
       <c r="A834" s="21" t="n">
@@ -37409,6 +39717,11 @@
         </is>
       </c>
       <c r="L836" s="6" t="n"/>
+      <c r="O836" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="837">
       <c r="A837" s="21" t="n">
@@ -37449,6 +39762,11 @@
         </is>
       </c>
       <c r="L837" s="6" t="n"/>
+      <c r="O837" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="838">
       <c r="A838" s="21" t="n">
@@ -37489,6 +39807,11 @@
         </is>
       </c>
       <c r="L838" s="6" t="n"/>
+      <c r="O838" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="839">
       <c r="A839" s="21" t="n">
@@ -37609,6 +39932,11 @@
         </is>
       </c>
       <c r="L841" s="6" t="n"/>
+      <c r="O841" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="842">
       <c r="A842" s="21" t="n">
@@ -37649,6 +39977,11 @@
         </is>
       </c>
       <c r="L842" s="6" t="n"/>
+      <c r="O842" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="843">
       <c r="A843" s="21" t="n">
@@ -38097,6 +40430,11 @@
         </is>
       </c>
       <c r="L853" s="6" t="n"/>
+      <c r="O853" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="854">
       <c r="A854" s="21" t="n">
@@ -38217,6 +40555,11 @@
         </is>
       </c>
       <c r="L856" s="6" t="n"/>
+      <c r="O856" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="857">
       <c r="A857" s="21" t="n">
@@ -38257,6 +40600,11 @@
         </is>
       </c>
       <c r="L857" s="6" t="n"/>
+      <c r="O857" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="858">
       <c r="A858" s="21" t="n">
@@ -38297,6 +40645,11 @@
         </is>
       </c>
       <c r="L858" s="6" t="n"/>
+      <c r="O858" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="859">
       <c r="A859" s="21" t="n">
@@ -38337,6 +40690,11 @@
         </is>
       </c>
       <c r="L859" s="6" t="n"/>
+      <c r="O859" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="860">
       <c r="A860" s="21" t="n">
@@ -38377,6 +40735,11 @@
         </is>
       </c>
       <c r="L860" s="6" t="n"/>
+      <c r="O860" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="861">
       <c r="A861" s="21" t="n">
@@ -38417,6 +40780,11 @@
         </is>
       </c>
       <c r="L861" s="6" t="n"/>
+      <c r="O861" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="862">
       <c r="A862" s="21" t="n">
@@ -38457,6 +40825,11 @@
         </is>
       </c>
       <c r="L862" s="6" t="n"/>
+      <c r="O862" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="863">
       <c r="A863" s="21" t="n">
@@ -38497,6 +40870,11 @@
         </is>
       </c>
       <c r="L863" s="6" t="n"/>
+      <c r="O863" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="864">
       <c r="A864" s="21" t="n">
@@ -39293,6 +41671,11 @@
         </is>
       </c>
       <c r="L882" s="6" t="n"/>
+      <c r="O882" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="883">
       <c r="A883" s="21" t="n">
@@ -39373,6 +41756,11 @@
         </is>
       </c>
       <c r="L884" s="6" t="n"/>
+      <c r="O884" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="885">
       <c r="A885" s="21" t="n">
@@ -39413,6 +41801,11 @@
         </is>
       </c>
       <c r="L885" s="6" t="n"/>
+      <c r="O885" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
+        </is>
+      </c>
     </row>
     <row r="886">
       <c r="A886" s="21" t="n">
@@ -39700,7 +42093,7 @@
           <t>ONLINE PAYMENT</t>
         </is>
       </c>
-      <c r="B3" s="34" t="n"/>
+      <c r="B3" s="36" t="n"/>
       <c r="D3" s="18" t="n"/>
       <c r="E3" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix CHQ matching logic and remove wrong Pending/Old Account data
Bank Statement:
- CHQ number matching ONLY for 'CHQ PAID' narrations (not FT/UPI/NEFT)
  e.g. 'FT-DR-A V TRADERS 002617' was incorrectly matched - now fixed
- GPAY/UPI matching only for narrations with UPI/GPAY/NEFT keywords

System_Purchase:
- PAIDTRAN filter: only use BILLDATE >= 29-May-2025 (post-takeover)
- Unmatched bills (no payment): leave ALL columns blank (no Pending fill)
- Partial pay: only fill Pending when PURBALAMT > 0

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -1120,17 +1120,6 @@
         </is>
       </c>
       <c r="L7" s="28" t="n"/>
-      <c r="M7" s="33" t="inlineStr"/>
-      <c r="N7" s="33" t="inlineStr">
-        <is>
-          <t>AGARWAL &amp; COMPANY</t>
-        </is>
-      </c>
-      <c r="O7" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="8" customFormat="1" s="31">
       <c r="A8" s="29" t="n">
@@ -1173,17 +1162,6 @@
         </is>
       </c>
       <c r="L8" s="28" t="n"/>
-      <c r="M8" s="33" t="inlineStr"/>
-      <c r="N8" s="33" t="inlineStr">
-        <is>
-          <t>AGARWAL &amp; COMPANY</t>
-        </is>
-      </c>
-      <c r="O8" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="n">
@@ -1470,21 +1448,6 @@
         </is>
       </c>
       <c r="L14" s="28" t="n"/>
-      <c r="M14" s="33" t="inlineStr">
-        <is>
-          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
-        </is>
-      </c>
-      <c r="N14" s="33" t="inlineStr">
-        <is>
-          <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O14" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="15" customFormat="1" s="31">
       <c r="A15" s="29" t="n">
@@ -1527,21 +1490,6 @@
         </is>
       </c>
       <c r="L15" s="28" t="n"/>
-      <c r="M15" s="33" t="inlineStr">
-        <is>
-          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
-        </is>
-      </c>
-      <c r="N15" s="33" t="inlineStr">
-        <is>
-          <t>SENIOR AGENCY</t>
-        </is>
-      </c>
-      <c r="O15" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="n">
@@ -2095,17 +2043,6 @@
         </is>
       </c>
       <c r="L27" s="28" t="n"/>
-      <c r="M27" s="33" t="inlineStr"/>
-      <c r="N27" s="33" t="inlineStr">
-        <is>
-          <t>SHINDE ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O27" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="28" customFormat="1" s="31">
       <c r="A28" s="29" t="n">
@@ -2148,21 +2085,6 @@
         </is>
       </c>
       <c r="L28" s="28" t="n"/>
-      <c r="M28" s="33" t="inlineStr">
-        <is>
-          <t>2601</t>
-        </is>
-      </c>
-      <c r="N28" s="33" t="inlineStr">
-        <is>
-          <t>NANDINI BEAUTY</t>
-        </is>
-      </c>
-      <c r="O28" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="21" t="n">
@@ -2205,21 +2127,6 @@
         </is>
       </c>
       <c r="L29" s="6" t="n"/>
-      <c r="M29" s="33" t="inlineStr">
-        <is>
-          <t>317</t>
-        </is>
-      </c>
-      <c r="N29" s="33" t="inlineStr">
-        <is>
-          <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O29" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="21" t="n">
@@ -3422,21 +3329,6 @@
         </is>
       </c>
       <c r="L54" s="6" t="n"/>
-      <c r="M54" s="35" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="N54" s="35" t="inlineStr">
-        <is>
-          <t>HDFC BANK</t>
-        </is>
-      </c>
-      <c r="O54" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" s="21" t="n">
@@ -6147,21 +6039,6 @@
         </is>
       </c>
       <c r="L109" s="6" t="n"/>
-      <c r="M109" s="35" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="N109" s="35" t="inlineStr">
-        <is>
-          <t>HDFC BANK</t>
-        </is>
-      </c>
-      <c r="O109" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" s="21" t="n">
@@ -8007,21 +7884,6 @@
         </is>
       </c>
       <c r="L146" s="6" t="n"/>
-      <c r="M146" s="33" t="inlineStr">
-        <is>
-          <t>510</t>
-        </is>
-      </c>
-      <c r="N146" s="33" t="inlineStr">
-        <is>
-          <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O146" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" s="21" t="n">
@@ -8521,21 +8383,6 @@
         </is>
       </c>
       <c r="L156" s="6" t="n"/>
-      <c r="M156" s="33" t="inlineStr">
-        <is>
-          <t>466,555</t>
-        </is>
-      </c>
-      <c r="N156" s="33" t="inlineStr">
-        <is>
-          <t>DHANLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O156" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" s="21" t="n">
@@ -8578,21 +8425,6 @@
         </is>
       </c>
       <c r="L157" s="6" t="n"/>
-      <c r="M157" s="35" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="N157" s="35" t="inlineStr">
-        <is>
-          <t>HDFC BANK</t>
-        </is>
-      </c>
-      <c r="O157" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" s="21" t="n">
@@ -8765,17 +8597,6 @@
         </is>
       </c>
       <c r="L161" s="6" t="n"/>
-      <c r="M161" s="33" t="inlineStr"/>
-      <c r="N161" s="33" t="inlineStr">
-        <is>
-          <t>ROYAL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O161" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" s="21" t="n">
@@ -9413,17 +9234,6 @@
         </is>
       </c>
       <c r="L174" s="6" t="n"/>
-      <c r="M174" s="33" t="inlineStr"/>
-      <c r="N174" s="33" t="inlineStr">
-        <is>
-          <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O174" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" s="21" t="n">
@@ -9466,17 +9276,6 @@
         </is>
       </c>
       <c r="L175" s="6" t="n"/>
-      <c r="M175" s="33" t="inlineStr"/>
-      <c r="N175" s="33" t="inlineStr">
-        <is>
-          <t>KHAMANG BEST CHIWDA</t>
-        </is>
-      </c>
-      <c r="O175" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" s="21" t="n">
@@ -9750,17 +9549,6 @@
         </is>
       </c>
       <c r="L181" s="6" t="n"/>
-      <c r="M181" s="33" t="inlineStr"/>
-      <c r="N181" s="33" t="inlineStr">
-        <is>
-          <t>DHYAANI NEXUS PVT.LTD.</t>
-        </is>
-      </c>
-      <c r="O181" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" s="21" t="n">
@@ -12313,17 +12101,6 @@
         </is>
       </c>
       <c r="L235" s="6" t="n"/>
-      <c r="M235" s="33" t="inlineStr"/>
-      <c r="N235" s="33" t="inlineStr">
-        <is>
-          <t>RADIANT ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O235" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="236">
       <c r="A236" s="21" t="n">
@@ -13735,21 +13512,6 @@
         </is>
       </c>
       <c r="L264" s="6" t="n"/>
-      <c r="M264" s="33" t="inlineStr">
-        <is>
-          <t>513</t>
-        </is>
-      </c>
-      <c r="N264" s="33" t="inlineStr">
-        <is>
-          <t>MANGAL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O264" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="265">
       <c r="A265" s="21" t="n">
@@ -13980,17 +13742,6 @@
         </is>
       </c>
       <c r="L269" s="6" t="n"/>
-      <c r="M269" s="33" t="inlineStr"/>
-      <c r="N269" s="33" t="inlineStr">
-        <is>
-          <t>SHREE GANESH ENTERPISES</t>
-        </is>
-      </c>
-      <c r="O269" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="270">
       <c r="A270" s="21" t="n">
@@ -14233,17 +13984,6 @@
         </is>
       </c>
       <c r="L274" s="6" t="n"/>
-      <c r="M274" s="33" t="inlineStr"/>
-      <c r="N274" s="33" t="inlineStr">
-        <is>
-          <t>RAJLAXMI ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O274" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="275">
       <c r="A275" s="21" t="n">
@@ -16340,15 +16080,9 @@
         </is>
       </c>
       <c r="L319" s="6" t="n"/>
-      <c r="M319" s="35" t="inlineStr"/>
-      <c r="N319" s="35" t="inlineStr">
-        <is>
-          <t>SHUBH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O319" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
+      <c r="O319" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
         </is>
       </c>
     </row>
@@ -17362,21 +17096,6 @@
         </is>
       </c>
       <c r="L341" s="6" t="n"/>
-      <c r="M341" s="33" t="inlineStr">
-        <is>
-          <t>174</t>
-        </is>
-      </c>
-      <c r="N341" s="33" t="inlineStr">
-        <is>
-          <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O341" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="342">
       <c r="A342" s="21" t="n">
@@ -19193,15 +18912,9 @@
         </is>
       </c>
       <c r="L381" s="6" t="n"/>
-      <c r="M381" s="35" t="inlineStr"/>
-      <c r="N381" s="35" t="inlineStr">
-        <is>
-          <t>SUMEET AGENCIES</t>
-        </is>
-      </c>
-      <c r="O381" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
+      <c r="O381" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
         </is>
       </c>
     </row>
@@ -19335,17 +19048,6 @@
         </is>
       </c>
       <c r="L384" s="6" t="n"/>
-      <c r="M384" s="33" t="inlineStr"/>
-      <c r="N384" s="33" t="inlineStr">
-        <is>
-          <t>SHREE GANESH ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O384" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="385">
       <c r="A385" s="21" t="n">
@@ -21326,21 +21028,6 @@
         </is>
       </c>
       <c r="L427" s="6" t="n"/>
-      <c r="M427" s="33" t="inlineStr">
-        <is>
-          <t>174</t>
-        </is>
-      </c>
-      <c r="N427" s="33" t="inlineStr">
-        <is>
-          <t>3P'S ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O427" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="428">
       <c r="A428" s="21" t="n">
@@ -21706,17 +21393,6 @@
         </is>
       </c>
       <c r="L435" s="6" t="n"/>
-      <c r="M435" s="33" t="inlineStr"/>
-      <c r="N435" s="33" t="inlineStr">
-        <is>
-          <t>HEALTH PLUS MEDICO</t>
-        </is>
-      </c>
-      <c r="O435" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="436">
       <c r="A436" s="21" t="n">
@@ -23834,21 +23510,6 @@
         </is>
       </c>
       <c r="L482" s="6" t="n"/>
-      <c r="M482" s="35" t="inlineStr">
-        <is>
-          <t>488</t>
-        </is>
-      </c>
-      <c r="N482" s="35" t="inlineStr">
-        <is>
-          <t>DHANVANTARI SALES</t>
-        </is>
-      </c>
-      <c r="O482" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="483">
       <c r="A483" s="21" t="n">
@@ -24866,17 +24527,6 @@
         </is>
       </c>
       <c r="L505" s="6" t="n"/>
-      <c r="M505" s="33" t="inlineStr"/>
-      <c r="N505" s="33" t="inlineStr">
-        <is>
-          <t>DHYAANI NEXUS PVT.LTD.</t>
-        </is>
-      </c>
-      <c r="O505" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="506">
       <c r="A506" s="21" t="n">
@@ -25293,17 +24943,6 @@
         </is>
       </c>
       <c r="L514" s="6" t="n"/>
-      <c r="M514" s="33" t="inlineStr"/>
-      <c r="N514" s="33" t="inlineStr">
-        <is>
-          <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O514" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="515">
       <c r="A515" s="21" t="n">
@@ -26774,17 +26413,6 @@
         </is>
       </c>
       <c r="L546" s="6" t="n"/>
-      <c r="M546" s="33" t="inlineStr"/>
-      <c r="N546" s="33" t="inlineStr">
-        <is>
-          <t>ATUL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O546" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="547">
       <c r="A547" s="21" t="n">
@@ -27502,17 +27130,6 @@
         </is>
       </c>
       <c r="L563" s="6" t="n"/>
-      <c r="M563" s="33" t="inlineStr"/>
-      <c r="N563" s="33" t="inlineStr">
-        <is>
-          <t>SARA MARKETING</t>
-        </is>
-      </c>
-      <c r="O563" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="564">
       <c r="A564" s="21" t="n">
@@ -29312,17 +28929,6 @@
         </is>
       </c>
       <c r="L603" s="6" t="n"/>
-      <c r="M603" s="33" t="inlineStr"/>
-      <c r="N603" s="33" t="inlineStr">
-        <is>
-          <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O603" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="604">
       <c r="A604" s="21" t="n">
@@ -29363,17 +28969,6 @@
         </is>
       </c>
       <c r="L604" s="6" t="n"/>
-      <c r="M604" s="33" t="inlineStr"/>
-      <c r="N604" s="33" t="inlineStr">
-        <is>
-          <t>M/S MANDAR AGENCY</t>
-        </is>
-      </c>
-      <c r="O604" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="605">
       <c r="A605" s="21" t="n">
@@ -32581,17 +32176,6 @@
         </is>
       </c>
       <c r="L677" s="6" t="n"/>
-      <c r="M677" s="33" t="inlineStr"/>
-      <c r="N677" s="33" t="inlineStr">
-        <is>
-          <t>R M ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O677" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="678">
       <c r="A678" s="21" t="n">
@@ -32632,17 +32216,6 @@
         </is>
       </c>
       <c r="L678" s="6" t="n"/>
-      <c r="M678" s="33" t="inlineStr"/>
-      <c r="N678" s="33" t="inlineStr">
-        <is>
-          <t>ATUL ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O678" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="679">
       <c r="A679" s="21" t="n">
@@ -33523,21 +33096,6 @@
         </is>
       </c>
       <c r="L698" s="6" t="n"/>
-      <c r="M698" s="33" t="inlineStr">
-        <is>
-          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
-        </is>
-      </c>
-      <c r="N698" s="33" t="inlineStr">
-        <is>
-          <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O698" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="699">
       <c r="A699" s="21" t="n">
@@ -33578,21 +33136,6 @@
         </is>
       </c>
       <c r="L699" s="6" t="n"/>
-      <c r="M699" s="33" t="inlineStr">
-        <is>
-          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
-        </is>
-      </c>
-      <c r="N699" s="33" t="inlineStr">
-        <is>
-          <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O699" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="700">
       <c r="A700" s="21" t="n">
@@ -33952,17 +33495,6 @@
         </is>
       </c>
       <c r="L707" s="6" t="n"/>
-      <c r="M707" s="33" t="inlineStr"/>
-      <c r="N707" s="33" t="inlineStr">
-        <is>
-          <t>AV TRADERS</t>
-        </is>
-      </c>
-      <c r="O707" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="708">
       <c r="A708" s="21" t="n">
@@ -34845,19 +34377,9 @@
         </is>
       </c>
       <c r="L726" s="6" t="n"/>
-      <c r="M726" s="35" t="inlineStr">
-        <is>
-          <t>201,199</t>
-        </is>
-      </c>
-      <c r="N726" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O726" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
+      <c r="O726" s="34" t="inlineStr">
+        <is>
+          <t>NOT_IN_SYSTEM</t>
         </is>
       </c>
     </row>
@@ -35123,11 +34645,6 @@
         </is>
       </c>
       <c r="L732" s="6" t="n"/>
-      <c r="O732" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="733">
       <c r="A733" s="21" t="n">
@@ -35168,11 +34685,6 @@
         </is>
       </c>
       <c r="L733" s="6" t="n"/>
-      <c r="O733" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="734">
       <c r="A734" s="21" t="n">
@@ -36905,21 +36417,6 @@
         </is>
       </c>
       <c r="L772" s="6" t="n"/>
-      <c r="M772" s="33" t="inlineStr">
-        <is>
-          <t>518,543,575,576,569,573,581,603,624,645,702,772,842,851,903,921,939</t>
-        </is>
-      </c>
-      <c r="N772" s="33" t="inlineStr">
-        <is>
-          <t>MEDIRAJ DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O772" s="33" t="inlineStr">
-        <is>
-          <t>CHQ_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="773">
       <c r="A773" s="21" t="n">
@@ -40645,11 +40142,6 @@
         </is>
       </c>
       <c r="L858" s="6" t="n"/>
-      <c r="O858" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="859">
       <c r="A859" s="21" t="n">
@@ -40690,11 +40182,6 @@
         </is>
       </c>
       <c r="L859" s="6" t="n"/>
-      <c r="O859" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="860">
       <c r="A860" s="21" t="n">
@@ -40780,11 +40267,6 @@
         </is>
       </c>
       <c r="L861" s="6" t="n"/>
-      <c r="O861" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="862">
       <c r="A862" s="21" t="n">
@@ -40825,11 +40307,6 @@
         </is>
       </c>
       <c r="L862" s="6" t="n"/>
-      <c r="O862" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="863">
       <c r="A863" s="21" t="n">
@@ -41756,11 +41233,6 @@
         </is>
       </c>
       <c r="L884" s="6" t="n"/>
-      <c r="O884" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="885">
       <c r="A885" s="21" t="n">
@@ -41801,11 +41273,6 @@
         </is>
       </c>
       <c r="L885" s="6" t="n"/>
-      <c r="O885" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="886">
       <c r="A886" s="21" t="n">

</xml_diff>

<commit_message>
Rewrite: clean reconciliation logic from scratch
Flow:
1. Join ACCOUNT+PAIDMAST+PAIDTRAN -> DBF_Joined_Data.xlsx
2. Scan bank statement CHQ PAID narrations -> build confirmed CHQ set (144 matched)
3. System_Purchase per Vou.No. (PAIDTRAN.PURVCHNO, BILLDATE >= 29-May-2025):
   - CHQ found in bank (CHQ PAID) -> Date, ChQ No., Old Account = PURPAIDAMT
   - CHQ NOT in bank              -> Pending = invoice Amount
   - No payment at all            -> leave blank
   Old Account = ONLY bank-confirmed entries, nothing else.
4. Bank: FT/UPI/NEFT narrations NOT matched via CHQ number (avoids false positives)

Result: OldAccount=Rs3.3L (116 bills), Pending=Rs5L (212 bills)

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -68,7 +68,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -109,12 +109,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2CFEF"/>
-        <bgColor rgb="00E2CFEF"/>
       </patternFill>
     </fill>
   </fills>
@@ -286,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -350,7 +344,6 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2169,21 +2162,6 @@
         </is>
       </c>
       <c r="L30" s="6" t="n"/>
-      <c r="M30" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N30" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O30" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="n">
@@ -2578,21 +2556,6 @@
         </is>
       </c>
       <c r="L39" s="6" t="n"/>
-      <c r="M39" s="35" t="inlineStr">
-        <is>
-          <t>327,344</t>
-        </is>
-      </c>
-      <c r="N39" s="35" t="inlineStr">
-        <is>
-          <t>PRIME DITRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O39" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
@@ -2635,21 +2598,6 @@
         </is>
       </c>
       <c r="L40" s="6" t="n"/>
-      <c r="M40" s="35" t="inlineStr">
-        <is>
-          <t>293,298,307,319</t>
-        </is>
-      </c>
-      <c r="N40" s="35" t="inlineStr">
-        <is>
-          <t>JM PHARMA</t>
-        </is>
-      </c>
-      <c r="O40" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
@@ -3028,21 +2976,6 @@
         </is>
       </c>
       <c r="L48" s="6" t="n"/>
-      <c r="M48" s="35" t="inlineStr">
-        <is>
-          <t>256</t>
-        </is>
-      </c>
-      <c r="N48" s="35" t="inlineStr">
-        <is>
-          <t>HDFC BANK</t>
-        </is>
-      </c>
-      <c r="O48" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" s="21" t="n">
@@ -3085,21 +3018,6 @@
         </is>
       </c>
       <c r="L49" s="6" t="n"/>
-      <c r="M49" s="35" t="inlineStr">
-        <is>
-          <t>334,347,357,379,390,391,402,414,428,435,446</t>
-        </is>
-      </c>
-      <c r="N49" s="35" t="inlineStr">
-        <is>
-          <t>JM PHARMA</t>
-        </is>
-      </c>
-      <c r="O49" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="n">
@@ -3371,21 +3289,6 @@
         </is>
       </c>
       <c r="L55" s="6" t="n"/>
-      <c r="M55" s="35" t="inlineStr">
-        <is>
-          <t>475</t>
-        </is>
-      </c>
-      <c r="N55" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O55" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="n">
@@ -3843,21 +3746,6 @@
         </is>
       </c>
       <c r="L64" s="6" t="n"/>
-      <c r="M64" s="35" t="inlineStr">
-        <is>
-          <t>480</t>
-        </is>
-      </c>
-      <c r="N64" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O64" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="n">
@@ -4155,21 +4043,6 @@
         </is>
       </c>
       <c r="L70" s="6" t="n"/>
-      <c r="M70" s="35" t="inlineStr">
-        <is>
-          <t>42,180,235,189,253,259</t>
-        </is>
-      </c>
-      <c r="N70" s="35" t="inlineStr">
-        <is>
-          <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O70" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" s="21" t="n">
@@ -5046,21 +4919,6 @@
         </is>
       </c>
       <c r="L89" s="6" t="n"/>
-      <c r="M89" s="35" t="inlineStr">
-        <is>
-          <t>508</t>
-        </is>
-      </c>
-      <c r="N89" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O89" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="n">
@@ -5642,21 +5500,6 @@
         </is>
       </c>
       <c r="L101" s="6" t="n"/>
-      <c r="M101" s="35" t="inlineStr">
-        <is>
-          <t>488</t>
-        </is>
-      </c>
-      <c r="N101" s="35" t="inlineStr">
-        <is>
-          <t>DHANVANTARI SALES</t>
-        </is>
-      </c>
-      <c r="O101" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" s="21" t="n">
@@ -5699,21 +5542,6 @@
         </is>
       </c>
       <c r="L102" s="6" t="n"/>
-      <c r="M102" s="35" t="inlineStr">
-        <is>
-          <t>531</t>
-        </is>
-      </c>
-      <c r="N102" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O102" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" s="21" t="n">
@@ -5982,21 +5810,6 @@
         </is>
       </c>
       <c r="L108" s="6" t="n"/>
-      <c r="M108" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N108" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O108" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="21" t="n">
@@ -6473,21 +6286,6 @@
         </is>
       </c>
       <c r="L118" s="6" t="n"/>
-      <c r="M118" s="35" t="inlineStr">
-        <is>
-          <t>567,549</t>
-        </is>
-      </c>
-      <c r="N118" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O118" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" s="21" t="n">
@@ -6572,21 +6370,6 @@
         </is>
       </c>
       <c r="L120" s="6" t="n"/>
-      <c r="M120" s="35" t="inlineStr">
-        <is>
-          <t>484,464,469,487,506,522</t>
-        </is>
-      </c>
-      <c r="N120" s="35" t="inlineStr">
-        <is>
-          <t>VARDAAN DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O120" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" s="21" t="n">
@@ -6675,21 +6458,6 @@
         </is>
       </c>
       <c r="L122" s="6" t="n"/>
-      <c r="M122" s="35" t="inlineStr">
-        <is>
-          <t>689</t>
-        </is>
-      </c>
-      <c r="N122" s="35" t="inlineStr">
-        <is>
-          <t>SUPARSHWA MEDCARE LLP</t>
-        </is>
-      </c>
-      <c r="O122" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" s="21" t="n">
@@ -6877,21 +6645,6 @@
         </is>
       </c>
       <c r="L126" s="6" t="n"/>
-      <c r="M126" s="35" t="inlineStr">
-        <is>
-          <t>523</t>
-        </is>
-      </c>
-      <c r="N126" s="35" t="inlineStr">
-        <is>
-          <t>ABHAY PHARMA</t>
-        </is>
-      </c>
-      <c r="O126" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" s="21" t="n">
@@ -6934,21 +6687,6 @@
         </is>
       </c>
       <c r="L127" s="6" t="n"/>
-      <c r="M127" s="35" t="inlineStr">
-        <is>
-          <t>478</t>
-        </is>
-      </c>
-      <c r="N127" s="35" t="inlineStr">
-        <is>
-          <t>PRIME AYURVED</t>
-        </is>
-      </c>
-      <c r="O127" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" s="21" t="n">
@@ -6991,21 +6729,6 @@
         </is>
       </c>
       <c r="L128" s="6" t="n"/>
-      <c r="M128" s="35" t="inlineStr">
-        <is>
-          <t>42,180,235,189,253,259</t>
-        </is>
-      </c>
-      <c r="N128" s="35" t="inlineStr">
-        <is>
-          <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O128" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" s="21" t="n">
@@ -7224,21 +6947,6 @@
         </is>
       </c>
       <c r="L133" s="6" t="n"/>
-      <c r="M133" s="35" t="inlineStr">
-        <is>
-          <t>578,577</t>
-        </is>
-      </c>
-      <c r="N133" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O133" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" s="21" t="n">
@@ -7377,21 +7085,6 @@
           <t>salary</t>
         </is>
       </c>
-      <c r="M136" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N136" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O136" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" s="21" t="n">
@@ -7968,21 +7661,6 @@
         </is>
       </c>
       <c r="L148" s="6" t="n"/>
-      <c r="M148" s="35" t="inlineStr">
-        <is>
-          <t>597</t>
-        </is>
-      </c>
-      <c r="N148" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O148" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" s="21" t="n">
@@ -8328,12 +8006,12 @@
       <c r="L155" s="6" t="n"/>
       <c r="M155" s="33" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>256,256</t>
         </is>
       </c>
       <c r="N155" s="33" t="inlineStr">
         <is>
-          <t>SHREE DATTA KRUPA AGENCY</t>
+          <t>SHREE DATTA KRUPA AGENCY / HDFC BANK</t>
         </is>
       </c>
       <c r="O155" s="33" t="inlineStr">
@@ -8960,21 +8638,6 @@
         </is>
       </c>
       <c r="L169" s="6" t="n"/>
-      <c r="M169" s="35" t="inlineStr">
-        <is>
-          <t>583,596,607</t>
-        </is>
-      </c>
-      <c r="N169" s="35" t="inlineStr">
-        <is>
-          <t>VARDAAN DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O169" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" s="21" t="n">
@@ -9725,21 +9388,6 @@
         </is>
       </c>
       <c r="L185" s="6" t="n"/>
-      <c r="M185" s="35" t="inlineStr">
-        <is>
-          <t>612</t>
-        </is>
-      </c>
-      <c r="N185" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O185" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" s="21" t="n">
@@ -10535,21 +10183,6 @@
         </is>
       </c>
       <c r="L203" s="6" t="n"/>
-      <c r="M203" s="35" t="inlineStr">
-        <is>
-          <t>629,630</t>
-        </is>
-      </c>
-      <c r="N203" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O203" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="204">
       <c r="A204" s="21" t="n">
@@ -10736,21 +10369,6 @@
         </is>
       </c>
       <c r="L207" s="6" t="n"/>
-      <c r="M207" s="35" t="inlineStr">
-        <is>
-          <t>638</t>
-        </is>
-      </c>
-      <c r="N207" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O207" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="208">
       <c r="A208" s="21" t="n">
@@ -10877,21 +10495,6 @@
         </is>
       </c>
       <c r="L210" s="6" t="n"/>
-      <c r="M210" s="35" t="inlineStr">
-        <is>
-          <t>472,467,481,505,525,532,546,548,586,592,606</t>
-        </is>
-      </c>
-      <c r="N210" s="35" t="inlineStr">
-        <is>
-          <t>JM PHARMA</t>
-        </is>
-      </c>
-      <c r="O210" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="211">
       <c r="A211" s="21" t="n">
@@ -11160,21 +10763,6 @@
         </is>
       </c>
       <c r="L216" s="6" t="n"/>
-      <c r="M216" s="35" t="inlineStr">
-        <is>
-          <t>651</t>
-        </is>
-      </c>
-      <c r="N216" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O216" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="217">
       <c r="A217" s="21" t="n">
@@ -11301,21 +10889,6 @@
         </is>
       </c>
       <c r="L219" s="6" t="n"/>
-      <c r="M219" s="35" t="inlineStr">
-        <is>
-          <t>216,221,234,244,265,292,301,305,308,324,333,349,363,362,372,389,393,400,418,429,437</t>
-        </is>
-      </c>
-      <c r="N219" s="35" t="inlineStr">
-        <is>
-          <t>JEEVAN MEDISALES PVT LTD</t>
-        </is>
-      </c>
-      <c r="O219" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="220">
       <c r="A220" s="21" t="n">
@@ -11746,21 +11319,6 @@
         </is>
       </c>
       <c r="L228" s="6" t="n"/>
-      <c r="M228" s="35" t="inlineStr">
-        <is>
-          <t>471,474,479,485,507,524,533,553,570</t>
-        </is>
-      </c>
-      <c r="N228" s="35" t="inlineStr">
-        <is>
-          <t>JEEVAN MEDISALES PVT LTD</t>
-        </is>
-      </c>
-      <c r="O228" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="229">
       <c r="A229" s="21" t="n">
@@ -12002,21 +11560,6 @@
         </is>
       </c>
       <c r="L233" s="6" t="n"/>
-      <c r="M233" s="35" t="inlineStr">
-        <is>
-          <t>670,673</t>
-        </is>
-      </c>
-      <c r="N233" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O233" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="234">
       <c r="A234" s="21" t="n">
@@ -12235,21 +11778,6 @@
         </is>
       </c>
       <c r="L238" s="6" t="n"/>
-      <c r="M238" s="35" t="inlineStr">
-        <is>
-          <t>126,127,133,151,179,189,209,240,246,258,303,337,411,355,364,376,415,425</t>
-        </is>
-      </c>
-      <c r="N238" s="35" t="inlineStr">
-        <is>
-          <t>D.K. ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O238" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="239">
       <c r="A239" s="21" t="n">
@@ -12292,21 +11820,6 @@
         </is>
       </c>
       <c r="L239" s="6" t="n"/>
-      <c r="M239" s="35" t="inlineStr">
-        <is>
-          <t>504,538,551,566,609,633,644</t>
-        </is>
-      </c>
-      <c r="N239" s="35" t="inlineStr">
-        <is>
-          <t>D.K. ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O239" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="240">
       <c r="A240" s="21" t="n">
@@ -12760,17 +12273,6 @@
         </is>
       </c>
       <c r="L249" s="6" t="n"/>
-      <c r="M249" s="35" t="inlineStr"/>
-      <c r="N249" s="35" t="inlineStr">
-        <is>
-          <t>MSEDCL  -----------X----------</t>
-        </is>
-      </c>
-      <c r="O249" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="250">
       <c r="A250" s="21" t="n">
@@ -12813,21 +12315,6 @@
         </is>
       </c>
       <c r="L250" s="6" t="n"/>
-      <c r="M250" s="35" t="inlineStr">
-        <is>
-          <t>671,692,657,672,691,690</t>
-        </is>
-      </c>
-      <c r="N250" s="35" t="inlineStr">
-        <is>
-          <t>VARDAAN DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O250" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="251">
       <c r="A251" s="21" t="n">
@@ -13310,21 +12797,6 @@
         </is>
       </c>
       <c r="L260" s="6" t="n"/>
-      <c r="M260" s="35" t="inlineStr">
-        <is>
-          <t>610</t>
-        </is>
-      </c>
-      <c r="N260" s="35" t="inlineStr">
-        <is>
-          <t>DHANWANTRI PHARMA</t>
-        </is>
-      </c>
-      <c r="O260" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="261">
       <c r="A261" s="21" t="n">
@@ -13365,21 +12837,6 @@
         </is>
       </c>
       <c r="L261" s="6" t="n"/>
-      <c r="M261" s="35" t="inlineStr">
-        <is>
-          <t>682,705</t>
-        </is>
-      </c>
-      <c r="N261" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O261" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="262">
       <c r="A262" s="21" t="n">
@@ -13782,21 +13239,6 @@
         </is>
       </c>
       <c r="L270" s="6" t="n"/>
-      <c r="M270" s="35" t="inlineStr">
-        <is>
-          <t>719</t>
-        </is>
-      </c>
-      <c r="N270" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O270" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="271">
       <c r="A271" s="21" t="n">
@@ -14906,21 +14348,6 @@
         </is>
       </c>
       <c r="L293" s="6" t="n"/>
-      <c r="M293" s="35" t="inlineStr">
-        <is>
-          <t>42,180,235,189,253,259</t>
-        </is>
-      </c>
-      <c r="N293" s="35" t="inlineStr">
-        <is>
-          <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O293" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="294">
       <c r="A294" s="21" t="n">
@@ -15404,17 +14831,6 @@
         </is>
       </c>
       <c r="L304" s="6" t="n"/>
-      <c r="M304" s="35" t="inlineStr"/>
-      <c r="N304" s="35" t="inlineStr">
-        <is>
-          <t>KAPILA PASHU AUSHADHALAYA</t>
-        </is>
-      </c>
-      <c r="O304" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="305">
       <c r="A305" s="21" t="n">
@@ -15455,21 +14871,6 @@
         </is>
       </c>
       <c r="L305" s="6" t="n"/>
-      <c r="M305" s="35" t="inlineStr">
-        <is>
-          <t>689</t>
-        </is>
-      </c>
-      <c r="N305" s="35" t="inlineStr">
-        <is>
-          <t>SUPARSHWA MEDCARE LLP</t>
-        </is>
-      </c>
-      <c r="O305" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="306">
       <c r="A306" s="21" t="n">
@@ -15634,21 +15035,6 @@
         </is>
       </c>
       <c r="L309" s="6" t="n"/>
-      <c r="M309" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N309" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O309" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="310">
       <c r="A310" s="21" t="n">
@@ -16125,21 +15511,6 @@
         </is>
       </c>
       <c r="L320" s="6" t="n"/>
-      <c r="M320" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N320" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O320" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="321" customFormat="1" s="2">
       <c r="A321" s="22" t="n">
@@ -17397,21 +16768,6 @@
         </is>
       </c>
       <c r="L348" s="6" t="n"/>
-      <c r="M348" s="35" t="inlineStr">
-        <is>
-          <t>497,656</t>
-        </is>
-      </c>
-      <c r="N348" s="35" t="inlineStr">
-        <is>
-          <t>SHREYAA AGENCIES</t>
-        </is>
-      </c>
-      <c r="O348" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="349">
       <c r="A349" s="21" t="n">
@@ -18449,7 +17805,7 @@
       <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
-          <t>G K ENTERPRISES</t>
+          <t>CG MARKETING PVT LTD / G K ENTERPRISES</t>
         </is>
       </c>
       <c r="O371" s="33" t="inlineStr">
@@ -18670,21 +18026,6 @@
         </is>
       </c>
       <c r="L376" s="6" t="n"/>
-      <c r="M376" s="35" t="inlineStr">
-        <is>
-          <t>804,753,805,770</t>
-        </is>
-      </c>
-      <c r="N376" s="35" t="inlineStr">
-        <is>
-          <t>VARDAAN DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O376" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="377">
       <c r="A377" s="21" t="n">
@@ -20039,7 +19380,7 @@
       <c r="M405" s="33" t="inlineStr"/>
       <c r="N405" s="33" t="inlineStr">
         <is>
-          <t>SHREYAA AGENCIES</t>
+          <t>SHREYAA AGENCIES / DHANLAXMI ENTERPRISES</t>
         </is>
       </c>
       <c r="O405" s="33" t="inlineStr">
@@ -20516,21 +19857,6 @@
         </is>
       </c>
       <c r="L416" s="6" t="n"/>
-      <c r="M416" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N416" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O416" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="417">
       <c r="A417" s="21" t="n">
@@ -21906,21 +21232,6 @@
         </is>
       </c>
       <c r="L446" s="6" t="n"/>
-      <c r="M446" s="35" t="inlineStr">
-        <is>
-          <t>623,632,640,648,661,676,687,707,722,728,736,744,750,758,774,783,807,818,857,875,894,902,909,925,934,941</t>
-        </is>
-      </c>
-      <c r="N446" s="35" t="inlineStr">
-        <is>
-          <t>JM PHARMA</t>
-        </is>
-      </c>
-      <c r="O446" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="447">
       <c r="A447" s="21" t="n">
@@ -22354,21 +21665,6 @@
         </is>
       </c>
       <c r="L456" s="6" t="n"/>
-      <c r="M456" s="35" t="inlineStr">
-        <is>
-          <t>477,678,776,869,960</t>
-        </is>
-      </c>
-      <c r="N456" s="35" t="inlineStr">
-        <is>
-          <t>PRIME DITRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O456" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="457">
       <c r="A457" s="21" t="n">
@@ -23331,21 +22627,6 @@
         </is>
       </c>
       <c r="L478" s="6" t="n"/>
-      <c r="M478" s="35" t="inlineStr">
-        <is>
-          <t>585,593,594,605,620,631,642,647,658,679,686,706,729,742,752,759,760,775,785,799,808,817,819,828,840,858,878,893,905,922,937,942</t>
-        </is>
-      </c>
-      <c r="N478" s="35" t="inlineStr">
-        <is>
-          <t>JEEVAN MEDISALES PVT LTD</t>
-        </is>
-      </c>
-      <c r="O478" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="479">
       <c r="A479" s="21" t="n">
@@ -24189,21 +23470,6 @@
         </is>
       </c>
       <c r="L498" s="6" t="n"/>
-      <c r="M498" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N498" s="35" t="inlineStr">
-        <is>
-          <t>VARDAAN DISTRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O498" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="499">
       <c r="A499" s="21" t="n">
@@ -25912,21 +25178,6 @@
         </is>
       </c>
       <c r="L535" s="6" t="n"/>
-      <c r="M535" s="35" t="inlineStr">
-        <is>
-          <t>2359,680,683,684,704,726,735,741,746,751,763,789,796,824,829,843,853,874,887,906,910,933</t>
-        </is>
-      </c>
-      <c r="N535" s="35" t="inlineStr">
-        <is>
-          <t>D.K. ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O535" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="536">
       <c r="A536" s="21" t="n">
@@ -26011,21 +25262,6 @@
           <t>salary</t>
         </is>
       </c>
-      <c r="M537" s="35" t="inlineStr">
-        <is>
-          <t>2954</t>
-        </is>
-      </c>
-      <c r="N537" s="35" t="inlineStr">
-        <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
-        </is>
-      </c>
-      <c r="O537" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="538">
       <c r="A538" s="21" t="n">
@@ -27452,21 +26688,6 @@
         </is>
       </c>
       <c r="L570" s="6" t="n"/>
-      <c r="M570" s="35" t="inlineStr">
-        <is>
-          <t>700</t>
-        </is>
-      </c>
-      <c r="N570" s="35" t="inlineStr">
-        <is>
-          <t>NAVMAHARASTRA ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="O570" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="571">
       <c r="A571" s="21" t="n">
@@ -29148,7 +28369,7 @@
       <c r="M608" s="33" t="inlineStr"/>
       <c r="N608" s="33" t="inlineStr">
         <is>
-          <t>M/S MANDAR AGENCY</t>
+          <t>SONIGARA DISTRIBUTOR / M/S MANDAR AGENCY</t>
         </is>
       </c>
       <c r="O608" s="33" t="inlineStr">
@@ -29236,21 +28457,6 @@
         </is>
       </c>
       <c r="L610" s="6" t="n"/>
-      <c r="M610" s="35" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="N610" s="35" t="inlineStr">
-        <is>
-          <t>LOCAL PURCHASE</t>
-        </is>
-      </c>
-      <c r="O610" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="611">
       <c r="A611" s="21" t="n">
@@ -30909,21 +30115,6 @@
         </is>
       </c>
       <c r="L648" s="6" t="n"/>
-      <c r="M648" s="35" t="inlineStr">
-        <is>
-          <t>949,957,969,980,987,1006,1011,1023,1032,1039,1053,1068,1076,1106</t>
-        </is>
-      </c>
-      <c r="N648" s="35" t="inlineStr">
-        <is>
-          <t>JM PHARMA</t>
-        </is>
-      </c>
-      <c r="O648" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="649">
       <c r="A649" s="21" t="n">
@@ -31048,21 +30239,6 @@
         </is>
       </c>
       <c r="L651" s="6" t="n"/>
-      <c r="M651" s="35" t="inlineStr">
-        <is>
-          <t>1083,1108,1128</t>
-        </is>
-      </c>
-      <c r="N651" s="35" t="inlineStr">
-        <is>
-          <t>PRIME DITRIBUTORS</t>
-        </is>
-      </c>
-      <c r="O651" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="652">
       <c r="A652" s="21" t="n">
@@ -35270,21 +34446,6 @@
         </is>
       </c>
       <c r="L746" s="6" t="n"/>
-      <c r="M746" s="35" t="inlineStr">
-        <is>
-          <t>42,180,235,189,253,259</t>
-        </is>
-      </c>
-      <c r="N746" s="35" t="inlineStr">
-        <is>
-          <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O746" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="747">
       <c r="A747" s="21" t="n">
@@ -37674,21 +36835,6 @@
         </is>
       </c>
       <c r="L801" s="6" t="n"/>
-      <c r="M801" s="35" t="inlineStr">
-        <is>
-          <t>42,180,235,189,253,259</t>
-        </is>
-      </c>
-      <c r="N801" s="35" t="inlineStr">
-        <is>
-          <t>YASHVI AGENCIES</t>
-        </is>
-      </c>
-      <c r="O801" s="35" t="inlineStr">
-        <is>
-          <t>GPAY_AMT_MATCHED</t>
-        </is>
-      </c>
     </row>
     <row r="802">
       <c r="A802" s="21" t="n">
@@ -41560,7 +40706,7 @@
           <t>ONLINE PAYMENT</t>
         </is>
       </c>
-      <c r="B3" s="36" t="n"/>
+      <c r="B3" s="35" t="n"/>
       <c r="D3" s="18" t="n"/>
       <c r="E3" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Re-run reconciliation on updated System_Purchase (b2600ff)
https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -8011,7 +8011,7 @@
       </c>
       <c r="N155" s="33" t="inlineStr">
         <is>
-          <t>SHREE DATTA KRUPA AGENCY / HDFC BANK</t>
+          <t>HDFC BANK / SHREE DATTA KRUPA AGENCY</t>
         </is>
       </c>
       <c r="O155" s="33" t="inlineStr">
@@ -17805,7 +17805,7 @@
       <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
-          <t>CG MARKETING PVT LTD / G K ENTERPRISES</t>
+          <t>G K ENTERPRISES / CG MARKETING PVT LTD</t>
         </is>
       </c>
       <c r="O371" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Write GPAY matches in Bank Statement with Voucher_No and Party_Name
- Bank Statement now shows GPAY_MATCHED (purple) for 49 UPI/GPAY rows
- Amount-based matching kept as last resort after CHQ matching
- CHQ_MATCHED: 144, GPAY_MATCHED: 49, NOT_IN_SYSTEM: 104

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -68,7 +68,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +109,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9B3FF"/>
+        <bgColor rgb="00D9B3FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -280,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -345,6 +351,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2162,6 +2169,21 @@
         </is>
       </c>
       <c r="L30" s="6" t="n"/>
+      <c r="M30" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N30" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O30" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="n">
@@ -2556,6 +2578,21 @@
         </is>
       </c>
       <c r="L39" s="6" t="n"/>
+      <c r="M39" s="36" t="inlineStr">
+        <is>
+          <t>327,344</t>
+        </is>
+      </c>
+      <c r="N39" s="36" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O39" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
@@ -2598,6 +2635,21 @@
         </is>
       </c>
       <c r="L40" s="6" t="n"/>
+      <c r="M40" s="36" t="inlineStr">
+        <is>
+          <t>293,298,307,319</t>
+        </is>
+      </c>
+      <c r="N40" s="36" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O40" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
@@ -3018,6 +3070,21 @@
         </is>
       </c>
       <c r="L49" s="6" t="n"/>
+      <c r="M49" s="36" t="inlineStr">
+        <is>
+          <t>334,347,357,379,390,391,402,414,428,435,446</t>
+        </is>
+      </c>
+      <c r="N49" s="36" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O49" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="21" t="n">
@@ -3289,6 +3356,21 @@
         </is>
       </c>
       <c r="L55" s="6" t="n"/>
+      <c r="M55" s="36" t="inlineStr">
+        <is>
+          <t>475</t>
+        </is>
+      </c>
+      <c r="N55" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O55" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="21" t="n">
@@ -3746,6 +3828,21 @@
         </is>
       </c>
       <c r="L64" s="6" t="n"/>
+      <c r="M64" s="36" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="N64" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O64" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="21" t="n">
@@ -4919,6 +5016,21 @@
         </is>
       </c>
       <c r="L89" s="6" t="n"/>
+      <c r="M89" s="36" t="inlineStr">
+        <is>
+          <t>508</t>
+        </is>
+      </c>
+      <c r="N89" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O89" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="21" t="n">
@@ -5500,6 +5612,21 @@
         </is>
       </c>
       <c r="L101" s="6" t="n"/>
+      <c r="M101" s="36" t="inlineStr">
+        <is>
+          <t>488</t>
+        </is>
+      </c>
+      <c r="N101" s="36" t="inlineStr">
+        <is>
+          <t>DHANVANTARI SALES</t>
+        </is>
+      </c>
+      <c r="O101" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="21" t="n">
@@ -5542,6 +5669,21 @@
         </is>
       </c>
       <c r="L102" s="6" t="n"/>
+      <c r="M102" s="36" t="inlineStr">
+        <is>
+          <t>531</t>
+        </is>
+      </c>
+      <c r="N102" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O102" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="21" t="n">
@@ -5810,6 +5952,21 @@
         </is>
       </c>
       <c r="L108" s="6" t="n"/>
+      <c r="M108" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N108" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O108" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="21" t="n">
@@ -6286,6 +6443,21 @@
         </is>
       </c>
       <c r="L118" s="6" t="n"/>
+      <c r="M118" s="36" t="inlineStr">
+        <is>
+          <t>567,549</t>
+        </is>
+      </c>
+      <c r="N118" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O118" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="21" t="n">
@@ -6370,6 +6542,21 @@
         </is>
       </c>
       <c r="L120" s="6" t="n"/>
+      <c r="M120" s="36" t="inlineStr">
+        <is>
+          <t>484,464,469,487,506,522</t>
+        </is>
+      </c>
+      <c r="N120" s="36" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O120" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="21" t="n">
@@ -6458,6 +6645,21 @@
         </is>
       </c>
       <c r="L122" s="6" t="n"/>
+      <c r="M122" s="36" t="inlineStr">
+        <is>
+          <t>689</t>
+        </is>
+      </c>
+      <c r="N122" s="36" t="inlineStr">
+        <is>
+          <t>SUPARSHWA MEDCARE LLP</t>
+        </is>
+      </c>
+      <c r="O122" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="21" t="n">
@@ -6645,6 +6847,21 @@
         </is>
       </c>
       <c r="L126" s="6" t="n"/>
+      <c r="M126" s="36" t="inlineStr">
+        <is>
+          <t>523</t>
+        </is>
+      </c>
+      <c r="N126" s="36" t="inlineStr">
+        <is>
+          <t>ABHAY PHARMA</t>
+        </is>
+      </c>
+      <c r="O126" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="21" t="n">
@@ -6687,6 +6904,21 @@
         </is>
       </c>
       <c r="L127" s="6" t="n"/>
+      <c r="M127" s="36" t="inlineStr">
+        <is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="N127" s="36" t="inlineStr">
+        <is>
+          <t>PRIME AYURVED</t>
+        </is>
+      </c>
+      <c r="O127" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="21" t="n">
@@ -6947,6 +7179,21 @@
         </is>
       </c>
       <c r="L133" s="6" t="n"/>
+      <c r="M133" s="36" t="inlineStr">
+        <is>
+          <t>578,577</t>
+        </is>
+      </c>
+      <c r="N133" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O133" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="21" t="n">
@@ -7085,6 +7332,21 @@
           <t>salary</t>
         </is>
       </c>
+      <c r="M136" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N136" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O136" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="21" t="n">
@@ -7661,6 +7923,21 @@
         </is>
       </c>
       <c r="L148" s="6" t="n"/>
+      <c r="M148" s="36" t="inlineStr">
+        <is>
+          <t>597</t>
+        </is>
+      </c>
+      <c r="N148" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O148" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="21" t="n">
@@ -8638,6 +8915,21 @@
         </is>
       </c>
       <c r="L169" s="6" t="n"/>
+      <c r="M169" s="36" t="inlineStr">
+        <is>
+          <t>583,596,607</t>
+        </is>
+      </c>
+      <c r="N169" s="36" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O169" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="21" t="n">
@@ -9388,6 +9680,21 @@
         </is>
       </c>
       <c r="L185" s="6" t="n"/>
+      <c r="M185" s="36" t="inlineStr">
+        <is>
+          <t>612</t>
+        </is>
+      </c>
+      <c r="N185" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O185" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="21" t="n">
@@ -10183,6 +10490,21 @@
         </is>
       </c>
       <c r="L203" s="6" t="n"/>
+      <c r="M203" s="36" t="inlineStr">
+        <is>
+          <t>629,630</t>
+        </is>
+      </c>
+      <c r="N203" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O203" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="21" t="n">
@@ -10369,6 +10691,21 @@
         </is>
       </c>
       <c r="L207" s="6" t="n"/>
+      <c r="M207" s="36" t="inlineStr">
+        <is>
+          <t>638</t>
+        </is>
+      </c>
+      <c r="N207" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O207" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="21" t="n">
@@ -10495,6 +10832,21 @@
         </is>
       </c>
       <c r="L210" s="6" t="n"/>
+      <c r="M210" s="36" t="inlineStr">
+        <is>
+          <t>472,467,481,505,525,532,546,548,586,592,606</t>
+        </is>
+      </c>
+      <c r="N210" s="36" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O210" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="21" t="n">
@@ -10763,6 +11115,21 @@
         </is>
       </c>
       <c r="L216" s="6" t="n"/>
+      <c r="M216" s="36" t="inlineStr">
+        <is>
+          <t>651</t>
+        </is>
+      </c>
+      <c r="N216" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O216" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="21" t="n">
@@ -10889,6 +11256,21 @@
         </is>
       </c>
       <c r="L219" s="6" t="n"/>
+      <c r="M219" s="36" t="inlineStr">
+        <is>
+          <t>216,221,234,244,265,292,301,305,308,324,333,349,363,362,372,389,393,400,418,429,437</t>
+        </is>
+      </c>
+      <c r="N219" s="36" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O219" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="21" t="n">
@@ -11319,6 +11701,21 @@
         </is>
       </c>
       <c r="L228" s="6" t="n"/>
+      <c r="M228" s="36" t="inlineStr">
+        <is>
+          <t>471,474,479,485,507,524,533,553,570</t>
+        </is>
+      </c>
+      <c r="N228" s="36" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O228" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="21" t="n">
@@ -11560,6 +11957,21 @@
         </is>
       </c>
       <c r="L233" s="6" t="n"/>
+      <c r="M233" s="36" t="inlineStr">
+        <is>
+          <t>670,673</t>
+        </is>
+      </c>
+      <c r="N233" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O233" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="21" t="n">
@@ -11778,6 +12190,21 @@
         </is>
       </c>
       <c r="L238" s="6" t="n"/>
+      <c r="M238" s="36" t="inlineStr">
+        <is>
+          <t>126,127,133,151,179,189,209,240,246,258,303,337,411,355,364,376,415,425</t>
+        </is>
+      </c>
+      <c r="N238" s="36" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O238" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="21" t="n">
@@ -11820,6 +12247,21 @@
         </is>
       </c>
       <c r="L239" s="6" t="n"/>
+      <c r="M239" s="36" t="inlineStr">
+        <is>
+          <t>504,538,551,566,609,633,644</t>
+        </is>
+      </c>
+      <c r="N239" s="36" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O239" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="21" t="n">
@@ -12273,6 +12715,17 @@
         </is>
       </c>
       <c r="L249" s="6" t="n"/>
+      <c r="M249" s="36" t="inlineStr"/>
+      <c r="N249" s="36" t="inlineStr">
+        <is>
+          <t>MSEDCL  -----------X----------</t>
+        </is>
+      </c>
+      <c r="O249" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="21" t="n">
@@ -12315,6 +12768,21 @@
         </is>
       </c>
       <c r="L250" s="6" t="n"/>
+      <c r="M250" s="36" t="inlineStr">
+        <is>
+          <t>671,692,657,672,691,690</t>
+        </is>
+      </c>
+      <c r="N250" s="36" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O250" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="21" t="n">
@@ -12797,6 +13265,21 @@
         </is>
       </c>
       <c r="L260" s="6" t="n"/>
+      <c r="M260" s="36" t="inlineStr">
+        <is>
+          <t>610</t>
+        </is>
+      </c>
+      <c r="N260" s="36" t="inlineStr">
+        <is>
+          <t>DHANWANTRI PHARMA</t>
+        </is>
+      </c>
+      <c r="O260" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="21" t="n">
@@ -12837,6 +13320,21 @@
         </is>
       </c>
       <c r="L261" s="6" t="n"/>
+      <c r="M261" s="36" t="inlineStr">
+        <is>
+          <t>682,705</t>
+        </is>
+      </c>
+      <c r="N261" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O261" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="21" t="n">
@@ -13239,6 +13737,21 @@
         </is>
       </c>
       <c r="L270" s="6" t="n"/>
+      <c r="M270" s="36" t="inlineStr">
+        <is>
+          <t>719</t>
+        </is>
+      </c>
+      <c r="N270" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O270" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="21" t="n">
@@ -14831,6 +15344,17 @@
         </is>
       </c>
       <c r="L304" s="6" t="n"/>
+      <c r="M304" s="36" t="inlineStr"/>
+      <c r="N304" s="36" t="inlineStr">
+        <is>
+          <t>KAPILA PASHU AUSHADHALAYA</t>
+        </is>
+      </c>
+      <c r="O304" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="21" t="n">
@@ -14871,6 +15395,21 @@
         </is>
       </c>
       <c r="L305" s="6" t="n"/>
+      <c r="M305" s="36" t="inlineStr">
+        <is>
+          <t>689</t>
+        </is>
+      </c>
+      <c r="N305" s="36" t="inlineStr">
+        <is>
+          <t>SUPARSHWA MEDCARE LLP</t>
+        </is>
+      </c>
+      <c r="O305" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="21" t="n">
@@ -15035,6 +15574,21 @@
         </is>
       </c>
       <c r="L309" s="6" t="n"/>
+      <c r="M309" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N309" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O309" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="21" t="n">
@@ -15511,6 +16065,21 @@
         </is>
       </c>
       <c r="L320" s="6" t="n"/>
+      <c r="M320" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N320" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O320" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="321" customFormat="1" s="2">
       <c r="A321" s="22" t="n">
@@ -16768,6 +17337,21 @@
         </is>
       </c>
       <c r="L348" s="6" t="n"/>
+      <c r="M348" s="36" t="inlineStr">
+        <is>
+          <t>497,656</t>
+        </is>
+      </c>
+      <c r="N348" s="36" t="inlineStr">
+        <is>
+          <t>SHREYAA AGENCIES</t>
+        </is>
+      </c>
+      <c r="O348" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="21" t="n">
@@ -17805,7 +18389,7 @@
       <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
-          <t>G K ENTERPRISES / CG MARKETING PVT LTD</t>
+          <t>CG MARKETING PVT LTD / G K ENTERPRISES</t>
         </is>
       </c>
       <c r="O371" s="33" t="inlineStr">
@@ -18026,6 +18610,21 @@
         </is>
       </c>
       <c r="L376" s="6" t="n"/>
+      <c r="M376" s="36" t="inlineStr">
+        <is>
+          <t>804,753,805,770</t>
+        </is>
+      </c>
+      <c r="N376" s="36" t="inlineStr">
+        <is>
+          <t>VARDAAN DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O376" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="21" t="n">
@@ -19857,6 +20456,21 @@
         </is>
       </c>
       <c r="L416" s="6" t="n"/>
+      <c r="M416" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N416" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O416" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="417">
       <c r="A417" s="21" t="n">
@@ -21232,6 +21846,21 @@
         </is>
       </c>
       <c r="L446" s="6" t="n"/>
+      <c r="M446" s="36" t="inlineStr">
+        <is>
+          <t>623,632,640,648,661,676,687,707,722,728,736,744,750,758,774,783,807,818,857,875,894,902,909,925,934,941</t>
+        </is>
+      </c>
+      <c r="N446" s="36" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O446" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="21" t="n">
@@ -21665,6 +22294,21 @@
         </is>
       </c>
       <c r="L456" s="6" t="n"/>
+      <c r="M456" s="36" t="inlineStr">
+        <is>
+          <t>477,678,776,869,960</t>
+        </is>
+      </c>
+      <c r="N456" s="36" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O456" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="21" t="n">
@@ -22627,6 +23271,21 @@
         </is>
       </c>
       <c r="L478" s="6" t="n"/>
+      <c r="M478" s="36" t="inlineStr">
+        <is>
+          <t>585,593,594,605,620,631,642,647,658,679,686,706,729,742,752,759,760,775,785,799,808,817,819,828,840,858,878,893,905,922,937,942</t>
+        </is>
+      </c>
+      <c r="N478" s="36" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O478" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" s="21" t="n">
@@ -25178,6 +25837,21 @@
         </is>
       </c>
       <c r="L535" s="6" t="n"/>
+      <c r="M535" s="36" t="inlineStr">
+        <is>
+          <t>2359,680,683,684,704,726,735,741,746,751,763,789,796,824,829,843,853,874,887,906,910,933</t>
+        </is>
+      </c>
+      <c r="N535" s="36" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O535" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="21" t="n">
@@ -25262,6 +25936,21 @@
           <t>salary</t>
         </is>
       </c>
+      <c r="M537" s="36" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="N537" s="36" t="inlineStr">
+        <is>
+          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+        </is>
+      </c>
+      <c r="O537" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" s="21" t="n">
@@ -26688,6 +27377,21 @@
         </is>
       </c>
       <c r="L570" s="6" t="n"/>
+      <c r="M570" s="36" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="N570" s="36" t="inlineStr">
+        <is>
+          <t>NAVMAHARASTRA ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O570" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" s="21" t="n">
@@ -30115,6 +30819,21 @@
         </is>
       </c>
       <c r="L648" s="6" t="n"/>
+      <c r="M648" s="36" t="inlineStr">
+        <is>
+          <t>949,957,969,980,987,1006,1011,1023,1032,1039,1053,1068,1076,1106</t>
+        </is>
+      </c>
+      <c r="N648" s="36" t="inlineStr">
+        <is>
+          <t>JM PHARMA</t>
+        </is>
+      </c>
+      <c r="O648" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="649">
       <c r="A649" s="21" t="n">
@@ -30239,6 +30958,21 @@
         </is>
       </c>
       <c r="L651" s="6" t="n"/>
+      <c r="M651" s="36" t="inlineStr">
+        <is>
+          <t>1083,1108,1128</t>
+        </is>
+      </c>
+      <c r="N651" s="36" t="inlineStr">
+        <is>
+          <t>PRIME DITRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O651" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="652">
       <c r="A652" s="21" t="n">

</xml_diff>

<commit_message>
Re-run reconciliation on updated PAIDMAST+PAIDTRAN DBF (a40f3bd)
PAIDMAST: 379->387, PAIDTRAN: 904->980
CHQ_MATCHED: 147, GPAY_MATCHED: 51, NOT_IN_SYSTEM: 101
Old Account CHQ: 150, GPAY: 210, Pending: 44, Prev Pending: 43

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -8288,7 +8288,7 @@
       </c>
       <c r="N155" s="33" t="inlineStr">
         <is>
-          <t>HDFC BANK / SHREE DATTA KRUPA AGENCY</t>
+          <t>SHREE DATTA KRUPA AGENCY / HDFC BANK</t>
         </is>
       </c>
       <c r="O155" s="33" t="inlineStr">
@@ -18389,7 +18389,7 @@
       <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
-          <t>CG MARKETING PVT LTD / G K ENTERPRISES</t>
+          <t>G K ENTERPRISES / CG MARKETING PVT LTD</t>
         </is>
       </c>
       <c r="O371" s="33" t="inlineStr">
@@ -29073,7 +29073,7 @@
       <c r="M608" s="33" t="inlineStr"/>
       <c r="N608" s="33" t="inlineStr">
         <is>
-          <t>M/S MANDAR AGENCY / SONIGARA DISTRIBUTOR</t>
+          <t>SONIGARA DISTRIBUTOR / M/S MANDAR AGENCY</t>
         </is>
       </c>
       <c r="O608" s="33" t="inlineStr">
@@ -32955,7 +32955,11 @@
         </is>
       </c>
       <c r="L697" s="6" t="n"/>
-      <c r="M697" s="33" t="inlineStr"/>
+      <c r="M697" s="33" t="inlineStr">
+        <is>
+          <t>1145</t>
+        </is>
+      </c>
       <c r="N697" s="33" t="inlineStr">
         <is>
           <t>SHINDE ENTERPRISES</t>
@@ -34332,9 +34336,15 @@
         </is>
       </c>
       <c r="L727" s="6" t="n"/>
-      <c r="O727" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
+      <c r="M727" s="33" t="inlineStr"/>
+      <c r="N727" s="33" t="inlineStr">
+        <is>
+          <t>MEDIRAJ DISTRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O727" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
         </is>
       </c>
     </row>
@@ -36224,6 +36234,21 @@
         </is>
       </c>
       <c r="L770" s="6" t="n"/>
+      <c r="M770" s="36" t="inlineStr">
+        <is>
+          <t>1040,1052,1061,1070,1078,1105,1115,1132,1144,1154,1167,1174,1182,1190,1195,1201,1209,1224,1233</t>
+        </is>
+      </c>
+      <c r="N770" s="36" t="inlineStr">
+        <is>
+          <t>JEEVAN MEDISALES PVT LTD</t>
+        </is>
+      </c>
+      <c r="O770" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="771">
       <c r="A771" s="21" t="n">
@@ -36432,6 +36457,21 @@
         </is>
       </c>
       <c r="L775" s="6" t="n"/>
+      <c r="M775" s="36" t="inlineStr">
+        <is>
+          <t>948,956,1000,1033,1051,1057,1067,1095,1107,1127,1126</t>
+        </is>
+      </c>
+      <c r="N775" s="36" t="inlineStr">
+        <is>
+          <t>D.K. ENTERPRISES</t>
+        </is>
+      </c>
+      <c r="O775" s="36" t="inlineStr">
+        <is>
+          <t>GPAY_MATCHED</t>
+        </is>
+      </c>
     </row>
     <row r="776">
       <c r="A776" s="21" t="n">
@@ -38570,9 +38610,19 @@
         </is>
       </c>
       <c r="L824" s="6" t="n"/>
-      <c r="O824" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
+      <c r="M824" s="33" t="inlineStr">
+        <is>
+          <t>951,958,967,982,990,998,1008,1007,1010,1021,1031,1044,1049,1060,1066,1077,1096,1111,1116,1125</t>
+        </is>
+      </c>
+      <c r="N824" s="33" t="inlineStr">
+        <is>
+          <t>SENIOR AGENCY</t>
+        </is>
+      </c>
+      <c r="O824" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
         </is>
       </c>
     </row>
@@ -39094,9 +39144,19 @@
         </is>
       </c>
       <c r="L836" s="6" t="n"/>
-      <c r="O836" s="34" t="inlineStr">
-        <is>
-          <t>NOT_IN_SYSTEM</t>
+      <c r="M836" s="33" t="inlineStr">
+        <is>
+          <t>972,988,985,997,1005,1009,1018,1038,1047,1059,1071,1079,1109</t>
+        </is>
+      </c>
+      <c r="N836" s="33" t="inlineStr">
+        <is>
+          <t>MAHENDRA DISRIBUTORS</t>
+        </is>
+      </c>
+      <c r="O836" s="33" t="inlineStr">
+        <is>
+          <t>CHQ_MATCHED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split Voucher_No: System_Purchase matched vs Old_Voucher_No (pre-system)
- Voucher_No filled only when PURVCHNO exists in System_Purchase (green)
- Old_Voucher_No new column for PURVCHNOs not in System_Purchase (gold)
- Applies to both CHQ_MATCHED and GPAY_MATCHED bank rows

https://claude.ai/code/session_01KRmwYvagtCo5dfJvTUZdhu
</commit_message>
<xml_diff>
--- a/Old_Bank_Statement_Shree_Seva_Medical.xlsx
+++ b/Old_Bank_Statement_Shree_Seva_Medical.xlsx
@@ -68,7 +68,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9B3FF"/>
         <bgColor rgb="00D9B3FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+        <bgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
   </fills>
@@ -286,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -352,6 +358,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,7 +736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O891"/>
+  <dimension ref="A1:P891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" style="23" min="1" max="1"/>
@@ -822,6 +829,11 @@
           <t>Match_Status</t>
         </is>
       </c>
+      <c r="P1" s="32" t="inlineStr">
+        <is>
+          <t>Old_Voucher_No</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="21" t="n">
@@ -921,6 +933,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P3" s="37" t="inlineStr">
+        <is>
+          <t>208,250</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="n">
@@ -978,6 +995,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P4" s="37" t="inlineStr">
+        <is>
+          <t>276,330</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="n">
@@ -1406,6 +1428,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P13" s="37" t="inlineStr">
+        <is>
+          <t>2601</t>
+        </is>
+      </c>
     </row>
     <row r="14" customFormat="1" s="31">
       <c r="A14" s="29" t="n">
@@ -1631,6 +1658,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P18" s="37" t="inlineStr">
+        <is>
+          <t>2747,2751,2771,2774,2782,2787,2799,2802,2818</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="21" t="n">
@@ -2176,12 +2208,17 @@
       </c>
       <c r="N30" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O30" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P30" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -2593,6 +2630,11 @@
           <t>GPAY_MATCHED</t>
         </is>
       </c>
+      <c r="P39" s="37" t="inlineStr">
+        <is>
+          <t>327,344</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="21" t="n">
@@ -2650,6 +2692,11 @@
           <t>GPAY_MATCHED</t>
         </is>
       </c>
+      <c r="P40" s="37" t="inlineStr">
+        <is>
+          <t>293,298,307,319</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="21" t="n">
@@ -2845,6 +2892,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P44" s="37" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="21" t="n">
@@ -2902,6 +2954,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P45" s="37" t="inlineStr">
+        <is>
+          <t>2518,2529,2560,2566,2561,2588,2591,2611,2620,2621,2629,2657,2666,2761,2760,2766,2798,2833,2837,2891,2909,2921,2942</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="21" t="n">
@@ -3072,7 +3129,7 @@
       <c r="L49" s="6" t="n"/>
       <c r="M49" s="36" t="inlineStr">
         <is>
-          <t>334,347,357,379,390,391,402,414,428,435,446</t>
+          <t>428,435,446</t>
         </is>
       </c>
       <c r="N49" s="36" t="inlineStr">
@@ -3083,6 +3140,11 @@
       <c r="O49" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P49" s="37" t="inlineStr">
+        <is>
+          <t>334,347,357,379,390,391,402,414</t>
         </is>
       </c>
     </row>
@@ -3687,6 +3749,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P61" s="37" t="inlineStr">
+        <is>
+          <t>406,409</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="21" t="n">
@@ -3744,6 +3811,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P62" s="37" t="inlineStr">
+        <is>
+          <t>399</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="n">
@@ -4003,6 +4075,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P67" s="37" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="21" t="n">
@@ -4426,6 +4503,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P76" s="37" t="inlineStr">
+        <is>
+          <t>2828,2835,2848,2852,2866,2867,2877,2884</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="21" t="n">
@@ -4572,6 +4654,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P79" s="37" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="21" t="n">
@@ -5184,6 +5271,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P92" s="37" t="inlineStr">
+        <is>
+          <t>412</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="21" t="n">
@@ -5959,12 +6051,17 @@
       </c>
       <c r="N108" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O108" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P108" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -6158,6 +6255,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P112" s="37" t="inlineStr">
+        <is>
+          <t>2916,2926,2928,2934,2939,2958,6,11,17,22,30,40,48,61,75,77,96,109,112,123,139,149,164,170,178,186,200,203,218,236,248,252,270,272,291,297,304,306,326,338,348,356,361,371,387,394,401,408,417</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="21" t="n">
@@ -7339,12 +7441,17 @@
       </c>
       <c r="N136" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O136" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P136" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -8296,6 +8403,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P155" s="37" t="inlineStr">
+        <is>
+          <t>256,256</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="21" t="n">
@@ -9134,7 +9246,7 @@
       <c r="L173" s="6" t="n"/>
       <c r="M173" s="33" t="inlineStr">
         <is>
-          <t>259,252,266,578,573,773</t>
+          <t>578,573,773</t>
         </is>
       </c>
       <c r="N173" s="33" t="inlineStr">
@@ -9145,6 +9257,11 @@
       <c r="O173" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P173" s="37" t="inlineStr">
+        <is>
+          <t>259,252,266</t>
         </is>
       </c>
     </row>
@@ -11258,7 +11375,7 @@
       <c r="L219" s="6" t="n"/>
       <c r="M219" s="36" t="inlineStr">
         <is>
-          <t>216,221,234,244,265,292,301,305,308,324,333,349,363,362,372,389,393,400,418,429,437</t>
+          <t>429,437</t>
         </is>
       </c>
       <c r="N219" s="36" t="inlineStr">
@@ -11269,6 +11386,11 @@
       <c r="O219" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P219" s="37" t="inlineStr">
+        <is>
+          <t>216,221,234,244,265,292,301,305,308,324,333,349,363,362,372,389,393,400,418</t>
         </is>
       </c>
     </row>
@@ -12192,7 +12314,7 @@
       <c r="L238" s="6" t="n"/>
       <c r="M238" s="36" t="inlineStr">
         <is>
-          <t>126,127,133,151,179,189,209,240,246,258,303,337,411,355,364,376,415,425</t>
+          <t>425</t>
         </is>
       </c>
       <c r="N238" s="36" t="inlineStr">
@@ -12203,6 +12325,11 @@
       <c r="O238" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P238" s="37" t="inlineStr">
+        <is>
+          <t>126,127,133,151,179,189,209,240,246,258,303,337,411,355,364,376,415</t>
         </is>
       </c>
     </row>
@@ -13116,7 +13243,7 @@
       <c r="L257" s="6" t="n"/>
       <c r="M257" s="33" t="inlineStr">
         <is>
-          <t>5,8,46,49,91,105,138,152,162,180,188,215,220,237,243,263,288,299,325,342,346,358,365,378,388,392,404,433</t>
+          <t>433</t>
         </is>
       </c>
       <c r="N257" s="33" t="inlineStr">
@@ -13127,6 +13254,11 @@
       <c r="O257" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P257" s="37" t="inlineStr">
+        <is>
+          <t>5,8,46,49,91,105,138,152,162,180,188,215,220,237,243,263,288,299,325,342,346,358,365,378,388,392,404</t>
         </is>
       </c>
     </row>
@@ -14808,7 +14940,7 @@
       <c r="L292" s="6" t="n"/>
       <c r="M292" s="33" t="inlineStr">
         <is>
-          <t>386,420,440,483</t>
+          <t>483</t>
         </is>
       </c>
       <c r="N292" s="33" t="inlineStr">
@@ -14819,6 +14951,11 @@
       <c r="O292" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P292" s="37" t="inlineStr">
+        <is>
+          <t>386,420,440</t>
         </is>
       </c>
     </row>
@@ -15581,12 +15718,17 @@
       </c>
       <c r="N309" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O309" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P309" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -16072,12 +16214,17 @@
       </c>
       <c r="N320" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O320" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P320" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -16843,6 +16990,11 @@
           <t>CHQ_MATCHED</t>
         </is>
       </c>
+      <c r="P337" s="37" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="21" t="n">
@@ -18243,7 +18395,7 @@
       <c r="L368" s="6" t="n"/>
       <c r="M368" s="33" t="inlineStr">
         <is>
-          <t>2864,2878,2886,2889,2901,2914,2915,2923,2925,2937,2944,2949,2950,16,34,159,213,249,269,289,302,311,375,416,432</t>
+          <t>432</t>
         </is>
       </c>
       <c r="N368" s="33" t="inlineStr">
@@ -18254,6 +18406,11 @@
       <c r="O368" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P368" s="37" t="inlineStr">
+        <is>
+          <t>2864,2878,2886,2889,2901,2914,2915,2923,2925,2937,2944,2949,2950,16,34,159,213,249,269,289,302,311,375,416</t>
         </is>
       </c>
     </row>
@@ -18389,7 +18546,7 @@
       <c r="M371" s="33" t="inlineStr"/>
       <c r="N371" s="33" t="inlineStr">
         <is>
-          <t>G K ENTERPRISES / CG MARKETING PVT LTD</t>
+          <t>CG MARKETING PVT LTD / G K ENTERPRISES</t>
         </is>
       </c>
       <c r="O371" s="33" t="inlineStr">
@@ -20463,12 +20620,17 @@
       </c>
       <c r="N416" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O416" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P416" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -25839,7 +26001,7 @@
       <c r="L535" s="6" t="n"/>
       <c r="M535" s="36" t="inlineStr">
         <is>
-          <t>2359,680,683,684,704,726,735,741,746,751,763,789,796,824,829,843,853,874,887,906,910,933</t>
+          <t>680,683,684,704,726,735,741,746,751,763,789,796,824,829,843,853,874,887,906,910,933</t>
         </is>
       </c>
       <c r="N535" s="36" t="inlineStr">
@@ -25850,6 +26012,11 @@
       <c r="O535" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P535" s="37" t="inlineStr">
+        <is>
+          <t>2359</t>
         </is>
       </c>
     </row>
@@ -25943,12 +26110,17 @@
       </c>
       <c r="N537" s="36" t="inlineStr">
         <is>
-          <t>MONT VERT BELAIR CO OPERAT. HO</t>
+          <t>VARDAAN DISTRIBUTORS</t>
         </is>
       </c>
       <c r="O537" s="36" t="inlineStr">
         <is>
           <t>GPAY_MATCHED</t>
+        </is>
+      </c>
+      <c r="P537" s="37" t="inlineStr">
+        <is>
+          <t>2954</t>
         </is>
       </c>
     </row>
@@ -27284,7 +27456,7 @@
       <c r="L568" s="6" t="n"/>
       <c r="M568" s="33" t="inlineStr">
         <is>
-          <t>310,341,343,351,353,427,434,457,460,521,537,613,649,723,782,821,825</t>
+          <t>427,434,457,460,521,537,613,649,723,782,821,825</t>
         </is>
       </c>
       <c r="N568" s="33" t="inlineStr">
@@ -27295,6 +27467,11 @@
       <c r="O568" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P568" s="37" t="inlineStr">
+        <is>
+          <t>310,341,343,351,353</t>
         </is>
       </c>
     </row>
@@ -28750,7 +28927,7 @@
       <c r="L601" s="6" t="n"/>
       <c r="M601" s="33" t="inlineStr">
         <is>
-          <t>2099,854,1444,1445,2406</t>
+          <t>854,1444,1445</t>
         </is>
       </c>
       <c r="N601" s="33" t="inlineStr">
@@ -28761,6 +28938,11 @@
       <c r="O601" s="33" t="inlineStr">
         <is>
           <t>CHQ_MATCHED</t>
+        </is>
+      </c>
+      <c r="P601" s="37" t="inlineStr">
+        <is>
+          <t>2099,2406</t>
         </is>
       </c>
     </row>

</xml_diff>